<commit_message>
Service ticket : un bloc = un mois civil, facturation mensuelle sur 3 mois
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/service_ticket_2027/Service_Ticket_Enedril_2027.xlsx
+++ b/service_ticket_2027/Service_Ticket_Enedril_2027.xlsx
@@ -367,7 +367,7 @@
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -926,7 +926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DO53"/>
+  <dimension ref="A1:DX53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -988,6 +988,15 @@
     <col hidden="1" width="13" customWidth="1" min="117" max="117"/>
     <col hidden="1" width="13" customWidth="1" min="118" max="118"/>
     <col hidden="1" width="13" customWidth="1" min="119" max="119"/>
+    <col hidden="1" width="13" customWidth="1" min="120" max="120"/>
+    <col hidden="1" width="13" customWidth="1" min="121" max="121"/>
+    <col hidden="1" width="13" customWidth="1" min="122" max="122"/>
+    <col hidden="1" width="13" customWidth="1" min="123" max="123"/>
+    <col hidden="1" width="13" customWidth="1" min="124" max="124"/>
+    <col hidden="1" width="13" customWidth="1" min="125" max="125"/>
+    <col hidden="1" width="13" customWidth="1" min="126" max="126"/>
+    <col hidden="1" width="13" customWidth="1" min="127" max="127"/>
+    <col hidden="1" width="13" customWidth="1" min="128" max="128"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1123,7 +1132,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>DATE DE FIN · END DATE (À MODIFIER)</t>
+          <t>DATE DE FIN (3 MOIS MAX)</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
@@ -1143,28 +1152,44 @@
       <c r="H9" s="7" t="n"/>
       <c r="I9" s="7" t="n"/>
       <c r="J9" s="9">
-        <f>IF(C9="","",MIN(93,MAX(1,IF(G9="",31,G9-C9+1))))</f>
+        <f>IF(C9="","",$DC$9-C9+1)</f>
         <v/>
       </c>
       <c r="K9" s="10" t="n"/>
       <c r="L9" s="10" t="n"/>
+      <c r="DC9">
+        <f>IF($C$9="","",MIN(IF($G$9="",EOMONTH($C$9,0),MAX($G$9,$C$9)),EOMONTH($C$9,2)))</f>
+        <v/>
+      </c>
+      <c r="DD9">
+        <f>IF($C$9="",0,MAX(0,MIN($DC$9,EOMONTH($C$9,0))-$C$9+1))</f>
+        <v/>
+      </c>
+      <c r="DE9">
+        <f>IF($C$9="",0,MAX(0,MIN($DC$9,EOMONTH($C$9,1))-DATE(YEAR($C$9),MONTH($C$9)+1,1)+1))</f>
+        <v/>
+      </c>
+      <c r="DF9">
+        <f>IF($C$9="",0,MAX(0,MIN($DC$9,EOMONTH($C$9,2))-DATE(YEAR($C$9),MONTH($C$9)+2,1)+1))</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="11">
-        <f>IF(N($J$9)&gt;31,"⚠  La date de fin dépasse le 1er bloc : cliquer sur le [+] au-dessus du calendrier pour déplier les jours suivants.","")</f>
+        <f>IF(N($DE$9)&gt;0,"⚠  Le chantier dépasse le 1er mois : cliquer sur le [+] au-dessus du calendrier pour déplier le mois suivant (et le 3e).","")</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Codes : S = stand-by · O = opérations · FOC = gratuit · VR = valeur de remplacement · RC = restocking · MOB / DEMOB = arrivée / départ (comptés en S)</t>
+          <t>Codes : S stand-by · O opérations · FOC gratuit · VR valeur de remplacement · RC restocking · MOB / DEMOB (comptés en S)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="M12" s="13">
-        <f>IF(OR($C$9="",N($J$9)&lt;=0),"","Du "&amp;TEXT(DAY($C$9+0),"00")&amp;"/"&amp;TEXT(MONTH($C$9+0),"00")&amp;" au "&amp;TEXT(DAY($C$9+MIN(30,$J$9-1)),"00")&amp;"/"&amp;TEXT(MONTH($C$9+MIN(30,$J$9-1)),"00")&amp;"/"&amp;YEAR($C$9+MIN(30,$J$9-1)))</f>
+        <f>IF(OR($C$9="",N($DD$9)=0),"",CHOOSE(MONTH($C$9),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR($C$9)&amp;"   ·   du "&amp;TEXT(DAY($C$9),"00")&amp;"/"&amp;TEXT(MONTH($C$9),"00")&amp;" au "&amp;TEXT(DAY(($C$9+$DD$9-1)),"00")&amp;"/"&amp;TEXT(MONTH(($C$9+$DD$9-1)),"00")&amp;"/"&amp;YEAR(($C$9+$DD$9-1)))</f>
         <v/>
       </c>
       <c r="N12" s="14" t="n"/>
@@ -1198,7 +1223,7 @@
       <c r="AP12" s="14" t="n"/>
       <c r="AQ12" s="14" t="n"/>
       <c r="AR12" s="15">
-        <f>IF(OR($C$9="",N($J$9)&lt;=31),"","Du "&amp;TEXT(DAY($C$9+31),"00")&amp;"/"&amp;TEXT(MONTH($C$9+31),"00")&amp;" au "&amp;TEXT(DAY($C$9+MIN(61,$J$9-1)),"00")&amp;"/"&amp;TEXT(MONTH($C$9+MIN(61,$J$9-1)),"00")&amp;"/"&amp;YEAR($C$9+MIN(61,$J$9-1)))</f>
+        <f>IF(OR($C$9="",N($DE$9)=0),"",CHOOSE(MONTH(DATE(YEAR($C$9),MONTH($C$9)+1,1)),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR(DATE(YEAR($C$9),MONTH($C$9)+1,1))&amp;"   ·   du "&amp;TEXT(DAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)),"00")&amp;"/"&amp;TEXT(MONTH(DATE(YEAR($C$9),MONTH($C$9)+1,1)),"00")&amp;" au "&amp;TEXT(DAY((DATE(YEAR($C$9),MONTH($C$9)+1,1)+$DE$9-1)),"00")&amp;"/"&amp;TEXT(MONTH((DATE(YEAR($C$9),MONTH($C$9)+1,1)+$DE$9-1)),"00")&amp;"/"&amp;YEAR((DATE(YEAR($C$9),MONTH($C$9)+1,1)+$DE$9-1)))</f>
         <v/>
       </c>
       <c r="AS12" s="1" t="n"/>
@@ -1232,7 +1257,7 @@
       <c r="BU12" s="1" t="n"/>
       <c r="BV12" s="1" t="n"/>
       <c r="BW12" s="13">
-        <f>IF(OR($C$9="",N($J$9)&lt;=62),"","Du "&amp;TEXT(DAY($C$9+62),"00")&amp;"/"&amp;TEXT(MONTH($C$9+62),"00")&amp;" au "&amp;TEXT(DAY($C$9+MIN(92,$J$9-1)),"00")&amp;"/"&amp;TEXT(MONTH($C$9+MIN(92,$J$9-1)),"00")&amp;"/"&amp;YEAR($C$9+MIN(92,$J$9-1)))</f>
+        <f>IF(OR($C$9="",N($DF$9)=0),"",CHOOSE(MONTH(DATE(YEAR($C$9),MONTH($C$9)+2,1)),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR(DATE(YEAR($C$9),MONTH($C$9)+2,1))&amp;"   ·   du "&amp;TEXT(DAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)),"00")&amp;"/"&amp;TEXT(MONTH(DATE(YEAR($C$9),MONTH($C$9)+2,1)),"00")&amp;" au "&amp;TEXT(DAY((DATE(YEAR($C$9),MONTH($C$9)+2,1)+$DF$9-1)),"00")&amp;"/"&amp;TEXT(MONTH((DATE(YEAR($C$9),MONTH($C$9)+2,1)+$DF$9-1)),"00")&amp;"/"&amp;YEAR((DATE(YEAR($C$9),MONTH($C$9)+2,1)+$DF$9-1)))</f>
         <v/>
       </c>
       <c r="BX12" s="14" t="n"/>
@@ -1339,375 +1364,375 @@
         </is>
       </c>
       <c r="M13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=0),"",$C$9+0)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=0),"",$C$9+0)</f>
         <v/>
       </c>
       <c r="N13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=1),"",$C$9+1)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=1),"",$C$9+1)</f>
         <v/>
       </c>
       <c r="O13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=2),"",$C$9+2)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=2),"",$C$9+2)</f>
         <v/>
       </c>
       <c r="P13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=3),"",$C$9+3)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=3),"",$C$9+3)</f>
         <v/>
       </c>
       <c r="Q13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=4),"",$C$9+4)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=4),"",$C$9+4)</f>
         <v/>
       </c>
       <c r="R13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=5),"",$C$9+5)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=5),"",$C$9+5)</f>
         <v/>
       </c>
       <c r="S13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=6),"",$C$9+6)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=6),"",$C$9+6)</f>
         <v/>
       </c>
       <c r="T13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=7),"",$C$9+7)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=7),"",$C$9+7)</f>
         <v/>
       </c>
       <c r="U13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=8),"",$C$9+8)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=8),"",$C$9+8)</f>
         <v/>
       </c>
       <c r="V13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=9),"",$C$9+9)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=9),"",$C$9+9)</f>
         <v/>
       </c>
       <c r="W13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=10),"",$C$9+10)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=10),"",$C$9+10)</f>
         <v/>
       </c>
       <c r="X13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=11),"",$C$9+11)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=11),"",$C$9+11)</f>
         <v/>
       </c>
       <c r="Y13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=12),"",$C$9+12)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=12),"",$C$9+12)</f>
         <v/>
       </c>
       <c r="Z13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=13),"",$C$9+13)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=13),"",$C$9+13)</f>
         <v/>
       </c>
       <c r="AA13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=14),"",$C$9+14)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=14),"",$C$9+14)</f>
         <v/>
       </c>
       <c r="AB13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=15),"",$C$9+15)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=15),"",$C$9+15)</f>
         <v/>
       </c>
       <c r="AC13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=16),"",$C$9+16)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=16),"",$C$9+16)</f>
         <v/>
       </c>
       <c r="AD13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=17),"",$C$9+17)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=17),"",$C$9+17)</f>
         <v/>
       </c>
       <c r="AE13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=18),"",$C$9+18)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=18),"",$C$9+18)</f>
         <v/>
       </c>
       <c r="AF13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=19),"",$C$9+19)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=19),"",$C$9+19)</f>
         <v/>
       </c>
       <c r="AG13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=20),"",$C$9+20)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=20),"",$C$9+20)</f>
         <v/>
       </c>
       <c r="AH13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=21),"",$C$9+21)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=21),"",$C$9+21)</f>
         <v/>
       </c>
       <c r="AI13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=22),"",$C$9+22)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=22),"",$C$9+22)</f>
         <v/>
       </c>
       <c r="AJ13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=23),"",$C$9+23)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=23),"",$C$9+23)</f>
         <v/>
       </c>
       <c r="AK13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=24),"",$C$9+24)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=24),"",$C$9+24)</f>
         <v/>
       </c>
       <c r="AL13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=25),"",$C$9+25)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=25),"",$C$9+25)</f>
         <v/>
       </c>
       <c r="AM13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=26),"",$C$9+26)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=26),"",$C$9+26)</f>
         <v/>
       </c>
       <c r="AN13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=27),"",$C$9+27)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=27),"",$C$9+27)</f>
         <v/>
       </c>
       <c r="AO13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=28),"",$C$9+28)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=28),"",$C$9+28)</f>
         <v/>
       </c>
       <c r="AP13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=29),"",$C$9+29)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=29),"",$C$9+29)</f>
         <v/>
       </c>
       <c r="AQ13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=30),"",$C$9+30)</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=30),"",$C$9+30)</f>
         <v/>
       </c>
       <c r="AR13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=31),"",$C$9+31)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=0),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+0)</f>
         <v/>
       </c>
       <c r="AS13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=32),"",$C$9+32)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=1),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+1)</f>
         <v/>
       </c>
       <c r="AT13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=33),"",$C$9+33)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=2),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+2)</f>
         <v/>
       </c>
       <c r="AU13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=34),"",$C$9+34)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=3),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+3)</f>
         <v/>
       </c>
       <c r="AV13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=35),"",$C$9+35)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=4),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+4)</f>
         <v/>
       </c>
       <c r="AW13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=36),"",$C$9+36)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=5),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+5)</f>
         <v/>
       </c>
       <c r="AX13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=37),"",$C$9+37)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=6),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+6)</f>
         <v/>
       </c>
       <c r="AY13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=38),"",$C$9+38)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=7),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+7)</f>
         <v/>
       </c>
       <c r="AZ13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=39),"",$C$9+39)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=8),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+8)</f>
         <v/>
       </c>
       <c r="BA13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=40),"",$C$9+40)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=9),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+9)</f>
         <v/>
       </c>
       <c r="BB13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=41),"",$C$9+41)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=10),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+10)</f>
         <v/>
       </c>
       <c r="BC13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=42),"",$C$9+42)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=11),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+11)</f>
         <v/>
       </c>
       <c r="BD13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=43),"",$C$9+43)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=12),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+12)</f>
         <v/>
       </c>
       <c r="BE13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=44),"",$C$9+44)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=13),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+13)</f>
         <v/>
       </c>
       <c r="BF13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=45),"",$C$9+45)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=14),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+14)</f>
         <v/>
       </c>
       <c r="BG13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=46),"",$C$9+46)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=15),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+15)</f>
         <v/>
       </c>
       <c r="BH13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=47),"",$C$9+47)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=16),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+16)</f>
         <v/>
       </c>
       <c r="BI13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=48),"",$C$9+48)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=17),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+17)</f>
         <v/>
       </c>
       <c r="BJ13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=49),"",$C$9+49)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=18),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+18)</f>
         <v/>
       </c>
       <c r="BK13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=50),"",$C$9+50)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=19),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+19)</f>
         <v/>
       </c>
       <c r="BL13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=51),"",$C$9+51)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=20),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+20)</f>
         <v/>
       </c>
       <c r="BM13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=52),"",$C$9+52)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=21),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+21)</f>
         <v/>
       </c>
       <c r="BN13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=53),"",$C$9+53)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=22),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+22)</f>
         <v/>
       </c>
       <c r="BO13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=54),"",$C$9+54)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=23),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+23)</f>
         <v/>
       </c>
       <c r="BP13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=55),"",$C$9+55)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=24),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+24)</f>
         <v/>
       </c>
       <c r="BQ13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=56),"",$C$9+56)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=25),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+25)</f>
         <v/>
       </c>
       <c r="BR13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=57),"",$C$9+57)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=26),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+26)</f>
         <v/>
       </c>
       <c r="BS13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=58),"",$C$9+58)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=27),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+27)</f>
         <v/>
       </c>
       <c r="BT13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=59),"",$C$9+59)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=28),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+28)</f>
         <v/>
       </c>
       <c r="BU13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=60),"",$C$9+60)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=29),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+29)</f>
         <v/>
       </c>
       <c r="BV13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=61),"",$C$9+61)</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=30),"",DATE(YEAR($C$9),MONTH($C$9)+1,1)+30)</f>
         <v/>
       </c>
       <c r="BW13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=62),"",$C$9+62)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=0),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+0)</f>
         <v/>
       </c>
       <c r="BX13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=63),"",$C$9+63)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=1),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+1)</f>
         <v/>
       </c>
       <c r="BY13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=64),"",$C$9+64)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=2),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+2)</f>
         <v/>
       </c>
       <c r="BZ13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=65),"",$C$9+65)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=3),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+3)</f>
         <v/>
       </c>
       <c r="CA13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=66),"",$C$9+66)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=4),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+4)</f>
         <v/>
       </c>
       <c r="CB13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=67),"",$C$9+67)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=5),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+5)</f>
         <v/>
       </c>
       <c r="CC13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=68),"",$C$9+68)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=6),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+6)</f>
         <v/>
       </c>
       <c r="CD13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=69),"",$C$9+69)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=7),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+7)</f>
         <v/>
       </c>
       <c r="CE13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=70),"",$C$9+70)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=8),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+8)</f>
         <v/>
       </c>
       <c r="CF13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=71),"",$C$9+71)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=9),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+9)</f>
         <v/>
       </c>
       <c r="CG13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=72),"",$C$9+72)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=10),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+10)</f>
         <v/>
       </c>
       <c r="CH13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=73),"",$C$9+73)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=11),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+11)</f>
         <v/>
       </c>
       <c r="CI13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=74),"",$C$9+74)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=12),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+12)</f>
         <v/>
       </c>
       <c r="CJ13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=75),"",$C$9+75)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=13),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+13)</f>
         <v/>
       </c>
       <c r="CK13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=76),"",$C$9+76)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=14),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+14)</f>
         <v/>
       </c>
       <c r="CL13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=77),"",$C$9+77)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=15),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+15)</f>
         <v/>
       </c>
       <c r="CM13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=78),"",$C$9+78)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=16),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+16)</f>
         <v/>
       </c>
       <c r="CN13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=79),"",$C$9+79)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=17),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+17)</f>
         <v/>
       </c>
       <c r="CO13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=80),"",$C$9+80)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=18),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+18)</f>
         <v/>
       </c>
       <c r="CP13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=81),"",$C$9+81)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=19),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+19)</f>
         <v/>
       </c>
       <c r="CQ13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=82),"",$C$9+82)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=20),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+20)</f>
         <v/>
       </c>
       <c r="CR13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=83),"",$C$9+83)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=21),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+21)</f>
         <v/>
       </c>
       <c r="CS13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=84),"",$C$9+84)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=22),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+22)</f>
         <v/>
       </c>
       <c r="CT13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=85),"",$C$9+85)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=23),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+23)</f>
         <v/>
       </c>
       <c r="CU13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=86),"",$C$9+86)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=24),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+24)</f>
         <v/>
       </c>
       <c r="CV13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=87),"",$C$9+87)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=25),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+25)</f>
         <v/>
       </c>
       <c r="CW13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=88),"",$C$9+88)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=26),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+26)</f>
         <v/>
       </c>
       <c r="CX13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=89),"",$C$9+89)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=27),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+27)</f>
         <v/>
       </c>
       <c r="CY13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=90),"",$C$9+90)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=28),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+28)</f>
         <v/>
       </c>
       <c r="CZ13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=91),"",$C$9+91)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=29),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+29)</f>
         <v/>
       </c>
       <c r="DA13" s="17">
-        <f>IF(OR($C$9="",N($J$9)&lt;=92),"",$C$9+92)</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=30),"",DATE(YEAR($C$9),MONTH($C$9)+2,1)+30)</f>
         <v/>
       </c>
     </row>
@@ -1725,440 +1750,485 @@
       <c r="K14" s="18" t="n"/>
       <c r="L14" s="18" t="n"/>
       <c r="M14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=0),"",CHOOSE(WEEKDAY($C$9+0,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=0),"",CHOOSE(WEEKDAY($C$9+0,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="N14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=1),"",CHOOSE(WEEKDAY($C$9+1,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=1),"",CHOOSE(WEEKDAY($C$9+1,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="O14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=2),"",CHOOSE(WEEKDAY($C$9+2,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=2),"",CHOOSE(WEEKDAY($C$9+2,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="P14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=3),"",CHOOSE(WEEKDAY($C$9+3,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=3),"",CHOOSE(WEEKDAY($C$9+3,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="Q14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=4),"",CHOOSE(WEEKDAY($C$9+4,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=4),"",CHOOSE(WEEKDAY($C$9+4,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="R14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=5),"",CHOOSE(WEEKDAY($C$9+5,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=5),"",CHOOSE(WEEKDAY($C$9+5,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="S14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=6),"",CHOOSE(WEEKDAY($C$9+6,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=6),"",CHOOSE(WEEKDAY($C$9+6,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="T14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=7),"",CHOOSE(WEEKDAY($C$9+7,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=7),"",CHOOSE(WEEKDAY($C$9+7,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="U14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=8),"",CHOOSE(WEEKDAY($C$9+8,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=8),"",CHOOSE(WEEKDAY($C$9+8,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="V14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=9),"",CHOOSE(WEEKDAY($C$9+9,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=9),"",CHOOSE(WEEKDAY($C$9+9,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="W14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=10),"",CHOOSE(WEEKDAY($C$9+10,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=10),"",CHOOSE(WEEKDAY($C$9+10,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="X14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=11),"",CHOOSE(WEEKDAY($C$9+11,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=11),"",CHOOSE(WEEKDAY($C$9+11,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="Y14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=12),"",CHOOSE(WEEKDAY($C$9+12,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=12),"",CHOOSE(WEEKDAY($C$9+12,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="Z14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=13),"",CHOOSE(WEEKDAY($C$9+13,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=13),"",CHOOSE(WEEKDAY($C$9+13,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AA14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=14),"",CHOOSE(WEEKDAY($C$9+14,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=14),"",CHOOSE(WEEKDAY($C$9+14,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AB14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=15),"",CHOOSE(WEEKDAY($C$9+15,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=15),"",CHOOSE(WEEKDAY($C$9+15,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AC14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=16),"",CHOOSE(WEEKDAY($C$9+16,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=16),"",CHOOSE(WEEKDAY($C$9+16,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AD14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=17),"",CHOOSE(WEEKDAY($C$9+17,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=17),"",CHOOSE(WEEKDAY($C$9+17,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AE14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=18),"",CHOOSE(WEEKDAY($C$9+18,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=18),"",CHOOSE(WEEKDAY($C$9+18,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AF14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=19),"",CHOOSE(WEEKDAY($C$9+19,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=19),"",CHOOSE(WEEKDAY($C$9+19,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AG14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=20),"",CHOOSE(WEEKDAY($C$9+20,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=20),"",CHOOSE(WEEKDAY($C$9+20,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AH14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=21),"",CHOOSE(WEEKDAY($C$9+21,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=21),"",CHOOSE(WEEKDAY($C$9+21,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AI14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=22),"",CHOOSE(WEEKDAY($C$9+22,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=22),"",CHOOSE(WEEKDAY($C$9+22,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AJ14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=23),"",CHOOSE(WEEKDAY($C$9+23,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=23),"",CHOOSE(WEEKDAY($C$9+23,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AK14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=24),"",CHOOSE(WEEKDAY($C$9+24,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=24),"",CHOOSE(WEEKDAY($C$9+24,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AL14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=25),"",CHOOSE(WEEKDAY($C$9+25,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=25),"",CHOOSE(WEEKDAY($C$9+25,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AM14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=26),"",CHOOSE(WEEKDAY($C$9+26,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=26),"",CHOOSE(WEEKDAY($C$9+26,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AN14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=27),"",CHOOSE(WEEKDAY($C$9+27,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=27),"",CHOOSE(WEEKDAY($C$9+27,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AO14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=28),"",CHOOSE(WEEKDAY($C$9+28,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=28),"",CHOOSE(WEEKDAY($C$9+28,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AP14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=29),"",CHOOSE(WEEKDAY($C$9+29,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=29),"",CHOOSE(WEEKDAY($C$9+29,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AQ14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=30),"",CHOOSE(WEEKDAY($C$9+30,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DD$9)&lt;=30),"",CHOOSE(WEEKDAY($C$9+30,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AR14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=31),"",CHOOSE(WEEKDAY($C$9+31,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=0),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+0,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AS14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=32),"",CHOOSE(WEEKDAY($C$9+32,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=1),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+1,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AT14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=33),"",CHOOSE(WEEKDAY($C$9+33,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=2),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+2,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AU14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=34),"",CHOOSE(WEEKDAY($C$9+34,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=3),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+3,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AV14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=35),"",CHOOSE(WEEKDAY($C$9+35,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=4),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+4,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AW14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=36),"",CHOOSE(WEEKDAY($C$9+36,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=5),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+5,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AX14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=37),"",CHOOSE(WEEKDAY($C$9+37,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=6),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+6,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AY14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=38),"",CHOOSE(WEEKDAY($C$9+38,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=7),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+7,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="AZ14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=39),"",CHOOSE(WEEKDAY($C$9+39,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=8),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+8,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BA14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=40),"",CHOOSE(WEEKDAY($C$9+40,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=9),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+9,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BB14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=41),"",CHOOSE(WEEKDAY($C$9+41,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=10),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+10,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BC14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=42),"",CHOOSE(WEEKDAY($C$9+42,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=11),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+11,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BD14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=43),"",CHOOSE(WEEKDAY($C$9+43,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=12),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+12,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BE14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=44),"",CHOOSE(WEEKDAY($C$9+44,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=13),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+13,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BF14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=45),"",CHOOSE(WEEKDAY($C$9+45,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=14),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+14,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BG14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=46),"",CHOOSE(WEEKDAY($C$9+46,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=15),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+15,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BH14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=47),"",CHOOSE(WEEKDAY($C$9+47,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=16),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+16,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BI14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=48),"",CHOOSE(WEEKDAY($C$9+48,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=17),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+17,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BJ14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=49),"",CHOOSE(WEEKDAY($C$9+49,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=18),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+18,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BK14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=50),"",CHOOSE(WEEKDAY($C$9+50,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=19),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+19,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BL14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=51),"",CHOOSE(WEEKDAY($C$9+51,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=20),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+20,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BM14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=52),"",CHOOSE(WEEKDAY($C$9+52,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=21),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+21,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BN14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=53),"",CHOOSE(WEEKDAY($C$9+53,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=22),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+22,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BO14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=54),"",CHOOSE(WEEKDAY($C$9+54,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=23),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+23,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BP14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=55),"",CHOOSE(WEEKDAY($C$9+55,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=24),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+24,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BQ14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=56),"",CHOOSE(WEEKDAY($C$9+56,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=25),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+25,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BR14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=57),"",CHOOSE(WEEKDAY($C$9+57,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=26),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+26,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BS14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=58),"",CHOOSE(WEEKDAY($C$9+58,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=27),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+27,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BT14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=59),"",CHOOSE(WEEKDAY($C$9+59,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=28),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+28,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BU14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=60),"",CHOOSE(WEEKDAY($C$9+60,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=29),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+29,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BV14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=61),"",CHOOSE(WEEKDAY($C$9+61,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DE$9)&lt;=30),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+1,1)+30,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BW14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=62),"",CHOOSE(WEEKDAY($C$9+62,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=0),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+0,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BX14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=63),"",CHOOSE(WEEKDAY($C$9+63,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=1),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+1,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BY14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=64),"",CHOOSE(WEEKDAY($C$9+64,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=2),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+2,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="BZ14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=65),"",CHOOSE(WEEKDAY($C$9+65,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=3),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+3,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CA14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=66),"",CHOOSE(WEEKDAY($C$9+66,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=4),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+4,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CB14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=67),"",CHOOSE(WEEKDAY($C$9+67,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=5),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+5,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CC14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=68),"",CHOOSE(WEEKDAY($C$9+68,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=6),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+6,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CD14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=69),"",CHOOSE(WEEKDAY($C$9+69,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=7),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+7,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CE14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=70),"",CHOOSE(WEEKDAY($C$9+70,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=8),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+8,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CF14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=71),"",CHOOSE(WEEKDAY($C$9+71,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=9),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+9,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CG14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=72),"",CHOOSE(WEEKDAY($C$9+72,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=10),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+10,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CH14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=73),"",CHOOSE(WEEKDAY($C$9+73,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=11),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+11,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CI14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=74),"",CHOOSE(WEEKDAY($C$9+74,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=12),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+12,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CJ14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=75),"",CHOOSE(WEEKDAY($C$9+75,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=13),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+13,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CK14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=76),"",CHOOSE(WEEKDAY($C$9+76,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=14),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+14,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CL14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=77),"",CHOOSE(WEEKDAY($C$9+77,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=15),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+15,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CM14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=78),"",CHOOSE(WEEKDAY($C$9+78,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=16),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+16,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CN14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=79),"",CHOOSE(WEEKDAY($C$9+79,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=17),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+17,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CO14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=80),"",CHOOSE(WEEKDAY($C$9+80,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=18),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+18,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CP14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=81),"",CHOOSE(WEEKDAY($C$9+81,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=19),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+19,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CQ14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=82),"",CHOOSE(WEEKDAY($C$9+82,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=20),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+20,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CR14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=83),"",CHOOSE(WEEKDAY($C$9+83,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=21),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+21,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CS14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=84),"",CHOOSE(WEEKDAY($C$9+84,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=22),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+22,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CT14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=85),"",CHOOSE(WEEKDAY($C$9+85,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=23),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+23,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CU14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=86),"",CHOOSE(WEEKDAY($C$9+86,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=24),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+24,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CV14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=87),"",CHOOSE(WEEKDAY($C$9+87,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=25),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+25,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CW14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=88),"",CHOOSE(WEEKDAY($C$9+88,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=26),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+26,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CX14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=89),"",CHOOSE(WEEKDAY($C$9+89,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=27),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+27,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CY14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=90),"",CHOOSE(WEEKDAY($C$9+90,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=28),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+28,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="CZ14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=91),"",CHOOSE(WEEKDAY($C$9+91,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=29),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+29,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="DA14" s="19">
-        <f>IF(OR($C$9="",N($J$9)&lt;=92),"",CHOOSE(WEEKDAY($C$9+92,2),"L","M","M","J","V","S","D"))</f>
+        <f>IF(OR($C$9="",N($DF$9)&lt;=30),"",CHOOSE(WEEKDAY(DATE(YEAR($C$9),MONTH($C$9)+2,1)+30,2),"L","M","M","J","V","S","D"))</f>
         <v/>
       </c>
       <c r="DC14" t="inlineStr">
         <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="DD14" t="inlineStr">
+        <is>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="DE14" t="inlineStr">
+        <is>
+          <t>mob1</t>
+        </is>
+      </c>
+      <c r="DF14" t="inlineStr">
+        <is>
           <t>loc1</t>
         </is>
       </c>
-      <c r="DD14" t="inlineStr">
+      <c r="DG14" t="inlineStr">
         <is>
           <t>uc1</t>
         </is>
       </c>
-      <c r="DE14" t="inlineStr">
+      <c r="DH14" t="inlineStr">
         <is>
           <t>vr1</t>
         </is>
       </c>
-      <c r="DF14" t="inlineStr">
+      <c r="DI14" t="inlineStr">
         <is>
           <t>foc1</t>
         </is>
       </c>
-      <c r="DG14" t="inlineStr">
+      <c r="DJ14" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="DK14" t="inlineStr">
+        <is>
+          <t>O2</t>
+        </is>
+      </c>
+      <c r="DL14" t="inlineStr">
+        <is>
+          <t>mob2</t>
+        </is>
+      </c>
+      <c r="DM14" t="inlineStr">
         <is>
           <t>loc2</t>
         </is>
       </c>
-      <c r="DH14" t="inlineStr">
+      <c r="DN14" t="inlineStr">
         <is>
           <t>uc2</t>
         </is>
       </c>
-      <c r="DI14" t="inlineStr">
+      <c r="DO14" t="inlineStr">
         <is>
           <t>vr2</t>
         </is>
       </c>
-      <c r="DJ14" t="inlineStr">
+      <c r="DP14" t="inlineStr">
         <is>
           <t>foc2</t>
         </is>
       </c>
-      <c r="DK14" t="inlineStr">
+      <c r="DQ14" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="DR14" t="inlineStr">
+        <is>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="DS14" t="inlineStr">
+        <is>
+          <t>mob3</t>
+        </is>
+      </c>
+      <c r="DT14" t="inlineStr">
         <is>
           <t>loc3</t>
         </is>
       </c>
-      <c r="DL14" t="inlineStr">
+      <c r="DU14" t="inlineStr">
         <is>
           <t>uc3</t>
         </is>
       </c>
-      <c r="DM14" t="inlineStr">
+      <c r="DV14" t="inlineStr">
         <is>
           <t>vr3</t>
         </is>
       </c>
-      <c r="DN14" t="inlineStr">
+      <c r="DW14" t="inlineStr">
         <is>
           <t>foc3</t>
         </is>
       </c>
-      <c r="DO14" t="inlineStr">
-        <is>
-          <t>bloc 1er O</t>
+      <c r="DX14" t="inlineStr">
+        <is>
+          <t>mois 1er O</t>
         </is>
       </c>
     </row>
@@ -2336,19 +2406,19 @@
       <c r="G17" s="26" t="n"/>
       <c r="H17" s="26" t="n"/>
       <c r="I17" s="27">
-        <f>COUNTIF($M17:INDEX($M17:$DA17,MAX(1,N($J$9))),"MOB")+COUNTIF($M17:INDEX($M17:$DA17,MAX(1,N($J$9))),"DEMOB")</f>
+        <f>DE17+DL17+DS17</f>
         <v/>
       </c>
       <c r="J17" s="28">
-        <f>COUNTIF($M17:INDEX($M17:$DA17,MAX(1,N($J$9))),"S")+COUNTIF($M17:INDEX($M17:$DA17,MAX(1,N($J$9))),"MOB")+COUNTIF($M17:INDEX($M17:$DA17,MAX(1,N($J$9))),"DEMOB")</f>
+        <f>DC17+DJ17+DQ17</f>
         <v/>
       </c>
       <c r="K17" s="28">
-        <f>COUNTIF($M17:INDEX($M17:$DA17,MAX(1,N($J$9))),"O")</f>
+        <f>DD17+DK17+DR17</f>
         <v/>
       </c>
       <c r="L17" s="29">
-        <f>IF(B17="","",DC17+DG17+DK17+DD17+DH17+DL17)</f>
+        <f>IF(B17="","",DF17+DM17+DT17+DG17+DN17+DU17)</f>
         <v/>
       </c>
       <c r="M17" s="30" t="n"/>
@@ -2445,48 +2515,84 @@
       <c r="CZ17" s="30" t="n"/>
       <c r="DA17" s="30" t="n"/>
       <c r="DC17" s="31">
-        <f>IF(OR(B17="",N($J$9)&lt;=0),0,(COUNTIF(INDEX($M17:$DA17,1):INDEX($M17:$DA17,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M17:$DA17,1):INDEX($M17:$DA17,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M17:$DA17,1):INDEX($M17:$DA17,MIN(31,N($J$9))),"DEMOB"))*N(D17)+(COUNTIF(INDEX($M17:$DA17,1):INDEX($M17:$DA17,MIN(31,N($J$9))),"O"))*N(E17))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M17:$DA17,1):INDEX($M17:$DA17,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M17:$DA17,1):INDEX($M17:$DA17,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M17:$DA17,1):INDEX($M17:$DA17,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD17" s="31">
-        <f>IF(OR(B17="",N($J$9)&lt;=0),0,(COUNTIF(INDEX($M17:$DA17,1):INDEX($M17:$DA17,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M17:$DA17,1):INDEX($M17:$DA17,MIN(31,N($J$9))),"DEMOB"))*N(F17))</f>
-        <v/>
-      </c>
-      <c r="DE17" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DF17" s="31" t="n">
-        <v>0</v>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M17:$DA17,1):INDEX($M17:$DA17,0+MAX(1,N($DD$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DE17" s="31">
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M17:$DA17,1):INDEX($M17:$DA17,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M17:$DA17,1):INDEX($M17:$DA17,0+MAX(1,N($DD$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DF17" s="31">
+        <f>IF(B17="",0,DC17*N(D17)+DD17*N(E17))</f>
+        <v/>
       </c>
       <c r="DG17" s="31">
-        <f>IF(OR(B17="",N($J$9)&lt;=31),0,(COUNTIF(INDEX($M17:$DA17,32):INDEX($M17:$DA17,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M17:$DA17,32):INDEX($M17:$DA17,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M17:$DA17,32):INDEX($M17:$DA17,MIN(62,N($J$9))),"DEMOB"))*N(D17)+(COUNTIF(INDEX($M17:$DA17,32):INDEX($M17:$DA17,MIN(62,N($J$9))),"O"))*N(E17))</f>
-        <v/>
-      </c>
-      <c r="DH17" s="31">
-        <f>IF(OR(B17="",N($J$9)&lt;=31),0,(COUNTIF(INDEX($M17:$DA17,32):INDEX($M17:$DA17,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M17:$DA17,32):INDEX($M17:$DA17,MIN(62,N($J$9))),"DEMOB"))*N(F17))</f>
-        <v/>
+        <f>IF(B17="",0,DE17*N(F17))</f>
+        <v/>
+      </c>
+      <c r="DH17" s="31" t="n">
+        <v>0</v>
       </c>
       <c r="DI17" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="DJ17" s="31" t="n">
-        <v>0</v>
+      <c r="DJ17" s="31">
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M17:$DA17,32):INDEX($M17:$DA17,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M17:$DA17,32):INDEX($M17:$DA17,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M17:$DA17,32):INDEX($M17:$DA17,31+MAX(1,N($DE$9))),"DEMOB"))</f>
+        <v/>
       </c>
       <c r="DK17" s="31">
-        <f>IF(OR(B17="",N($J$9)&lt;=62),0,(COUNTIF(INDEX($M17:$DA17,63):INDEX($M17:$DA17,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M17:$DA17,63):INDEX($M17:$DA17,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M17:$DA17,63):INDEX($M17:$DA17,MIN(93,N($J$9))),"DEMOB"))*N(D17)+(COUNTIF(INDEX($M17:$DA17,63):INDEX($M17:$DA17,MIN(93,N($J$9))),"O"))*N(E17))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M17:$DA17,32):INDEX($M17:$DA17,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL17" s="31">
-        <f>IF(OR(B17="",N($J$9)&lt;=62),0,(COUNTIF(INDEX($M17:$DA17,63):INDEX($M17:$DA17,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M17:$DA17,63):INDEX($M17:$DA17,MIN(93,N($J$9))),"DEMOB"))*N(F17))</f>
-        <v/>
-      </c>
-      <c r="DM17" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DN17" s="31" t="n">
-        <v>0</v>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M17:$DA17,32):INDEX($M17:$DA17,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M17:$DA17,32):INDEX($M17:$DA17,31+MAX(1,N($DE$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DM17" s="31">
+        <f>IF(B17="",0,DJ17*N(D17)+DK17*N(E17))</f>
+        <v/>
+      </c>
+      <c r="DN17" s="31">
+        <f>IF(B17="",0,DL17*N(F17))</f>
+        <v/>
       </c>
       <c r="DO17" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP17" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DQ17" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M17:$DA17,63):INDEX($M17:$DA17,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M17:$DA17,63):INDEX($M17:$DA17,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M17:$DA17,63):INDEX($M17:$DA17,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR17" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M17:$DA17,63):INDEX($M17:$DA17,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS17" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M17:$DA17,63):INDEX($M17:$DA17,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M17:$DA17,63):INDEX($M17:$DA17,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT17" s="31">
+        <f>IF(B17="",0,DQ17*N(D17)+DR17*N(E17))</f>
+        <v/>
+      </c>
+      <c r="DU17" s="31">
+        <f>IF(B17="",0,DS17*N(F17))</f>
+        <v/>
+      </c>
+      <c r="DV17" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW17" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX17" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2500,19 +2606,19 @@
       <c r="G18" s="26" t="n"/>
       <c r="H18" s="26" t="n"/>
       <c r="I18" s="27">
-        <f>COUNTIF($M18:INDEX($M18:$DA18,MAX(1,N($J$9))),"MOB")+COUNTIF($M18:INDEX($M18:$DA18,MAX(1,N($J$9))),"DEMOB")</f>
+        <f>DE18+DL18+DS18</f>
         <v/>
       </c>
       <c r="J18" s="28">
-        <f>COUNTIF($M18:INDEX($M18:$DA18,MAX(1,N($J$9))),"S")+COUNTIF($M18:INDEX($M18:$DA18,MAX(1,N($J$9))),"MOB")+COUNTIF($M18:INDEX($M18:$DA18,MAX(1,N($J$9))),"DEMOB")</f>
+        <f>DC18+DJ18+DQ18</f>
         <v/>
       </c>
       <c r="K18" s="28">
-        <f>COUNTIF($M18:INDEX($M18:$DA18,MAX(1,N($J$9))),"O")</f>
+        <f>DD18+DK18+DR18</f>
         <v/>
       </c>
       <c r="L18" s="29">
-        <f>IF(B18="","",DC18+DG18+DK18+DD18+DH18+DL18)</f>
+        <f>IF(B18="","",DF18+DM18+DT18+DG18+DN18+DU18)</f>
         <v/>
       </c>
       <c r="M18" s="30" t="n"/>
@@ -2609,48 +2715,84 @@
       <c r="CZ18" s="30" t="n"/>
       <c r="DA18" s="30" t="n"/>
       <c r="DC18" s="31">
-        <f>IF(OR(B18="",N($J$9)&lt;=0),0,(COUNTIF(INDEX($M18:$DA18,1):INDEX($M18:$DA18,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M18:$DA18,1):INDEX($M18:$DA18,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M18:$DA18,1):INDEX($M18:$DA18,MIN(31,N($J$9))),"DEMOB"))*N(D18)+(COUNTIF(INDEX($M18:$DA18,1):INDEX($M18:$DA18,MIN(31,N($J$9))),"O"))*N(E18))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M18:$DA18,1):INDEX($M18:$DA18,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M18:$DA18,1):INDEX($M18:$DA18,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M18:$DA18,1):INDEX($M18:$DA18,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD18" s="31">
-        <f>IF(OR(B18="",N($J$9)&lt;=0),0,(COUNTIF(INDEX($M18:$DA18,1):INDEX($M18:$DA18,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M18:$DA18,1):INDEX($M18:$DA18,MIN(31,N($J$9))),"DEMOB"))*N(F18))</f>
-        <v/>
-      </c>
-      <c r="DE18" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DF18" s="31" t="n">
-        <v>0</v>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M18:$DA18,1):INDEX($M18:$DA18,0+MAX(1,N($DD$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DE18" s="31">
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M18:$DA18,1):INDEX($M18:$DA18,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M18:$DA18,1):INDEX($M18:$DA18,0+MAX(1,N($DD$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DF18" s="31">
+        <f>IF(B18="",0,DC18*N(D18)+DD18*N(E18))</f>
+        <v/>
       </c>
       <c r="DG18" s="31">
-        <f>IF(OR(B18="",N($J$9)&lt;=31),0,(COUNTIF(INDEX($M18:$DA18,32):INDEX($M18:$DA18,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M18:$DA18,32):INDEX($M18:$DA18,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M18:$DA18,32):INDEX($M18:$DA18,MIN(62,N($J$9))),"DEMOB"))*N(D18)+(COUNTIF(INDEX($M18:$DA18,32):INDEX($M18:$DA18,MIN(62,N($J$9))),"O"))*N(E18))</f>
-        <v/>
-      </c>
-      <c r="DH18" s="31">
-        <f>IF(OR(B18="",N($J$9)&lt;=31),0,(COUNTIF(INDEX($M18:$DA18,32):INDEX($M18:$DA18,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M18:$DA18,32):INDEX($M18:$DA18,MIN(62,N($J$9))),"DEMOB"))*N(F18))</f>
-        <v/>
+        <f>IF(B18="",0,DE18*N(F18))</f>
+        <v/>
+      </c>
+      <c r="DH18" s="31" t="n">
+        <v>0</v>
       </c>
       <c r="DI18" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="DJ18" s="31" t="n">
-        <v>0</v>
+      <c r="DJ18" s="31">
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M18:$DA18,32):INDEX($M18:$DA18,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M18:$DA18,32):INDEX($M18:$DA18,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M18:$DA18,32):INDEX($M18:$DA18,31+MAX(1,N($DE$9))),"DEMOB"))</f>
+        <v/>
       </c>
       <c r="DK18" s="31">
-        <f>IF(OR(B18="",N($J$9)&lt;=62),0,(COUNTIF(INDEX($M18:$DA18,63):INDEX($M18:$DA18,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M18:$DA18,63):INDEX($M18:$DA18,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M18:$DA18,63):INDEX($M18:$DA18,MIN(93,N($J$9))),"DEMOB"))*N(D18)+(COUNTIF(INDEX($M18:$DA18,63):INDEX($M18:$DA18,MIN(93,N($J$9))),"O"))*N(E18))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M18:$DA18,32):INDEX($M18:$DA18,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL18" s="31">
-        <f>IF(OR(B18="",N($J$9)&lt;=62),0,(COUNTIF(INDEX($M18:$DA18,63):INDEX($M18:$DA18,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M18:$DA18,63):INDEX($M18:$DA18,MIN(93,N($J$9))),"DEMOB"))*N(F18))</f>
-        <v/>
-      </c>
-      <c r="DM18" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DN18" s="31" t="n">
-        <v>0</v>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M18:$DA18,32):INDEX($M18:$DA18,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M18:$DA18,32):INDEX($M18:$DA18,31+MAX(1,N($DE$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DM18" s="31">
+        <f>IF(B18="",0,DJ18*N(D18)+DK18*N(E18))</f>
+        <v/>
+      </c>
+      <c r="DN18" s="31">
+        <f>IF(B18="",0,DL18*N(F18))</f>
+        <v/>
       </c>
       <c r="DO18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DQ18" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M18:$DA18,63):INDEX($M18:$DA18,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M18:$DA18,63):INDEX($M18:$DA18,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M18:$DA18,63):INDEX($M18:$DA18,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR18" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M18:$DA18,63):INDEX($M18:$DA18,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS18" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M18:$DA18,63):INDEX($M18:$DA18,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M18:$DA18,63):INDEX($M18:$DA18,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT18" s="31">
+        <f>IF(B18="",0,DQ18*N(D18)+DR18*N(E18))</f>
+        <v/>
+      </c>
+      <c r="DU18" s="31">
+        <f>IF(B18="",0,DS18*N(F18))</f>
+        <v/>
+      </c>
+      <c r="DV18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX18" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2664,19 +2806,19 @@
       <c r="G19" s="26" t="n"/>
       <c r="H19" s="26" t="n"/>
       <c r="I19" s="27">
-        <f>COUNTIF($M19:INDEX($M19:$DA19,MAX(1,N($J$9))),"MOB")+COUNTIF($M19:INDEX($M19:$DA19,MAX(1,N($J$9))),"DEMOB")</f>
+        <f>DE19+DL19+DS19</f>
         <v/>
       </c>
       <c r="J19" s="28">
-        <f>COUNTIF($M19:INDEX($M19:$DA19,MAX(1,N($J$9))),"S")+COUNTIF($M19:INDEX($M19:$DA19,MAX(1,N($J$9))),"MOB")+COUNTIF($M19:INDEX($M19:$DA19,MAX(1,N($J$9))),"DEMOB")</f>
+        <f>DC19+DJ19+DQ19</f>
         <v/>
       </c>
       <c r="K19" s="28">
-        <f>COUNTIF($M19:INDEX($M19:$DA19,MAX(1,N($J$9))),"O")</f>
+        <f>DD19+DK19+DR19</f>
         <v/>
       </c>
       <c r="L19" s="29">
-        <f>IF(B19="","",DC19+DG19+DK19+DD19+DH19+DL19)</f>
+        <f>IF(B19="","",DF19+DM19+DT19+DG19+DN19+DU19)</f>
         <v/>
       </c>
       <c r="M19" s="30" t="n"/>
@@ -2773,48 +2915,84 @@
       <c r="CZ19" s="30" t="n"/>
       <c r="DA19" s="30" t="n"/>
       <c r="DC19" s="31">
-        <f>IF(OR(B19="",N($J$9)&lt;=0),0,(COUNTIF(INDEX($M19:$DA19,1):INDEX($M19:$DA19,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M19:$DA19,1):INDEX($M19:$DA19,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M19:$DA19,1):INDEX($M19:$DA19,MIN(31,N($J$9))),"DEMOB"))*N(D19)+(COUNTIF(INDEX($M19:$DA19,1):INDEX($M19:$DA19,MIN(31,N($J$9))),"O"))*N(E19))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M19:$DA19,1):INDEX($M19:$DA19,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M19:$DA19,1):INDEX($M19:$DA19,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M19:$DA19,1):INDEX($M19:$DA19,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD19" s="31">
-        <f>IF(OR(B19="",N($J$9)&lt;=0),0,(COUNTIF(INDEX($M19:$DA19,1):INDEX($M19:$DA19,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M19:$DA19,1):INDEX($M19:$DA19,MIN(31,N($J$9))),"DEMOB"))*N(F19))</f>
-        <v/>
-      </c>
-      <c r="DE19" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DF19" s="31" t="n">
-        <v>0</v>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M19:$DA19,1):INDEX($M19:$DA19,0+MAX(1,N($DD$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DE19" s="31">
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M19:$DA19,1):INDEX($M19:$DA19,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M19:$DA19,1):INDEX($M19:$DA19,0+MAX(1,N($DD$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DF19" s="31">
+        <f>IF(B19="",0,DC19*N(D19)+DD19*N(E19))</f>
+        <v/>
       </c>
       <c r="DG19" s="31">
-        <f>IF(OR(B19="",N($J$9)&lt;=31),0,(COUNTIF(INDEX($M19:$DA19,32):INDEX($M19:$DA19,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M19:$DA19,32):INDEX($M19:$DA19,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M19:$DA19,32):INDEX($M19:$DA19,MIN(62,N($J$9))),"DEMOB"))*N(D19)+(COUNTIF(INDEX($M19:$DA19,32):INDEX($M19:$DA19,MIN(62,N($J$9))),"O"))*N(E19))</f>
-        <v/>
-      </c>
-      <c r="DH19" s="31">
-        <f>IF(OR(B19="",N($J$9)&lt;=31),0,(COUNTIF(INDEX($M19:$DA19,32):INDEX($M19:$DA19,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M19:$DA19,32):INDEX($M19:$DA19,MIN(62,N($J$9))),"DEMOB"))*N(F19))</f>
-        <v/>
+        <f>IF(B19="",0,DE19*N(F19))</f>
+        <v/>
+      </c>
+      <c r="DH19" s="31" t="n">
+        <v>0</v>
       </c>
       <c r="DI19" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="DJ19" s="31" t="n">
-        <v>0</v>
+      <c r="DJ19" s="31">
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M19:$DA19,32):INDEX($M19:$DA19,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M19:$DA19,32):INDEX($M19:$DA19,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M19:$DA19,32):INDEX($M19:$DA19,31+MAX(1,N($DE$9))),"DEMOB"))</f>
+        <v/>
       </c>
       <c r="DK19" s="31">
-        <f>IF(OR(B19="",N($J$9)&lt;=62),0,(COUNTIF(INDEX($M19:$DA19,63):INDEX($M19:$DA19,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M19:$DA19,63):INDEX($M19:$DA19,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M19:$DA19,63):INDEX($M19:$DA19,MIN(93,N($J$9))),"DEMOB"))*N(D19)+(COUNTIF(INDEX($M19:$DA19,63):INDEX($M19:$DA19,MIN(93,N($J$9))),"O"))*N(E19))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M19:$DA19,32):INDEX($M19:$DA19,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL19" s="31">
-        <f>IF(OR(B19="",N($J$9)&lt;=62),0,(COUNTIF(INDEX($M19:$DA19,63):INDEX($M19:$DA19,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M19:$DA19,63):INDEX($M19:$DA19,MIN(93,N($J$9))),"DEMOB"))*N(F19))</f>
-        <v/>
-      </c>
-      <c r="DM19" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DN19" s="31" t="n">
-        <v>0</v>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M19:$DA19,32):INDEX($M19:$DA19,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M19:$DA19,32):INDEX($M19:$DA19,31+MAX(1,N($DE$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DM19" s="31">
+        <f>IF(B19="",0,DJ19*N(D19)+DK19*N(E19))</f>
+        <v/>
+      </c>
+      <c r="DN19" s="31">
+        <f>IF(B19="",0,DL19*N(F19))</f>
+        <v/>
       </c>
       <c r="DO19" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP19" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DQ19" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M19:$DA19,63):INDEX($M19:$DA19,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M19:$DA19,63):INDEX($M19:$DA19,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M19:$DA19,63):INDEX($M19:$DA19,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR19" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M19:$DA19,63):INDEX($M19:$DA19,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS19" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M19:$DA19,63):INDEX($M19:$DA19,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M19:$DA19,63):INDEX($M19:$DA19,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT19" s="31">
+        <f>IF(B19="",0,DQ19*N(D19)+DR19*N(E19))</f>
+        <v/>
+      </c>
+      <c r="DU19" s="31">
+        <f>IF(B19="",0,DS19*N(F19))</f>
+        <v/>
+      </c>
+      <c r="DV19" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW19" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX19" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2940,15 +3118,15 @@
       <c r="H22" s="25" t="n"/>
       <c r="I22" s="25" t="n"/>
       <c r="J22" s="28">
-        <f>IF(B22="","",COUNTIF($M22:INDEX($M22:$DA22,MAX(1,N($J$9))),"S")+COUNTIF($M22:INDEX($M22:$DA22,MAX(1,N($J$9))),"MOB")+COUNTIF($M22:INDEX($M22:$DA22,MAX(1,N($J$9))),"DEMOB"))</f>
+        <f>IF(B22="","",DC22+DJ22+DQ22)</f>
         <v/>
       </c>
       <c r="K22" s="28">
-        <f>IF(B22="","",COUNTIF($M22:INDEX($M22:$DA22,MAX(1,N($J$9))),"O"))</f>
+        <f>IF(B22="","",DD22+DK22+DR22)</f>
         <v/>
       </c>
       <c r="L22" s="29">
-        <f>IF(B22="","",DC22+DG22+DK22+DD22+DH22+DL22+DE22+DI22+DM22)</f>
+        <f>IF(B22="","",DF22+DM22+DT22+DG22+DN22+DU22+DH22+DO22+DV22)</f>
         <v/>
       </c>
       <c r="M22" s="30" t="n"/>
@@ -3045,55 +3223,91 @@
       <c r="CZ22" s="30" t="n"/>
       <c r="DA22" s="30" t="n"/>
       <c r="DC22" s="31">
-        <f>IF(OR(B22="",NOT(N($J$9)&gt;0)),0,IF(N(C22)&gt;0,C22,1)*((COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,MIN(31,N($J$9))),"DEMOB"))*N(D22)+(COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,MIN(31,N($J$9))),"O"))*N(E22)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD22" s="31">
-        <f>IF(OR(B22="",A22="Oui",DO22&lt;&gt;1),0,IF(N(C22)&gt;0,C22,1)*(N(F22)+N(H22)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,0+MAX(1,N($DD$9))),"O"))</f>
         <v/>
       </c>
       <c r="DE22" s="31">
-        <f>IF(OR(B22="",NOT(N($J$9)&gt;0)),0,IF(N(C22)&gt;0,C22,1)*(IF((COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,MIN(31,N($J$9))),"VR"))&gt;0,N(G22),0)+IF((COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,MIN(31,N($J$9))),"RC"))&gt;0,N(I22),0)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DF22" s="31">
-        <f>IF(OR(B22="",NOT(N($J$9)&gt;0)),0,IF(N(C22)&gt;0,C22,1)*(COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,MIN(31,N($J$9))),"FOC"))*N(E22))</f>
+        <f>IF(B22="",0,IF(N(C22)&gt;0,C22,1)*(DC22*N(D22)+DD22*N(E22)))</f>
         <v/>
       </c>
       <c r="DG22" s="31">
-        <f>IF(OR(B22="",NOT(N($J$9)&gt;31)),0,IF(N(C22)&gt;0,C22,1)*((COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,MIN(62,N($J$9))),"DEMOB"))*N(D22)+(COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,MIN(62,N($J$9))),"O"))*N(E22)))</f>
+        <f>IF(OR(B22="",A22="Oui",DX22&lt;&gt;1),0,IF(N(C22)&gt;0,C22,1)*(N(F22)+N(H22)))</f>
         <v/>
       </c>
       <c r="DH22" s="31">
-        <f>IF(OR(B22="",A22="Oui",DO22&lt;&gt;2),0,IF(N(C22)&gt;0,C22,1)*(N(F22)+N(H22)))</f>
+        <f>IF(OR(B22="",N($DD$9)=0),0,IF(N(C22)&gt;0,C22,1)*(IF((COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,0+MAX(1,N($DD$9))),"VR"))&gt;0,N(G22),0)+IF((COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,0+MAX(1,N($DD$9))),"RC"))&gt;0,N(I22),0)))</f>
         <v/>
       </c>
       <c r="DI22" s="31">
-        <f>IF(OR(B22="",NOT(N($J$9)&gt;31)),0,IF(N(C22)&gt;0,C22,1)*(IF((COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,MIN(62,N($J$9))),"VR"))&gt;0,N(G22),0)+IF((COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,MIN(62,N($J$9))),"RC"))&gt;0,N(I22),0)))</f>
+        <f>IF(OR(B22="",N($DD$9)=0),0,IF(N(C22)&gt;0,C22,1)*(COUNTIF(INDEX($M22:$DA22,1):INDEX($M22:$DA22,0+MAX(1,N($DD$9))),"FOC"))*N(E22))</f>
         <v/>
       </c>
       <c r="DJ22" s="31">
-        <f>IF(OR(B22="",NOT(N($J$9)&gt;31)),0,IF(N(C22)&gt;0,C22,1)*(COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,MIN(62,N($J$9))),"FOC"))*N(E22))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DK22" s="31">
-        <f>IF(OR(B22="",NOT(N($J$9)&gt;62)),0,IF(N(C22)&gt;0,C22,1)*((COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,MIN(93,N($J$9))),"DEMOB"))*N(D22)+(COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,MIN(93,N($J$9))),"O"))*N(E22)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL22" s="31">
-        <f>IF(OR(B22="",A22="Oui",DO22&lt;&gt;3),0,IF(N(C22)&gt;0,C22,1)*(N(F22)+N(H22)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DM22" s="31">
-        <f>IF(OR(B22="",NOT(N($J$9)&gt;62)),0,IF(N(C22)&gt;0,C22,1)*(IF((COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,MIN(93,N($J$9))),"VR"))&gt;0,N(G22),0)+IF((COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,MIN(93,N($J$9))),"RC"))&gt;0,N(I22),0)))</f>
+        <f>IF(B22="",0,IF(N(C22)&gt;0,C22,1)*(DJ22*N(D22)+DK22*N(E22)))</f>
         <v/>
       </c>
       <c r="DN22" s="31">
-        <f>IF(OR(B22="",NOT(N($J$9)&gt;62)),0,IF(N(C22)&gt;0,C22,1)*(COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,MIN(93,N($J$9))),"FOC"))*N(E22))</f>
+        <f>IF(OR(B22="",A22="Oui",DX22&lt;&gt;2),0,IF(N(C22)&gt;0,C22,1)*(N(F22)+N(H22)))</f>
         <v/>
       </c>
       <c r="DO22" s="31">
-        <f>IF(B22="",0,IFERROR(INT((MATCH("O",$M22:INDEX($M22:$DA22,MAX(1,N($J$9))),0)-1)/31)+1,0))</f>
+        <f>IF(OR(B22="",N($DE$9)=0),0,IF(N(C22)&gt;0,C22,1)*(IF((COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,31+MAX(1,N($DE$9))),"VR"))&gt;0,N(G22),0)+IF((COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,31+MAX(1,N($DE$9))),"RC"))&gt;0,N(I22),0)))</f>
+        <v/>
+      </c>
+      <c r="DP22" s="31">
+        <f>IF(OR(B22="",N($DE$9)=0),0,IF(N(C22)&gt;0,C22,1)*(COUNTIF(INDEX($M22:$DA22,32):INDEX($M22:$DA22,31+MAX(1,N($DE$9))),"FOC"))*N(E22))</f>
+        <v/>
+      </c>
+      <c r="DQ22" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR22" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS22" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT22" s="31">
+        <f>IF(B22="",0,IF(N(C22)&gt;0,C22,1)*(DQ22*N(D22)+DR22*N(E22)))</f>
+        <v/>
+      </c>
+      <c r="DU22" s="31">
+        <f>IF(OR(B22="",A22="Oui",DX22&lt;&gt;3),0,IF(N(C22)&gt;0,C22,1)*(N(F22)+N(H22)))</f>
+        <v/>
+      </c>
+      <c r="DV22" s="31">
+        <f>IF(OR(B22="",N($DF$9)=0),0,IF(N(C22)&gt;0,C22,1)*(IF((COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,62+MAX(1,N($DF$9))),"VR"))&gt;0,N(G22),0)+IF((COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,62+MAX(1,N($DF$9))),"RC"))&gt;0,N(I22),0)))</f>
+        <v/>
+      </c>
+      <c r="DW22" s="31">
+        <f>IF(OR(B22="",N($DF$9)=0),0,IF(N(C22)&gt;0,C22,1)*(COUNTIF(INDEX($M22:$DA22,63):INDEX($M22:$DA22,62+MAX(1,N($DF$9))),"FOC"))*N(E22))</f>
+        <v/>
+      </c>
+      <c r="DX22" s="31">
+        <f>IF(B22="",0,IF(DD22&gt;0,1,IF(DK22&gt;0,2,IF(DR22&gt;0,3,0))))</f>
         <v/>
       </c>
     </row>
@@ -3108,15 +3322,15 @@
       <c r="H23" s="25" t="n"/>
       <c r="I23" s="25" t="n"/>
       <c r="J23" s="28">
-        <f>IF(B23="","",COUNTIF($M23:INDEX($M23:$DA23,MAX(1,N($J$9))),"S")+COUNTIF($M23:INDEX($M23:$DA23,MAX(1,N($J$9))),"MOB")+COUNTIF($M23:INDEX($M23:$DA23,MAX(1,N($J$9))),"DEMOB"))</f>
+        <f>IF(B23="","",DC23+DJ23+DQ23)</f>
         <v/>
       </c>
       <c r="K23" s="28">
-        <f>IF(B23="","",COUNTIF($M23:INDEX($M23:$DA23,MAX(1,N($J$9))),"O"))</f>
+        <f>IF(B23="","",DD23+DK23+DR23)</f>
         <v/>
       </c>
       <c r="L23" s="29">
-        <f>IF(B23="","",DC23+DG23+DK23+DD23+DH23+DL23+DE23+DI23+DM23)</f>
+        <f>IF(B23="","",DF23+DM23+DT23+DG23+DN23+DU23+DH23+DO23+DV23)</f>
         <v/>
       </c>
       <c r="M23" s="30" t="n"/>
@@ -3213,55 +3427,91 @@
       <c r="CZ23" s="30" t="n"/>
       <c r="DA23" s="30" t="n"/>
       <c r="DC23" s="31">
-        <f>IF(OR(B23="",NOT(N($J$9)&gt;0)),0,IF(N(C23)&gt;0,C23,1)*((COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,MIN(31,N($J$9))),"DEMOB"))*N(D23)+(COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,MIN(31,N($J$9))),"O"))*N(E23)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD23" s="31">
-        <f>IF(OR(B23="",A23="Oui",DO23&lt;&gt;1),0,IF(N(C23)&gt;0,C23,1)*(N(F23)+N(H23)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,0+MAX(1,N($DD$9))),"O"))</f>
         <v/>
       </c>
       <c r="DE23" s="31">
-        <f>IF(OR(B23="",NOT(N($J$9)&gt;0)),0,IF(N(C23)&gt;0,C23,1)*(IF((COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,MIN(31,N($J$9))),"VR"))&gt;0,N(G23),0)+IF((COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,MIN(31,N($J$9))),"RC"))&gt;0,N(I23),0)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DF23" s="31">
-        <f>IF(OR(B23="",NOT(N($J$9)&gt;0)),0,IF(N(C23)&gt;0,C23,1)*(COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,MIN(31,N($J$9))),"FOC"))*N(E23))</f>
+        <f>IF(B23="",0,IF(N(C23)&gt;0,C23,1)*(DC23*N(D23)+DD23*N(E23)))</f>
         <v/>
       </c>
       <c r="DG23" s="31">
-        <f>IF(OR(B23="",NOT(N($J$9)&gt;31)),0,IF(N(C23)&gt;0,C23,1)*((COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,MIN(62,N($J$9))),"DEMOB"))*N(D23)+(COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,MIN(62,N($J$9))),"O"))*N(E23)))</f>
+        <f>IF(OR(B23="",A23="Oui",DX23&lt;&gt;1),0,IF(N(C23)&gt;0,C23,1)*(N(F23)+N(H23)))</f>
         <v/>
       </c>
       <c r="DH23" s="31">
-        <f>IF(OR(B23="",A23="Oui",DO23&lt;&gt;2),0,IF(N(C23)&gt;0,C23,1)*(N(F23)+N(H23)))</f>
+        <f>IF(OR(B23="",N($DD$9)=0),0,IF(N(C23)&gt;0,C23,1)*(IF((COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,0+MAX(1,N($DD$9))),"VR"))&gt;0,N(G23),0)+IF((COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,0+MAX(1,N($DD$9))),"RC"))&gt;0,N(I23),0)))</f>
         <v/>
       </c>
       <c r="DI23" s="31">
-        <f>IF(OR(B23="",NOT(N($J$9)&gt;31)),0,IF(N(C23)&gt;0,C23,1)*(IF((COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,MIN(62,N($J$9))),"VR"))&gt;0,N(G23),0)+IF((COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,MIN(62,N($J$9))),"RC"))&gt;0,N(I23),0)))</f>
+        <f>IF(OR(B23="",N($DD$9)=0),0,IF(N(C23)&gt;0,C23,1)*(COUNTIF(INDEX($M23:$DA23,1):INDEX($M23:$DA23,0+MAX(1,N($DD$9))),"FOC"))*N(E23))</f>
         <v/>
       </c>
       <c r="DJ23" s="31">
-        <f>IF(OR(B23="",NOT(N($J$9)&gt;31)),0,IF(N(C23)&gt;0,C23,1)*(COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,MIN(62,N($J$9))),"FOC"))*N(E23))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DK23" s="31">
-        <f>IF(OR(B23="",NOT(N($J$9)&gt;62)),0,IF(N(C23)&gt;0,C23,1)*((COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,MIN(93,N($J$9))),"DEMOB"))*N(D23)+(COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,MIN(93,N($J$9))),"O"))*N(E23)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL23" s="31">
-        <f>IF(OR(B23="",A23="Oui",DO23&lt;&gt;3),0,IF(N(C23)&gt;0,C23,1)*(N(F23)+N(H23)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DM23" s="31">
-        <f>IF(OR(B23="",NOT(N($J$9)&gt;62)),0,IF(N(C23)&gt;0,C23,1)*(IF((COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,MIN(93,N($J$9))),"VR"))&gt;0,N(G23),0)+IF((COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,MIN(93,N($J$9))),"RC"))&gt;0,N(I23),0)))</f>
+        <f>IF(B23="",0,IF(N(C23)&gt;0,C23,1)*(DJ23*N(D23)+DK23*N(E23)))</f>
         <v/>
       </c>
       <c r="DN23" s="31">
-        <f>IF(OR(B23="",NOT(N($J$9)&gt;62)),0,IF(N(C23)&gt;0,C23,1)*(COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,MIN(93,N($J$9))),"FOC"))*N(E23))</f>
+        <f>IF(OR(B23="",A23="Oui",DX23&lt;&gt;2),0,IF(N(C23)&gt;0,C23,1)*(N(F23)+N(H23)))</f>
         <v/>
       </c>
       <c r="DO23" s="31">
-        <f>IF(B23="",0,IFERROR(INT((MATCH("O",$M23:INDEX($M23:$DA23,MAX(1,N($J$9))),0)-1)/31)+1,0))</f>
+        <f>IF(OR(B23="",N($DE$9)=0),0,IF(N(C23)&gt;0,C23,1)*(IF((COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,31+MAX(1,N($DE$9))),"VR"))&gt;0,N(G23),0)+IF((COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,31+MAX(1,N($DE$9))),"RC"))&gt;0,N(I23),0)))</f>
+        <v/>
+      </c>
+      <c r="DP23" s="31">
+        <f>IF(OR(B23="",N($DE$9)=0),0,IF(N(C23)&gt;0,C23,1)*(COUNTIF(INDEX($M23:$DA23,32):INDEX($M23:$DA23,31+MAX(1,N($DE$9))),"FOC"))*N(E23))</f>
+        <v/>
+      </c>
+      <c r="DQ23" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR23" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS23" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT23" s="31">
+        <f>IF(B23="",0,IF(N(C23)&gt;0,C23,1)*(DQ23*N(D23)+DR23*N(E23)))</f>
+        <v/>
+      </c>
+      <c r="DU23" s="31">
+        <f>IF(OR(B23="",A23="Oui",DX23&lt;&gt;3),0,IF(N(C23)&gt;0,C23,1)*(N(F23)+N(H23)))</f>
+        <v/>
+      </c>
+      <c r="DV23" s="31">
+        <f>IF(OR(B23="",N($DF$9)=0),0,IF(N(C23)&gt;0,C23,1)*(IF((COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,62+MAX(1,N($DF$9))),"VR"))&gt;0,N(G23),0)+IF((COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,62+MAX(1,N($DF$9))),"RC"))&gt;0,N(I23),0)))</f>
+        <v/>
+      </c>
+      <c r="DW23" s="31">
+        <f>IF(OR(B23="",N($DF$9)=0),0,IF(N(C23)&gt;0,C23,1)*(COUNTIF(INDEX($M23:$DA23,63):INDEX($M23:$DA23,62+MAX(1,N($DF$9))),"FOC"))*N(E23))</f>
+        <v/>
+      </c>
+      <c r="DX23" s="31">
+        <f>IF(B23="",0,IF(DD23&gt;0,1,IF(DK23&gt;0,2,IF(DR23&gt;0,3,0))))</f>
         <v/>
       </c>
     </row>
@@ -3276,15 +3526,15 @@
       <c r="H24" s="25" t="n"/>
       <c r="I24" s="25" t="n"/>
       <c r="J24" s="28">
-        <f>IF(B24="","",COUNTIF($M24:INDEX($M24:$DA24,MAX(1,N($J$9))),"S")+COUNTIF($M24:INDEX($M24:$DA24,MAX(1,N($J$9))),"MOB")+COUNTIF($M24:INDEX($M24:$DA24,MAX(1,N($J$9))),"DEMOB"))</f>
+        <f>IF(B24="","",DC24+DJ24+DQ24)</f>
         <v/>
       </c>
       <c r="K24" s="28">
-        <f>IF(B24="","",COUNTIF($M24:INDEX($M24:$DA24,MAX(1,N($J$9))),"O"))</f>
+        <f>IF(B24="","",DD24+DK24+DR24)</f>
         <v/>
       </c>
       <c r="L24" s="29">
-        <f>IF(B24="","",DC24+DG24+DK24+DD24+DH24+DL24+DE24+DI24+DM24)</f>
+        <f>IF(B24="","",DF24+DM24+DT24+DG24+DN24+DU24+DH24+DO24+DV24)</f>
         <v/>
       </c>
       <c r="M24" s="30" t="n"/>
@@ -3381,55 +3631,91 @@
       <c r="CZ24" s="30" t="n"/>
       <c r="DA24" s="30" t="n"/>
       <c r="DC24" s="31">
-        <f>IF(OR(B24="",NOT(N($J$9)&gt;0)),0,IF(N(C24)&gt;0,C24,1)*((COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,MIN(31,N($J$9))),"DEMOB"))*N(D24)+(COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,MIN(31,N($J$9))),"O"))*N(E24)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD24" s="31">
-        <f>IF(OR(B24="",A24="Oui",DO24&lt;&gt;1),0,IF(N(C24)&gt;0,C24,1)*(N(F24)+N(H24)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,0+MAX(1,N($DD$9))),"O"))</f>
         <v/>
       </c>
       <c r="DE24" s="31">
-        <f>IF(OR(B24="",NOT(N($J$9)&gt;0)),0,IF(N(C24)&gt;0,C24,1)*(IF((COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,MIN(31,N($J$9))),"VR"))&gt;0,N(G24),0)+IF((COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,MIN(31,N($J$9))),"RC"))&gt;0,N(I24),0)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DF24" s="31">
-        <f>IF(OR(B24="",NOT(N($J$9)&gt;0)),0,IF(N(C24)&gt;0,C24,1)*(COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,MIN(31,N($J$9))),"FOC"))*N(E24))</f>
+        <f>IF(B24="",0,IF(N(C24)&gt;0,C24,1)*(DC24*N(D24)+DD24*N(E24)))</f>
         <v/>
       </c>
       <c r="DG24" s="31">
-        <f>IF(OR(B24="",NOT(N($J$9)&gt;31)),0,IF(N(C24)&gt;0,C24,1)*((COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,MIN(62,N($J$9))),"DEMOB"))*N(D24)+(COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,MIN(62,N($J$9))),"O"))*N(E24)))</f>
+        <f>IF(OR(B24="",A24="Oui",DX24&lt;&gt;1),0,IF(N(C24)&gt;0,C24,1)*(N(F24)+N(H24)))</f>
         <v/>
       </c>
       <c r="DH24" s="31">
-        <f>IF(OR(B24="",A24="Oui",DO24&lt;&gt;2),0,IF(N(C24)&gt;0,C24,1)*(N(F24)+N(H24)))</f>
+        <f>IF(OR(B24="",N($DD$9)=0),0,IF(N(C24)&gt;0,C24,1)*(IF((COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,0+MAX(1,N($DD$9))),"VR"))&gt;0,N(G24),0)+IF((COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,0+MAX(1,N($DD$9))),"RC"))&gt;0,N(I24),0)))</f>
         <v/>
       </c>
       <c r="DI24" s="31">
-        <f>IF(OR(B24="",NOT(N($J$9)&gt;31)),0,IF(N(C24)&gt;0,C24,1)*(IF((COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,MIN(62,N($J$9))),"VR"))&gt;0,N(G24),0)+IF((COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,MIN(62,N($J$9))),"RC"))&gt;0,N(I24),0)))</f>
+        <f>IF(OR(B24="",N($DD$9)=0),0,IF(N(C24)&gt;0,C24,1)*(COUNTIF(INDEX($M24:$DA24,1):INDEX($M24:$DA24,0+MAX(1,N($DD$9))),"FOC"))*N(E24))</f>
         <v/>
       </c>
       <c r="DJ24" s="31">
-        <f>IF(OR(B24="",NOT(N($J$9)&gt;31)),0,IF(N(C24)&gt;0,C24,1)*(COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,MIN(62,N($J$9))),"FOC"))*N(E24))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DK24" s="31">
-        <f>IF(OR(B24="",NOT(N($J$9)&gt;62)),0,IF(N(C24)&gt;0,C24,1)*((COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,MIN(93,N($J$9))),"DEMOB"))*N(D24)+(COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,MIN(93,N($J$9))),"O"))*N(E24)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL24" s="31">
-        <f>IF(OR(B24="",A24="Oui",DO24&lt;&gt;3),0,IF(N(C24)&gt;0,C24,1)*(N(F24)+N(H24)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DM24" s="31">
-        <f>IF(OR(B24="",NOT(N($J$9)&gt;62)),0,IF(N(C24)&gt;0,C24,1)*(IF((COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,MIN(93,N($J$9))),"VR"))&gt;0,N(G24),0)+IF((COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,MIN(93,N($J$9))),"RC"))&gt;0,N(I24),0)))</f>
+        <f>IF(B24="",0,IF(N(C24)&gt;0,C24,1)*(DJ24*N(D24)+DK24*N(E24)))</f>
         <v/>
       </c>
       <c r="DN24" s="31">
-        <f>IF(OR(B24="",NOT(N($J$9)&gt;62)),0,IF(N(C24)&gt;0,C24,1)*(COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,MIN(93,N($J$9))),"FOC"))*N(E24))</f>
+        <f>IF(OR(B24="",A24="Oui",DX24&lt;&gt;2),0,IF(N(C24)&gt;0,C24,1)*(N(F24)+N(H24)))</f>
         <v/>
       </c>
       <c r="DO24" s="31">
-        <f>IF(B24="",0,IFERROR(INT((MATCH("O",$M24:INDEX($M24:$DA24,MAX(1,N($J$9))),0)-1)/31)+1,0))</f>
+        <f>IF(OR(B24="",N($DE$9)=0),0,IF(N(C24)&gt;0,C24,1)*(IF((COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,31+MAX(1,N($DE$9))),"VR"))&gt;0,N(G24),0)+IF((COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,31+MAX(1,N($DE$9))),"RC"))&gt;0,N(I24),0)))</f>
+        <v/>
+      </c>
+      <c r="DP24" s="31">
+        <f>IF(OR(B24="",N($DE$9)=0),0,IF(N(C24)&gt;0,C24,1)*(COUNTIF(INDEX($M24:$DA24,32):INDEX($M24:$DA24,31+MAX(1,N($DE$9))),"FOC"))*N(E24))</f>
+        <v/>
+      </c>
+      <c r="DQ24" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR24" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS24" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT24" s="31">
+        <f>IF(B24="",0,IF(N(C24)&gt;0,C24,1)*(DQ24*N(D24)+DR24*N(E24)))</f>
+        <v/>
+      </c>
+      <c r="DU24" s="31">
+        <f>IF(OR(B24="",A24="Oui",DX24&lt;&gt;3),0,IF(N(C24)&gt;0,C24,1)*(N(F24)+N(H24)))</f>
+        <v/>
+      </c>
+      <c r="DV24" s="31">
+        <f>IF(OR(B24="",N($DF$9)=0),0,IF(N(C24)&gt;0,C24,1)*(IF((COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,62+MAX(1,N($DF$9))),"VR"))&gt;0,N(G24),0)+IF((COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,62+MAX(1,N($DF$9))),"RC"))&gt;0,N(I24),0)))</f>
+        <v/>
+      </c>
+      <c r="DW24" s="31">
+        <f>IF(OR(B24="",N($DF$9)=0),0,IF(N(C24)&gt;0,C24,1)*(COUNTIF(INDEX($M24:$DA24,63):INDEX($M24:$DA24,62+MAX(1,N($DF$9))),"FOC"))*N(E24))</f>
+        <v/>
+      </c>
+      <c r="DX24" s="31">
+        <f>IF(B24="",0,IF(DD24&gt;0,1,IF(DK24&gt;0,2,IF(DR24&gt;0,3,0))))</f>
         <v/>
       </c>
     </row>
@@ -3444,15 +3730,15 @@
       <c r="H25" s="25" t="n"/>
       <c r="I25" s="25" t="n"/>
       <c r="J25" s="28">
-        <f>IF(B25="","",COUNTIF($M25:INDEX($M25:$DA25,MAX(1,N($J$9))),"S")+COUNTIF($M25:INDEX($M25:$DA25,MAX(1,N($J$9))),"MOB")+COUNTIF($M25:INDEX($M25:$DA25,MAX(1,N($J$9))),"DEMOB"))</f>
+        <f>IF(B25="","",DC25+DJ25+DQ25)</f>
         <v/>
       </c>
       <c r="K25" s="28">
-        <f>IF(B25="","",COUNTIF($M25:INDEX($M25:$DA25,MAX(1,N($J$9))),"O"))</f>
+        <f>IF(B25="","",DD25+DK25+DR25)</f>
         <v/>
       </c>
       <c r="L25" s="29">
-        <f>IF(B25="","",DC25+DG25+DK25+DD25+DH25+DL25+DE25+DI25+DM25)</f>
+        <f>IF(B25="","",DF25+DM25+DT25+DG25+DN25+DU25+DH25+DO25+DV25)</f>
         <v/>
       </c>
       <c r="M25" s="30" t="n"/>
@@ -3549,55 +3835,91 @@
       <c r="CZ25" s="30" t="n"/>
       <c r="DA25" s="30" t="n"/>
       <c r="DC25" s="31">
-        <f>IF(OR(B25="",NOT(N($J$9)&gt;0)),0,IF(N(C25)&gt;0,C25,1)*((COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,MIN(31,N($J$9))),"DEMOB"))*N(D25)+(COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,MIN(31,N($J$9))),"O"))*N(E25)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD25" s="31">
-        <f>IF(OR(B25="",A25="Oui",DO25&lt;&gt;1),0,IF(N(C25)&gt;0,C25,1)*(N(F25)+N(H25)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,0+MAX(1,N($DD$9))),"O"))</f>
         <v/>
       </c>
       <c r="DE25" s="31">
-        <f>IF(OR(B25="",NOT(N($J$9)&gt;0)),0,IF(N(C25)&gt;0,C25,1)*(IF((COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,MIN(31,N($J$9))),"VR"))&gt;0,N(G25),0)+IF((COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,MIN(31,N($J$9))),"RC"))&gt;0,N(I25),0)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DF25" s="31">
-        <f>IF(OR(B25="",NOT(N($J$9)&gt;0)),0,IF(N(C25)&gt;0,C25,1)*(COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,MIN(31,N($J$9))),"FOC"))*N(E25))</f>
+        <f>IF(B25="",0,IF(N(C25)&gt;0,C25,1)*(DC25*N(D25)+DD25*N(E25)))</f>
         <v/>
       </c>
       <c r="DG25" s="31">
-        <f>IF(OR(B25="",NOT(N($J$9)&gt;31)),0,IF(N(C25)&gt;0,C25,1)*((COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,MIN(62,N($J$9))),"DEMOB"))*N(D25)+(COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,MIN(62,N($J$9))),"O"))*N(E25)))</f>
+        <f>IF(OR(B25="",A25="Oui",DX25&lt;&gt;1),0,IF(N(C25)&gt;0,C25,1)*(N(F25)+N(H25)))</f>
         <v/>
       </c>
       <c r="DH25" s="31">
-        <f>IF(OR(B25="",A25="Oui",DO25&lt;&gt;2),0,IF(N(C25)&gt;0,C25,1)*(N(F25)+N(H25)))</f>
+        <f>IF(OR(B25="",N($DD$9)=0),0,IF(N(C25)&gt;0,C25,1)*(IF((COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,0+MAX(1,N($DD$9))),"VR"))&gt;0,N(G25),0)+IF((COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,0+MAX(1,N($DD$9))),"RC"))&gt;0,N(I25),0)))</f>
         <v/>
       </c>
       <c r="DI25" s="31">
-        <f>IF(OR(B25="",NOT(N($J$9)&gt;31)),0,IF(N(C25)&gt;0,C25,1)*(IF((COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,MIN(62,N($J$9))),"VR"))&gt;0,N(G25),0)+IF((COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,MIN(62,N($J$9))),"RC"))&gt;0,N(I25),0)))</f>
+        <f>IF(OR(B25="",N($DD$9)=0),0,IF(N(C25)&gt;0,C25,1)*(COUNTIF(INDEX($M25:$DA25,1):INDEX($M25:$DA25,0+MAX(1,N($DD$9))),"FOC"))*N(E25))</f>
         <v/>
       </c>
       <c r="DJ25" s="31">
-        <f>IF(OR(B25="",NOT(N($J$9)&gt;31)),0,IF(N(C25)&gt;0,C25,1)*(COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,MIN(62,N($J$9))),"FOC"))*N(E25))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DK25" s="31">
-        <f>IF(OR(B25="",NOT(N($J$9)&gt;62)),0,IF(N(C25)&gt;0,C25,1)*((COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,MIN(93,N($J$9))),"DEMOB"))*N(D25)+(COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,MIN(93,N($J$9))),"O"))*N(E25)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL25" s="31">
-        <f>IF(OR(B25="",A25="Oui",DO25&lt;&gt;3),0,IF(N(C25)&gt;0,C25,1)*(N(F25)+N(H25)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DM25" s="31">
-        <f>IF(OR(B25="",NOT(N($J$9)&gt;62)),0,IF(N(C25)&gt;0,C25,1)*(IF((COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,MIN(93,N($J$9))),"VR"))&gt;0,N(G25),0)+IF((COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,MIN(93,N($J$9))),"RC"))&gt;0,N(I25),0)))</f>
+        <f>IF(B25="",0,IF(N(C25)&gt;0,C25,1)*(DJ25*N(D25)+DK25*N(E25)))</f>
         <v/>
       </c>
       <c r="DN25" s="31">
-        <f>IF(OR(B25="",NOT(N($J$9)&gt;62)),0,IF(N(C25)&gt;0,C25,1)*(COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,MIN(93,N($J$9))),"FOC"))*N(E25))</f>
+        <f>IF(OR(B25="",A25="Oui",DX25&lt;&gt;2),0,IF(N(C25)&gt;0,C25,1)*(N(F25)+N(H25)))</f>
         <v/>
       </c>
       <c r="DO25" s="31">
-        <f>IF(B25="",0,IFERROR(INT((MATCH("O",$M25:INDEX($M25:$DA25,MAX(1,N($J$9))),0)-1)/31)+1,0))</f>
+        <f>IF(OR(B25="",N($DE$9)=0),0,IF(N(C25)&gt;0,C25,1)*(IF((COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,31+MAX(1,N($DE$9))),"VR"))&gt;0,N(G25),0)+IF((COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,31+MAX(1,N($DE$9))),"RC"))&gt;0,N(I25),0)))</f>
+        <v/>
+      </c>
+      <c r="DP25" s="31">
+        <f>IF(OR(B25="",N($DE$9)=0),0,IF(N(C25)&gt;0,C25,1)*(COUNTIF(INDEX($M25:$DA25,32):INDEX($M25:$DA25,31+MAX(1,N($DE$9))),"FOC"))*N(E25))</f>
+        <v/>
+      </c>
+      <c r="DQ25" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR25" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS25" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT25" s="31">
+        <f>IF(B25="",0,IF(N(C25)&gt;0,C25,1)*(DQ25*N(D25)+DR25*N(E25)))</f>
+        <v/>
+      </c>
+      <c r="DU25" s="31">
+        <f>IF(OR(B25="",A25="Oui",DX25&lt;&gt;3),0,IF(N(C25)&gt;0,C25,1)*(N(F25)+N(H25)))</f>
+        <v/>
+      </c>
+      <c r="DV25" s="31">
+        <f>IF(OR(B25="",N($DF$9)=0),0,IF(N(C25)&gt;0,C25,1)*(IF((COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,62+MAX(1,N($DF$9))),"VR"))&gt;0,N(G25),0)+IF((COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,62+MAX(1,N($DF$9))),"RC"))&gt;0,N(I25),0)))</f>
+        <v/>
+      </c>
+      <c r="DW25" s="31">
+        <f>IF(OR(B25="",N($DF$9)=0),0,IF(N(C25)&gt;0,C25,1)*(COUNTIF(INDEX($M25:$DA25,63):INDEX($M25:$DA25,62+MAX(1,N($DF$9))),"FOC"))*N(E25))</f>
+        <v/>
+      </c>
+      <c r="DX25" s="31">
+        <f>IF(B25="",0,IF(DD25&gt;0,1,IF(DK25&gt;0,2,IF(DR25&gt;0,3,0))))</f>
         <v/>
       </c>
     </row>
@@ -3612,15 +3934,15 @@
       <c r="H26" s="25" t="n"/>
       <c r="I26" s="25" t="n"/>
       <c r="J26" s="28">
-        <f>IF(B26="","",COUNTIF($M26:INDEX($M26:$DA26,MAX(1,N($J$9))),"S")+COUNTIF($M26:INDEX($M26:$DA26,MAX(1,N($J$9))),"MOB")+COUNTIF($M26:INDEX($M26:$DA26,MAX(1,N($J$9))),"DEMOB"))</f>
+        <f>IF(B26="","",DC26+DJ26+DQ26)</f>
         <v/>
       </c>
       <c r="K26" s="28">
-        <f>IF(B26="","",COUNTIF($M26:INDEX($M26:$DA26,MAX(1,N($J$9))),"O"))</f>
+        <f>IF(B26="","",DD26+DK26+DR26)</f>
         <v/>
       </c>
       <c r="L26" s="29">
-        <f>IF(B26="","",DC26+DG26+DK26+DD26+DH26+DL26+DE26+DI26+DM26)</f>
+        <f>IF(B26="","",DF26+DM26+DT26+DG26+DN26+DU26+DH26+DO26+DV26)</f>
         <v/>
       </c>
       <c r="M26" s="30" t="n"/>
@@ -3717,55 +4039,91 @@
       <c r="CZ26" s="30" t="n"/>
       <c r="DA26" s="30" t="n"/>
       <c r="DC26" s="31">
-        <f>IF(OR(B26="",NOT(N($J$9)&gt;0)),0,IF(N(C26)&gt;0,C26,1)*((COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,MIN(31,N($J$9))),"DEMOB"))*N(D26)+(COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,MIN(31,N($J$9))),"O"))*N(E26)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD26" s="31">
-        <f>IF(OR(B26="",A26="Oui",DO26&lt;&gt;1),0,IF(N(C26)&gt;0,C26,1)*(N(F26)+N(H26)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,0+MAX(1,N($DD$9))),"O"))</f>
         <v/>
       </c>
       <c r="DE26" s="31">
-        <f>IF(OR(B26="",NOT(N($J$9)&gt;0)),0,IF(N(C26)&gt;0,C26,1)*(IF((COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,MIN(31,N($J$9))),"VR"))&gt;0,N(G26),0)+IF((COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,MIN(31,N($J$9))),"RC"))&gt;0,N(I26),0)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DF26" s="31">
-        <f>IF(OR(B26="",NOT(N($J$9)&gt;0)),0,IF(N(C26)&gt;0,C26,1)*(COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,MIN(31,N($J$9))),"FOC"))*N(E26))</f>
+        <f>IF(B26="",0,IF(N(C26)&gt;0,C26,1)*(DC26*N(D26)+DD26*N(E26)))</f>
         <v/>
       </c>
       <c r="DG26" s="31">
-        <f>IF(OR(B26="",NOT(N($J$9)&gt;31)),0,IF(N(C26)&gt;0,C26,1)*((COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,MIN(62,N($J$9))),"DEMOB"))*N(D26)+(COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,MIN(62,N($J$9))),"O"))*N(E26)))</f>
+        <f>IF(OR(B26="",A26="Oui",DX26&lt;&gt;1),0,IF(N(C26)&gt;0,C26,1)*(N(F26)+N(H26)))</f>
         <v/>
       </c>
       <c r="DH26" s="31">
-        <f>IF(OR(B26="",A26="Oui",DO26&lt;&gt;2),0,IF(N(C26)&gt;0,C26,1)*(N(F26)+N(H26)))</f>
+        <f>IF(OR(B26="",N($DD$9)=0),0,IF(N(C26)&gt;0,C26,1)*(IF((COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,0+MAX(1,N($DD$9))),"VR"))&gt;0,N(G26),0)+IF((COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,0+MAX(1,N($DD$9))),"RC"))&gt;0,N(I26),0)))</f>
         <v/>
       </c>
       <c r="DI26" s="31">
-        <f>IF(OR(B26="",NOT(N($J$9)&gt;31)),0,IF(N(C26)&gt;0,C26,1)*(IF((COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,MIN(62,N($J$9))),"VR"))&gt;0,N(G26),0)+IF((COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,MIN(62,N($J$9))),"RC"))&gt;0,N(I26),0)))</f>
+        <f>IF(OR(B26="",N($DD$9)=0),0,IF(N(C26)&gt;0,C26,1)*(COUNTIF(INDEX($M26:$DA26,1):INDEX($M26:$DA26,0+MAX(1,N($DD$9))),"FOC"))*N(E26))</f>
         <v/>
       </c>
       <c r="DJ26" s="31">
-        <f>IF(OR(B26="",NOT(N($J$9)&gt;31)),0,IF(N(C26)&gt;0,C26,1)*(COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,MIN(62,N($J$9))),"FOC"))*N(E26))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DK26" s="31">
-        <f>IF(OR(B26="",NOT(N($J$9)&gt;62)),0,IF(N(C26)&gt;0,C26,1)*((COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,MIN(93,N($J$9))),"DEMOB"))*N(D26)+(COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,MIN(93,N($J$9))),"O"))*N(E26)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL26" s="31">
-        <f>IF(OR(B26="",A26="Oui",DO26&lt;&gt;3),0,IF(N(C26)&gt;0,C26,1)*(N(F26)+N(H26)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DM26" s="31">
-        <f>IF(OR(B26="",NOT(N($J$9)&gt;62)),0,IF(N(C26)&gt;0,C26,1)*(IF((COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,MIN(93,N($J$9))),"VR"))&gt;0,N(G26),0)+IF((COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,MIN(93,N($J$9))),"RC"))&gt;0,N(I26),0)))</f>
+        <f>IF(B26="",0,IF(N(C26)&gt;0,C26,1)*(DJ26*N(D26)+DK26*N(E26)))</f>
         <v/>
       </c>
       <c r="DN26" s="31">
-        <f>IF(OR(B26="",NOT(N($J$9)&gt;62)),0,IF(N(C26)&gt;0,C26,1)*(COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,MIN(93,N($J$9))),"FOC"))*N(E26))</f>
+        <f>IF(OR(B26="",A26="Oui",DX26&lt;&gt;2),0,IF(N(C26)&gt;0,C26,1)*(N(F26)+N(H26)))</f>
         <v/>
       </c>
       <c r="DO26" s="31">
-        <f>IF(B26="",0,IFERROR(INT((MATCH("O",$M26:INDEX($M26:$DA26,MAX(1,N($J$9))),0)-1)/31)+1,0))</f>
+        <f>IF(OR(B26="",N($DE$9)=0),0,IF(N(C26)&gt;0,C26,1)*(IF((COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,31+MAX(1,N($DE$9))),"VR"))&gt;0,N(G26),0)+IF((COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,31+MAX(1,N($DE$9))),"RC"))&gt;0,N(I26),0)))</f>
+        <v/>
+      </c>
+      <c r="DP26" s="31">
+        <f>IF(OR(B26="",N($DE$9)=0),0,IF(N(C26)&gt;0,C26,1)*(COUNTIF(INDEX($M26:$DA26,32):INDEX($M26:$DA26,31+MAX(1,N($DE$9))),"FOC"))*N(E26))</f>
+        <v/>
+      </c>
+      <c r="DQ26" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR26" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS26" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT26" s="31">
+        <f>IF(B26="",0,IF(N(C26)&gt;0,C26,1)*(DQ26*N(D26)+DR26*N(E26)))</f>
+        <v/>
+      </c>
+      <c r="DU26" s="31">
+        <f>IF(OR(B26="",A26="Oui",DX26&lt;&gt;3),0,IF(N(C26)&gt;0,C26,1)*(N(F26)+N(H26)))</f>
+        <v/>
+      </c>
+      <c r="DV26" s="31">
+        <f>IF(OR(B26="",N($DF$9)=0),0,IF(N(C26)&gt;0,C26,1)*(IF((COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,62+MAX(1,N($DF$9))),"VR"))&gt;0,N(G26),0)+IF((COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,62+MAX(1,N($DF$9))),"RC"))&gt;0,N(I26),0)))</f>
+        <v/>
+      </c>
+      <c r="DW26" s="31">
+        <f>IF(OR(B26="",N($DF$9)=0),0,IF(N(C26)&gt;0,C26,1)*(COUNTIF(INDEX($M26:$DA26,63):INDEX($M26:$DA26,62+MAX(1,N($DF$9))),"FOC"))*N(E26))</f>
+        <v/>
+      </c>
+      <c r="DX26" s="31">
+        <f>IF(B26="",0,IF(DD26&gt;0,1,IF(DK26&gt;0,2,IF(DR26&gt;0,3,0))))</f>
         <v/>
       </c>
     </row>
@@ -3780,15 +4138,15 @@
       <c r="H27" s="25" t="n"/>
       <c r="I27" s="25" t="n"/>
       <c r="J27" s="28">
-        <f>IF(B27="","",COUNTIF($M27:INDEX($M27:$DA27,MAX(1,N($J$9))),"S")+COUNTIF($M27:INDEX($M27:$DA27,MAX(1,N($J$9))),"MOB")+COUNTIF($M27:INDEX($M27:$DA27,MAX(1,N($J$9))),"DEMOB"))</f>
+        <f>IF(B27="","",DC27+DJ27+DQ27)</f>
         <v/>
       </c>
       <c r="K27" s="28">
-        <f>IF(B27="","",COUNTIF($M27:INDEX($M27:$DA27,MAX(1,N($J$9))),"O"))</f>
+        <f>IF(B27="","",DD27+DK27+DR27)</f>
         <v/>
       </c>
       <c r="L27" s="29">
-        <f>IF(B27="","",DC27+DG27+DK27+DD27+DH27+DL27+DE27+DI27+DM27)</f>
+        <f>IF(B27="","",DF27+DM27+DT27+DG27+DN27+DU27+DH27+DO27+DV27)</f>
         <v/>
       </c>
       <c r="M27" s="30" t="n"/>
@@ -3885,55 +4243,91 @@
       <c r="CZ27" s="30" t="n"/>
       <c r="DA27" s="30" t="n"/>
       <c r="DC27" s="31">
-        <f>IF(OR(B27="",NOT(N($J$9)&gt;0)),0,IF(N(C27)&gt;0,C27,1)*((COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,MIN(31,N($J$9))),"DEMOB"))*N(D27)+(COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,MIN(31,N($J$9))),"O"))*N(E27)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD27" s="31">
-        <f>IF(OR(B27="",A27="Oui",DO27&lt;&gt;1),0,IF(N(C27)&gt;0,C27,1)*(N(F27)+N(H27)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,0+MAX(1,N($DD$9))),"O"))</f>
         <v/>
       </c>
       <c r="DE27" s="31">
-        <f>IF(OR(B27="",NOT(N($J$9)&gt;0)),0,IF(N(C27)&gt;0,C27,1)*(IF((COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,MIN(31,N($J$9))),"VR"))&gt;0,N(G27),0)+IF((COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,MIN(31,N($J$9))),"RC"))&gt;0,N(I27),0)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DF27" s="31">
-        <f>IF(OR(B27="",NOT(N($J$9)&gt;0)),0,IF(N(C27)&gt;0,C27,1)*(COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,MIN(31,N($J$9))),"FOC"))*N(E27))</f>
+        <f>IF(B27="",0,IF(N(C27)&gt;0,C27,1)*(DC27*N(D27)+DD27*N(E27)))</f>
         <v/>
       </c>
       <c r="DG27" s="31">
-        <f>IF(OR(B27="",NOT(N($J$9)&gt;31)),0,IF(N(C27)&gt;0,C27,1)*((COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,MIN(62,N($J$9))),"DEMOB"))*N(D27)+(COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,MIN(62,N($J$9))),"O"))*N(E27)))</f>
+        <f>IF(OR(B27="",A27="Oui",DX27&lt;&gt;1),0,IF(N(C27)&gt;0,C27,1)*(N(F27)+N(H27)))</f>
         <v/>
       </c>
       <c r="DH27" s="31">
-        <f>IF(OR(B27="",A27="Oui",DO27&lt;&gt;2),0,IF(N(C27)&gt;0,C27,1)*(N(F27)+N(H27)))</f>
+        <f>IF(OR(B27="",N($DD$9)=0),0,IF(N(C27)&gt;0,C27,1)*(IF((COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,0+MAX(1,N($DD$9))),"VR"))&gt;0,N(G27),0)+IF((COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,0+MAX(1,N($DD$9))),"RC"))&gt;0,N(I27),0)))</f>
         <v/>
       </c>
       <c r="DI27" s="31">
-        <f>IF(OR(B27="",NOT(N($J$9)&gt;31)),0,IF(N(C27)&gt;0,C27,1)*(IF((COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,MIN(62,N($J$9))),"VR"))&gt;0,N(G27),0)+IF((COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,MIN(62,N($J$9))),"RC"))&gt;0,N(I27),0)))</f>
+        <f>IF(OR(B27="",N($DD$9)=0),0,IF(N(C27)&gt;0,C27,1)*(COUNTIF(INDEX($M27:$DA27,1):INDEX($M27:$DA27,0+MAX(1,N($DD$9))),"FOC"))*N(E27))</f>
         <v/>
       </c>
       <c r="DJ27" s="31">
-        <f>IF(OR(B27="",NOT(N($J$9)&gt;31)),0,IF(N(C27)&gt;0,C27,1)*(COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,MIN(62,N($J$9))),"FOC"))*N(E27))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DK27" s="31">
-        <f>IF(OR(B27="",NOT(N($J$9)&gt;62)),0,IF(N(C27)&gt;0,C27,1)*((COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,MIN(93,N($J$9))),"DEMOB"))*N(D27)+(COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,MIN(93,N($J$9))),"O"))*N(E27)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL27" s="31">
-        <f>IF(OR(B27="",A27="Oui",DO27&lt;&gt;3),0,IF(N(C27)&gt;0,C27,1)*(N(F27)+N(H27)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DM27" s="31">
-        <f>IF(OR(B27="",NOT(N($J$9)&gt;62)),0,IF(N(C27)&gt;0,C27,1)*(IF((COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,MIN(93,N($J$9))),"VR"))&gt;0,N(G27),0)+IF((COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,MIN(93,N($J$9))),"RC"))&gt;0,N(I27),0)))</f>
+        <f>IF(B27="",0,IF(N(C27)&gt;0,C27,1)*(DJ27*N(D27)+DK27*N(E27)))</f>
         <v/>
       </c>
       <c r="DN27" s="31">
-        <f>IF(OR(B27="",NOT(N($J$9)&gt;62)),0,IF(N(C27)&gt;0,C27,1)*(COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,MIN(93,N($J$9))),"FOC"))*N(E27))</f>
+        <f>IF(OR(B27="",A27="Oui",DX27&lt;&gt;2),0,IF(N(C27)&gt;0,C27,1)*(N(F27)+N(H27)))</f>
         <v/>
       </c>
       <c r="DO27" s="31">
-        <f>IF(B27="",0,IFERROR(INT((MATCH("O",$M27:INDEX($M27:$DA27,MAX(1,N($J$9))),0)-1)/31)+1,0))</f>
+        <f>IF(OR(B27="",N($DE$9)=0),0,IF(N(C27)&gt;0,C27,1)*(IF((COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,31+MAX(1,N($DE$9))),"VR"))&gt;0,N(G27),0)+IF((COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,31+MAX(1,N($DE$9))),"RC"))&gt;0,N(I27),0)))</f>
+        <v/>
+      </c>
+      <c r="DP27" s="31">
+        <f>IF(OR(B27="",N($DE$9)=0),0,IF(N(C27)&gt;0,C27,1)*(COUNTIF(INDEX($M27:$DA27,32):INDEX($M27:$DA27,31+MAX(1,N($DE$9))),"FOC"))*N(E27))</f>
+        <v/>
+      </c>
+      <c r="DQ27" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR27" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS27" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT27" s="31">
+        <f>IF(B27="",0,IF(N(C27)&gt;0,C27,1)*(DQ27*N(D27)+DR27*N(E27)))</f>
+        <v/>
+      </c>
+      <c r="DU27" s="31">
+        <f>IF(OR(B27="",A27="Oui",DX27&lt;&gt;3),0,IF(N(C27)&gt;0,C27,1)*(N(F27)+N(H27)))</f>
+        <v/>
+      </c>
+      <c r="DV27" s="31">
+        <f>IF(OR(B27="",N($DF$9)=0),0,IF(N(C27)&gt;0,C27,1)*(IF((COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,62+MAX(1,N($DF$9))),"VR"))&gt;0,N(G27),0)+IF((COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,62+MAX(1,N($DF$9))),"RC"))&gt;0,N(I27),0)))</f>
+        <v/>
+      </c>
+      <c r="DW27" s="31">
+        <f>IF(OR(B27="",N($DF$9)=0),0,IF(N(C27)&gt;0,C27,1)*(COUNTIF(INDEX($M27:$DA27,63):INDEX($M27:$DA27,62+MAX(1,N($DF$9))),"FOC"))*N(E27))</f>
+        <v/>
+      </c>
+      <c r="DX27" s="31">
+        <f>IF(B27="",0,IF(DD27&gt;0,1,IF(DK27&gt;0,2,IF(DR27&gt;0,3,0))))</f>
         <v/>
       </c>
     </row>
@@ -3948,15 +4342,15 @@
       <c r="H28" s="25" t="n"/>
       <c r="I28" s="25" t="n"/>
       <c r="J28" s="28">
-        <f>IF(B28="","",COUNTIF($M28:INDEX($M28:$DA28,MAX(1,N($J$9))),"S")+COUNTIF($M28:INDEX($M28:$DA28,MAX(1,N($J$9))),"MOB")+COUNTIF($M28:INDEX($M28:$DA28,MAX(1,N($J$9))),"DEMOB"))</f>
+        <f>IF(B28="","",DC28+DJ28+DQ28)</f>
         <v/>
       </c>
       <c r="K28" s="28">
-        <f>IF(B28="","",COUNTIF($M28:INDEX($M28:$DA28,MAX(1,N($J$9))),"O"))</f>
+        <f>IF(B28="","",DD28+DK28+DR28)</f>
         <v/>
       </c>
       <c r="L28" s="29">
-        <f>IF(B28="","",DC28+DG28+DK28+DD28+DH28+DL28+DE28+DI28+DM28)</f>
+        <f>IF(B28="","",DF28+DM28+DT28+DG28+DN28+DU28+DH28+DO28+DV28)</f>
         <v/>
       </c>
       <c r="M28" s="30" t="n"/>
@@ -4053,55 +4447,91 @@
       <c r="CZ28" s="30" t="n"/>
       <c r="DA28" s="30" t="n"/>
       <c r="DC28" s="31">
-        <f>IF(OR(B28="",NOT(N($J$9)&gt;0)),0,IF(N(C28)&gt;0,C28,1)*((COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,MIN(31,N($J$9))),"DEMOB"))*N(D28)+(COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,MIN(31,N($J$9))),"O"))*N(E28)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD28" s="31">
-        <f>IF(OR(B28="",A28="Oui",DO28&lt;&gt;1),0,IF(N(C28)&gt;0,C28,1)*(N(F28)+N(H28)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,0+MAX(1,N($DD$9))),"O"))</f>
         <v/>
       </c>
       <c r="DE28" s="31">
-        <f>IF(OR(B28="",NOT(N($J$9)&gt;0)),0,IF(N(C28)&gt;0,C28,1)*(IF((COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,MIN(31,N($J$9))),"VR"))&gt;0,N(G28),0)+IF((COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,MIN(31,N($J$9))),"RC"))&gt;0,N(I28),0)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DF28" s="31">
-        <f>IF(OR(B28="",NOT(N($J$9)&gt;0)),0,IF(N(C28)&gt;0,C28,1)*(COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,MIN(31,N($J$9))),"FOC"))*N(E28))</f>
+        <f>IF(B28="",0,IF(N(C28)&gt;0,C28,1)*(DC28*N(D28)+DD28*N(E28)))</f>
         <v/>
       </c>
       <c r="DG28" s="31">
-        <f>IF(OR(B28="",NOT(N($J$9)&gt;31)),0,IF(N(C28)&gt;0,C28,1)*((COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,MIN(62,N($J$9))),"DEMOB"))*N(D28)+(COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,MIN(62,N($J$9))),"O"))*N(E28)))</f>
+        <f>IF(OR(B28="",A28="Oui",DX28&lt;&gt;1),0,IF(N(C28)&gt;0,C28,1)*(N(F28)+N(H28)))</f>
         <v/>
       </c>
       <c r="DH28" s="31">
-        <f>IF(OR(B28="",A28="Oui",DO28&lt;&gt;2),0,IF(N(C28)&gt;0,C28,1)*(N(F28)+N(H28)))</f>
+        <f>IF(OR(B28="",N($DD$9)=0),0,IF(N(C28)&gt;0,C28,1)*(IF((COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,0+MAX(1,N($DD$9))),"VR"))&gt;0,N(G28),0)+IF((COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,0+MAX(1,N($DD$9))),"RC"))&gt;0,N(I28),0)))</f>
         <v/>
       </c>
       <c r="DI28" s="31">
-        <f>IF(OR(B28="",NOT(N($J$9)&gt;31)),0,IF(N(C28)&gt;0,C28,1)*(IF((COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,MIN(62,N($J$9))),"VR"))&gt;0,N(G28),0)+IF((COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,MIN(62,N($J$9))),"RC"))&gt;0,N(I28),0)))</f>
+        <f>IF(OR(B28="",N($DD$9)=0),0,IF(N(C28)&gt;0,C28,1)*(COUNTIF(INDEX($M28:$DA28,1):INDEX($M28:$DA28,0+MAX(1,N($DD$9))),"FOC"))*N(E28))</f>
         <v/>
       </c>
       <c r="DJ28" s="31">
-        <f>IF(OR(B28="",NOT(N($J$9)&gt;31)),0,IF(N(C28)&gt;0,C28,1)*(COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,MIN(62,N($J$9))),"FOC"))*N(E28))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DK28" s="31">
-        <f>IF(OR(B28="",NOT(N($J$9)&gt;62)),0,IF(N(C28)&gt;0,C28,1)*((COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,MIN(93,N($J$9))),"DEMOB"))*N(D28)+(COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,MIN(93,N($J$9))),"O"))*N(E28)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL28" s="31">
-        <f>IF(OR(B28="",A28="Oui",DO28&lt;&gt;3),0,IF(N(C28)&gt;0,C28,1)*(N(F28)+N(H28)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DM28" s="31">
-        <f>IF(OR(B28="",NOT(N($J$9)&gt;62)),0,IF(N(C28)&gt;0,C28,1)*(IF((COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,MIN(93,N($J$9))),"VR"))&gt;0,N(G28),0)+IF((COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,MIN(93,N($J$9))),"RC"))&gt;0,N(I28),0)))</f>
+        <f>IF(B28="",0,IF(N(C28)&gt;0,C28,1)*(DJ28*N(D28)+DK28*N(E28)))</f>
         <v/>
       </c>
       <c r="DN28" s="31">
-        <f>IF(OR(B28="",NOT(N($J$9)&gt;62)),0,IF(N(C28)&gt;0,C28,1)*(COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,MIN(93,N($J$9))),"FOC"))*N(E28))</f>
+        <f>IF(OR(B28="",A28="Oui",DX28&lt;&gt;2),0,IF(N(C28)&gt;0,C28,1)*(N(F28)+N(H28)))</f>
         <v/>
       </c>
       <c r="DO28" s="31">
-        <f>IF(B28="",0,IFERROR(INT((MATCH("O",$M28:INDEX($M28:$DA28,MAX(1,N($J$9))),0)-1)/31)+1,0))</f>
+        <f>IF(OR(B28="",N($DE$9)=0),0,IF(N(C28)&gt;0,C28,1)*(IF((COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,31+MAX(1,N($DE$9))),"VR"))&gt;0,N(G28),0)+IF((COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,31+MAX(1,N($DE$9))),"RC"))&gt;0,N(I28),0)))</f>
+        <v/>
+      </c>
+      <c r="DP28" s="31">
+        <f>IF(OR(B28="",N($DE$9)=0),0,IF(N(C28)&gt;0,C28,1)*(COUNTIF(INDEX($M28:$DA28,32):INDEX($M28:$DA28,31+MAX(1,N($DE$9))),"FOC"))*N(E28))</f>
+        <v/>
+      </c>
+      <c r="DQ28" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR28" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS28" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT28" s="31">
+        <f>IF(B28="",0,IF(N(C28)&gt;0,C28,1)*(DQ28*N(D28)+DR28*N(E28)))</f>
+        <v/>
+      </c>
+      <c r="DU28" s="31">
+        <f>IF(OR(B28="",A28="Oui",DX28&lt;&gt;3),0,IF(N(C28)&gt;0,C28,1)*(N(F28)+N(H28)))</f>
+        <v/>
+      </c>
+      <c r="DV28" s="31">
+        <f>IF(OR(B28="",N($DF$9)=0),0,IF(N(C28)&gt;0,C28,1)*(IF((COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,62+MAX(1,N($DF$9))),"VR"))&gt;0,N(G28),0)+IF((COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,62+MAX(1,N($DF$9))),"RC"))&gt;0,N(I28),0)))</f>
+        <v/>
+      </c>
+      <c r="DW28" s="31">
+        <f>IF(OR(B28="",N($DF$9)=0),0,IF(N(C28)&gt;0,C28,1)*(COUNTIF(INDEX($M28:$DA28,63):INDEX($M28:$DA28,62+MAX(1,N($DF$9))),"FOC"))*N(E28))</f>
+        <v/>
+      </c>
+      <c r="DX28" s="31">
+        <f>IF(B28="",0,IF(DD28&gt;0,1,IF(DK28&gt;0,2,IF(DR28&gt;0,3,0))))</f>
         <v/>
       </c>
     </row>
@@ -4116,15 +4546,15 @@
       <c r="H29" s="25" t="n"/>
       <c r="I29" s="25" t="n"/>
       <c r="J29" s="28">
-        <f>IF(B29="","",COUNTIF($M29:INDEX($M29:$DA29,MAX(1,N($J$9))),"S")+COUNTIF($M29:INDEX($M29:$DA29,MAX(1,N($J$9))),"MOB")+COUNTIF($M29:INDEX($M29:$DA29,MAX(1,N($J$9))),"DEMOB"))</f>
+        <f>IF(B29="","",DC29+DJ29+DQ29)</f>
         <v/>
       </c>
       <c r="K29" s="28">
-        <f>IF(B29="","",COUNTIF($M29:INDEX($M29:$DA29,MAX(1,N($J$9))),"O"))</f>
+        <f>IF(B29="","",DD29+DK29+DR29)</f>
         <v/>
       </c>
       <c r="L29" s="29">
-        <f>IF(B29="","",DC29+DG29+DK29+DD29+DH29+DL29+DE29+DI29+DM29)</f>
+        <f>IF(B29="","",DF29+DM29+DT29+DG29+DN29+DU29+DH29+DO29+DV29)</f>
         <v/>
       </c>
       <c r="M29" s="30" t="n"/>
@@ -4221,55 +4651,91 @@
       <c r="CZ29" s="30" t="n"/>
       <c r="DA29" s="30" t="n"/>
       <c r="DC29" s="31">
-        <f>IF(OR(B29="",NOT(N($J$9)&gt;0)),0,IF(N(C29)&gt;0,C29,1)*((COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,MIN(31,N($J$9))),"DEMOB"))*N(D29)+(COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,MIN(31,N($J$9))),"O"))*N(E29)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD29" s="31">
-        <f>IF(OR(B29="",A29="Oui",DO29&lt;&gt;1),0,IF(N(C29)&gt;0,C29,1)*(N(F29)+N(H29)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,0+MAX(1,N($DD$9))),"O"))</f>
         <v/>
       </c>
       <c r="DE29" s="31">
-        <f>IF(OR(B29="",NOT(N($J$9)&gt;0)),0,IF(N(C29)&gt;0,C29,1)*(IF((COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,MIN(31,N($J$9))),"VR"))&gt;0,N(G29),0)+IF((COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,MIN(31,N($J$9))),"RC"))&gt;0,N(I29),0)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DF29" s="31">
-        <f>IF(OR(B29="",NOT(N($J$9)&gt;0)),0,IF(N(C29)&gt;0,C29,1)*(COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,MIN(31,N($J$9))),"FOC"))*N(E29))</f>
+        <f>IF(B29="",0,IF(N(C29)&gt;0,C29,1)*(DC29*N(D29)+DD29*N(E29)))</f>
         <v/>
       </c>
       <c r="DG29" s="31">
-        <f>IF(OR(B29="",NOT(N($J$9)&gt;31)),0,IF(N(C29)&gt;0,C29,1)*((COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,MIN(62,N($J$9))),"DEMOB"))*N(D29)+(COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,MIN(62,N($J$9))),"O"))*N(E29)))</f>
+        <f>IF(OR(B29="",A29="Oui",DX29&lt;&gt;1),0,IF(N(C29)&gt;0,C29,1)*(N(F29)+N(H29)))</f>
         <v/>
       </c>
       <c r="DH29" s="31">
-        <f>IF(OR(B29="",A29="Oui",DO29&lt;&gt;2),0,IF(N(C29)&gt;0,C29,1)*(N(F29)+N(H29)))</f>
+        <f>IF(OR(B29="",N($DD$9)=0),0,IF(N(C29)&gt;0,C29,1)*(IF((COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,0+MAX(1,N($DD$9))),"VR"))&gt;0,N(G29),0)+IF((COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,0+MAX(1,N($DD$9))),"RC"))&gt;0,N(I29),0)))</f>
         <v/>
       </c>
       <c r="DI29" s="31">
-        <f>IF(OR(B29="",NOT(N($J$9)&gt;31)),0,IF(N(C29)&gt;0,C29,1)*(IF((COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,MIN(62,N($J$9))),"VR"))&gt;0,N(G29),0)+IF((COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,MIN(62,N($J$9))),"RC"))&gt;0,N(I29),0)))</f>
+        <f>IF(OR(B29="",N($DD$9)=0),0,IF(N(C29)&gt;0,C29,1)*(COUNTIF(INDEX($M29:$DA29,1):INDEX($M29:$DA29,0+MAX(1,N($DD$9))),"FOC"))*N(E29))</f>
         <v/>
       </c>
       <c r="DJ29" s="31">
-        <f>IF(OR(B29="",NOT(N($J$9)&gt;31)),0,IF(N(C29)&gt;0,C29,1)*(COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,MIN(62,N($J$9))),"FOC"))*N(E29))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DK29" s="31">
-        <f>IF(OR(B29="",NOT(N($J$9)&gt;62)),0,IF(N(C29)&gt;0,C29,1)*((COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,MIN(93,N($J$9))),"DEMOB"))*N(D29)+(COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,MIN(93,N($J$9))),"O"))*N(E29)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL29" s="31">
-        <f>IF(OR(B29="",A29="Oui",DO29&lt;&gt;3),0,IF(N(C29)&gt;0,C29,1)*(N(F29)+N(H29)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DM29" s="31">
-        <f>IF(OR(B29="",NOT(N($J$9)&gt;62)),0,IF(N(C29)&gt;0,C29,1)*(IF((COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,MIN(93,N($J$9))),"VR"))&gt;0,N(G29),0)+IF((COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,MIN(93,N($J$9))),"RC"))&gt;0,N(I29),0)))</f>
+        <f>IF(B29="",0,IF(N(C29)&gt;0,C29,1)*(DJ29*N(D29)+DK29*N(E29)))</f>
         <v/>
       </c>
       <c r="DN29" s="31">
-        <f>IF(OR(B29="",NOT(N($J$9)&gt;62)),0,IF(N(C29)&gt;0,C29,1)*(COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,MIN(93,N($J$9))),"FOC"))*N(E29))</f>
+        <f>IF(OR(B29="",A29="Oui",DX29&lt;&gt;2),0,IF(N(C29)&gt;0,C29,1)*(N(F29)+N(H29)))</f>
         <v/>
       </c>
       <c r="DO29" s="31">
-        <f>IF(B29="",0,IFERROR(INT((MATCH("O",$M29:INDEX($M29:$DA29,MAX(1,N($J$9))),0)-1)/31)+1,0))</f>
+        <f>IF(OR(B29="",N($DE$9)=0),0,IF(N(C29)&gt;0,C29,1)*(IF((COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,31+MAX(1,N($DE$9))),"VR"))&gt;0,N(G29),0)+IF((COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,31+MAX(1,N($DE$9))),"RC"))&gt;0,N(I29),0)))</f>
+        <v/>
+      </c>
+      <c r="DP29" s="31">
+        <f>IF(OR(B29="",N($DE$9)=0),0,IF(N(C29)&gt;0,C29,1)*(COUNTIF(INDEX($M29:$DA29,32):INDEX($M29:$DA29,31+MAX(1,N($DE$9))),"FOC"))*N(E29))</f>
+        <v/>
+      </c>
+      <c r="DQ29" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR29" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS29" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT29" s="31">
+        <f>IF(B29="",0,IF(N(C29)&gt;0,C29,1)*(DQ29*N(D29)+DR29*N(E29)))</f>
+        <v/>
+      </c>
+      <c r="DU29" s="31">
+        <f>IF(OR(B29="",A29="Oui",DX29&lt;&gt;3),0,IF(N(C29)&gt;0,C29,1)*(N(F29)+N(H29)))</f>
+        <v/>
+      </c>
+      <c r="DV29" s="31">
+        <f>IF(OR(B29="",N($DF$9)=0),0,IF(N(C29)&gt;0,C29,1)*(IF((COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,62+MAX(1,N($DF$9))),"VR"))&gt;0,N(G29),0)+IF((COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,62+MAX(1,N($DF$9))),"RC"))&gt;0,N(I29),0)))</f>
+        <v/>
+      </c>
+      <c r="DW29" s="31">
+        <f>IF(OR(B29="",N($DF$9)=0),0,IF(N(C29)&gt;0,C29,1)*(COUNTIF(INDEX($M29:$DA29,63):INDEX($M29:$DA29,62+MAX(1,N($DF$9))),"FOC"))*N(E29))</f>
+        <v/>
+      </c>
+      <c r="DX29" s="31">
+        <f>IF(B29="",0,IF(DD29&gt;0,1,IF(DK29&gt;0,2,IF(DR29&gt;0,3,0))))</f>
         <v/>
       </c>
     </row>
@@ -4284,15 +4750,15 @@
       <c r="H30" s="25" t="n"/>
       <c r="I30" s="25" t="n"/>
       <c r="J30" s="28">
-        <f>IF(B30="","",COUNTIF($M30:INDEX($M30:$DA30,MAX(1,N($J$9))),"S")+COUNTIF($M30:INDEX($M30:$DA30,MAX(1,N($J$9))),"MOB")+COUNTIF($M30:INDEX($M30:$DA30,MAX(1,N($J$9))),"DEMOB"))</f>
+        <f>IF(B30="","",DC30+DJ30+DQ30)</f>
         <v/>
       </c>
       <c r="K30" s="28">
-        <f>IF(B30="","",COUNTIF($M30:INDEX($M30:$DA30,MAX(1,N($J$9))),"O"))</f>
+        <f>IF(B30="","",DD30+DK30+DR30)</f>
         <v/>
       </c>
       <c r="L30" s="29">
-        <f>IF(B30="","",DC30+DG30+DK30+DD30+DH30+DL30+DE30+DI30+DM30)</f>
+        <f>IF(B30="","",DF30+DM30+DT30+DG30+DN30+DU30+DH30+DO30+DV30)</f>
         <v/>
       </c>
       <c r="M30" s="30" t="n"/>
@@ -4389,55 +4855,91 @@
       <c r="CZ30" s="30" t="n"/>
       <c r="DA30" s="30" t="n"/>
       <c r="DC30" s="31">
-        <f>IF(OR(B30="",NOT(N($J$9)&gt;0)),0,IF(N(C30)&gt;0,C30,1)*((COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,MIN(31,N($J$9))),"DEMOB"))*N(D30)+(COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,MIN(31,N($J$9))),"O"))*N(E30)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD30" s="31">
-        <f>IF(OR(B30="",A30="Oui",DO30&lt;&gt;1),0,IF(N(C30)&gt;0,C30,1)*(N(F30)+N(H30)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,0+MAX(1,N($DD$9))),"O"))</f>
         <v/>
       </c>
       <c r="DE30" s="31">
-        <f>IF(OR(B30="",NOT(N($J$9)&gt;0)),0,IF(N(C30)&gt;0,C30,1)*(IF((COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,MIN(31,N($J$9))),"VR"))&gt;0,N(G30),0)+IF((COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,MIN(31,N($J$9))),"RC"))&gt;0,N(I30),0)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DF30" s="31">
-        <f>IF(OR(B30="",NOT(N($J$9)&gt;0)),0,IF(N(C30)&gt;0,C30,1)*(COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,MIN(31,N($J$9))),"FOC"))*N(E30))</f>
+        <f>IF(B30="",0,IF(N(C30)&gt;0,C30,1)*(DC30*N(D30)+DD30*N(E30)))</f>
         <v/>
       </c>
       <c r="DG30" s="31">
-        <f>IF(OR(B30="",NOT(N($J$9)&gt;31)),0,IF(N(C30)&gt;0,C30,1)*((COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,MIN(62,N($J$9))),"DEMOB"))*N(D30)+(COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,MIN(62,N($J$9))),"O"))*N(E30)))</f>
+        <f>IF(OR(B30="",A30="Oui",DX30&lt;&gt;1),0,IF(N(C30)&gt;0,C30,1)*(N(F30)+N(H30)))</f>
         <v/>
       </c>
       <c r="DH30" s="31">
-        <f>IF(OR(B30="",A30="Oui",DO30&lt;&gt;2),0,IF(N(C30)&gt;0,C30,1)*(N(F30)+N(H30)))</f>
+        <f>IF(OR(B30="",N($DD$9)=0),0,IF(N(C30)&gt;0,C30,1)*(IF((COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,0+MAX(1,N($DD$9))),"VR"))&gt;0,N(G30),0)+IF((COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,0+MAX(1,N($DD$9))),"RC"))&gt;0,N(I30),0)))</f>
         <v/>
       </c>
       <c r="DI30" s="31">
-        <f>IF(OR(B30="",NOT(N($J$9)&gt;31)),0,IF(N(C30)&gt;0,C30,1)*(IF((COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,MIN(62,N($J$9))),"VR"))&gt;0,N(G30),0)+IF((COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,MIN(62,N($J$9))),"RC"))&gt;0,N(I30),0)))</f>
+        <f>IF(OR(B30="",N($DD$9)=0),0,IF(N(C30)&gt;0,C30,1)*(COUNTIF(INDEX($M30:$DA30,1):INDEX($M30:$DA30,0+MAX(1,N($DD$9))),"FOC"))*N(E30))</f>
         <v/>
       </c>
       <c r="DJ30" s="31">
-        <f>IF(OR(B30="",NOT(N($J$9)&gt;31)),0,IF(N(C30)&gt;0,C30,1)*(COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,MIN(62,N($J$9))),"FOC"))*N(E30))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DK30" s="31">
-        <f>IF(OR(B30="",NOT(N($J$9)&gt;62)),0,IF(N(C30)&gt;0,C30,1)*((COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,MIN(93,N($J$9))),"DEMOB"))*N(D30)+(COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,MIN(93,N($J$9))),"O"))*N(E30)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL30" s="31">
-        <f>IF(OR(B30="",A30="Oui",DO30&lt;&gt;3),0,IF(N(C30)&gt;0,C30,1)*(N(F30)+N(H30)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DM30" s="31">
-        <f>IF(OR(B30="",NOT(N($J$9)&gt;62)),0,IF(N(C30)&gt;0,C30,1)*(IF((COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,MIN(93,N($J$9))),"VR"))&gt;0,N(G30),0)+IF((COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,MIN(93,N($J$9))),"RC"))&gt;0,N(I30),0)))</f>
+        <f>IF(B30="",0,IF(N(C30)&gt;0,C30,1)*(DJ30*N(D30)+DK30*N(E30)))</f>
         <v/>
       </c>
       <c r="DN30" s="31">
-        <f>IF(OR(B30="",NOT(N($J$9)&gt;62)),0,IF(N(C30)&gt;0,C30,1)*(COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,MIN(93,N($J$9))),"FOC"))*N(E30))</f>
+        <f>IF(OR(B30="",A30="Oui",DX30&lt;&gt;2),0,IF(N(C30)&gt;0,C30,1)*(N(F30)+N(H30)))</f>
         <v/>
       </c>
       <c r="DO30" s="31">
-        <f>IF(B30="",0,IFERROR(INT((MATCH("O",$M30:INDEX($M30:$DA30,MAX(1,N($J$9))),0)-1)/31)+1,0))</f>
+        <f>IF(OR(B30="",N($DE$9)=0),0,IF(N(C30)&gt;0,C30,1)*(IF((COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,31+MAX(1,N($DE$9))),"VR"))&gt;0,N(G30),0)+IF((COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,31+MAX(1,N($DE$9))),"RC"))&gt;0,N(I30),0)))</f>
+        <v/>
+      </c>
+      <c r="DP30" s="31">
+        <f>IF(OR(B30="",N($DE$9)=0),0,IF(N(C30)&gt;0,C30,1)*(COUNTIF(INDEX($M30:$DA30,32):INDEX($M30:$DA30,31+MAX(1,N($DE$9))),"FOC"))*N(E30))</f>
+        <v/>
+      </c>
+      <c r="DQ30" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR30" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS30" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT30" s="31">
+        <f>IF(B30="",0,IF(N(C30)&gt;0,C30,1)*(DQ30*N(D30)+DR30*N(E30)))</f>
+        <v/>
+      </c>
+      <c r="DU30" s="31">
+        <f>IF(OR(B30="",A30="Oui",DX30&lt;&gt;3),0,IF(N(C30)&gt;0,C30,1)*(N(F30)+N(H30)))</f>
+        <v/>
+      </c>
+      <c r="DV30" s="31">
+        <f>IF(OR(B30="",N($DF$9)=0),0,IF(N(C30)&gt;0,C30,1)*(IF((COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,62+MAX(1,N($DF$9))),"VR"))&gt;0,N(G30),0)+IF((COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,62+MAX(1,N($DF$9))),"RC"))&gt;0,N(I30),0)))</f>
+        <v/>
+      </c>
+      <c r="DW30" s="31">
+        <f>IF(OR(B30="",N($DF$9)=0),0,IF(N(C30)&gt;0,C30,1)*(COUNTIF(INDEX($M30:$DA30,63):INDEX($M30:$DA30,62+MAX(1,N($DF$9))),"FOC"))*N(E30))</f>
+        <v/>
+      </c>
+      <c r="DX30" s="31">
+        <f>IF(B30="",0,IF(DD30&gt;0,1,IF(DK30&gt;0,2,IF(DR30&gt;0,3,0))))</f>
         <v/>
       </c>
     </row>
@@ -4452,15 +4954,15 @@
       <c r="H31" s="25" t="n"/>
       <c r="I31" s="25" t="n"/>
       <c r="J31" s="28">
-        <f>IF(B31="","",COUNTIF($M31:INDEX($M31:$DA31,MAX(1,N($J$9))),"S")+COUNTIF($M31:INDEX($M31:$DA31,MAX(1,N($J$9))),"MOB")+COUNTIF($M31:INDEX($M31:$DA31,MAX(1,N($J$9))),"DEMOB"))</f>
+        <f>IF(B31="","",DC31+DJ31+DQ31)</f>
         <v/>
       </c>
       <c r="K31" s="28">
-        <f>IF(B31="","",COUNTIF($M31:INDEX($M31:$DA31,MAX(1,N($J$9))),"O"))</f>
+        <f>IF(B31="","",DD31+DK31+DR31)</f>
         <v/>
       </c>
       <c r="L31" s="29">
-        <f>IF(B31="","",DC31+DG31+DK31+DD31+DH31+DL31+DE31+DI31+DM31)</f>
+        <f>IF(B31="","",DF31+DM31+DT31+DG31+DN31+DU31+DH31+DO31+DV31)</f>
         <v/>
       </c>
       <c r="M31" s="30" t="n"/>
@@ -4557,55 +5059,91 @@
       <c r="CZ31" s="30" t="n"/>
       <c r="DA31" s="30" t="n"/>
       <c r="DC31" s="31">
-        <f>IF(OR(B31="",NOT(N($J$9)&gt;0)),0,IF(N(C31)&gt;0,C31,1)*((COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,MIN(31,N($J$9))),"DEMOB"))*N(D31)+(COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,MIN(31,N($J$9))),"O"))*N(E31)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD31" s="31">
-        <f>IF(OR(B31="",A31="Oui",DO31&lt;&gt;1),0,IF(N(C31)&gt;0,C31,1)*(N(F31)+N(H31)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,0+MAX(1,N($DD$9))),"O"))</f>
         <v/>
       </c>
       <c r="DE31" s="31">
-        <f>IF(OR(B31="",NOT(N($J$9)&gt;0)),0,IF(N(C31)&gt;0,C31,1)*(IF((COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,MIN(31,N($J$9))),"VR"))&gt;0,N(G31),0)+IF((COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,MIN(31,N($J$9))),"RC"))&gt;0,N(I31),0)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DF31" s="31">
-        <f>IF(OR(B31="",NOT(N($J$9)&gt;0)),0,IF(N(C31)&gt;0,C31,1)*(COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,MIN(31,N($J$9))),"FOC"))*N(E31))</f>
+        <f>IF(B31="",0,IF(N(C31)&gt;0,C31,1)*(DC31*N(D31)+DD31*N(E31)))</f>
         <v/>
       </c>
       <c r="DG31" s="31">
-        <f>IF(OR(B31="",NOT(N($J$9)&gt;31)),0,IF(N(C31)&gt;0,C31,1)*((COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,MIN(62,N($J$9))),"DEMOB"))*N(D31)+(COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,MIN(62,N($J$9))),"O"))*N(E31)))</f>
+        <f>IF(OR(B31="",A31="Oui",DX31&lt;&gt;1),0,IF(N(C31)&gt;0,C31,1)*(N(F31)+N(H31)))</f>
         <v/>
       </c>
       <c r="DH31" s="31">
-        <f>IF(OR(B31="",A31="Oui",DO31&lt;&gt;2),0,IF(N(C31)&gt;0,C31,1)*(N(F31)+N(H31)))</f>
+        <f>IF(OR(B31="",N($DD$9)=0),0,IF(N(C31)&gt;0,C31,1)*(IF((COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,0+MAX(1,N($DD$9))),"VR"))&gt;0,N(G31),0)+IF((COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,0+MAX(1,N($DD$9))),"RC"))&gt;0,N(I31),0)))</f>
         <v/>
       </c>
       <c r="DI31" s="31">
-        <f>IF(OR(B31="",NOT(N($J$9)&gt;31)),0,IF(N(C31)&gt;0,C31,1)*(IF((COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,MIN(62,N($J$9))),"VR"))&gt;0,N(G31),0)+IF((COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,MIN(62,N($J$9))),"RC"))&gt;0,N(I31),0)))</f>
+        <f>IF(OR(B31="",N($DD$9)=0),0,IF(N(C31)&gt;0,C31,1)*(COUNTIF(INDEX($M31:$DA31,1):INDEX($M31:$DA31,0+MAX(1,N($DD$9))),"FOC"))*N(E31))</f>
         <v/>
       </c>
       <c r="DJ31" s="31">
-        <f>IF(OR(B31="",NOT(N($J$9)&gt;31)),0,IF(N(C31)&gt;0,C31,1)*(COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,MIN(62,N($J$9))),"FOC"))*N(E31))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DK31" s="31">
-        <f>IF(OR(B31="",NOT(N($J$9)&gt;62)),0,IF(N(C31)&gt;0,C31,1)*((COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,MIN(93,N($J$9))),"DEMOB"))*N(D31)+(COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,MIN(93,N($J$9))),"O"))*N(E31)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL31" s="31">
-        <f>IF(OR(B31="",A31="Oui",DO31&lt;&gt;3),0,IF(N(C31)&gt;0,C31,1)*(N(F31)+N(H31)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DM31" s="31">
-        <f>IF(OR(B31="",NOT(N($J$9)&gt;62)),0,IF(N(C31)&gt;0,C31,1)*(IF((COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,MIN(93,N($J$9))),"VR"))&gt;0,N(G31),0)+IF((COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,MIN(93,N($J$9))),"RC"))&gt;0,N(I31),0)))</f>
+        <f>IF(B31="",0,IF(N(C31)&gt;0,C31,1)*(DJ31*N(D31)+DK31*N(E31)))</f>
         <v/>
       </c>
       <c r="DN31" s="31">
-        <f>IF(OR(B31="",NOT(N($J$9)&gt;62)),0,IF(N(C31)&gt;0,C31,1)*(COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,MIN(93,N($J$9))),"FOC"))*N(E31))</f>
+        <f>IF(OR(B31="",A31="Oui",DX31&lt;&gt;2),0,IF(N(C31)&gt;0,C31,1)*(N(F31)+N(H31)))</f>
         <v/>
       </c>
       <c r="DO31" s="31">
-        <f>IF(B31="",0,IFERROR(INT((MATCH("O",$M31:INDEX($M31:$DA31,MAX(1,N($J$9))),0)-1)/31)+1,0))</f>
+        <f>IF(OR(B31="",N($DE$9)=0),0,IF(N(C31)&gt;0,C31,1)*(IF((COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,31+MAX(1,N($DE$9))),"VR"))&gt;0,N(G31),0)+IF((COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,31+MAX(1,N($DE$9))),"RC"))&gt;0,N(I31),0)))</f>
+        <v/>
+      </c>
+      <c r="DP31" s="31">
+        <f>IF(OR(B31="",N($DE$9)=0),0,IF(N(C31)&gt;0,C31,1)*(COUNTIF(INDEX($M31:$DA31,32):INDEX($M31:$DA31,31+MAX(1,N($DE$9))),"FOC"))*N(E31))</f>
+        <v/>
+      </c>
+      <c r="DQ31" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR31" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS31" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT31" s="31">
+        <f>IF(B31="",0,IF(N(C31)&gt;0,C31,1)*(DQ31*N(D31)+DR31*N(E31)))</f>
+        <v/>
+      </c>
+      <c r="DU31" s="31">
+        <f>IF(OR(B31="",A31="Oui",DX31&lt;&gt;3),0,IF(N(C31)&gt;0,C31,1)*(N(F31)+N(H31)))</f>
+        <v/>
+      </c>
+      <c r="DV31" s="31">
+        <f>IF(OR(B31="",N($DF$9)=0),0,IF(N(C31)&gt;0,C31,1)*(IF((COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,62+MAX(1,N($DF$9))),"VR"))&gt;0,N(G31),0)+IF((COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,62+MAX(1,N($DF$9))),"RC"))&gt;0,N(I31),0)))</f>
+        <v/>
+      </c>
+      <c r="DW31" s="31">
+        <f>IF(OR(B31="",N($DF$9)=0),0,IF(N(C31)&gt;0,C31,1)*(COUNTIF(INDEX($M31:$DA31,63):INDEX($M31:$DA31,62+MAX(1,N($DF$9))),"FOC"))*N(E31))</f>
+        <v/>
+      </c>
+      <c r="DX31" s="31">
+        <f>IF(B31="",0,IF(DD31&gt;0,1,IF(DK31&gt;0,2,IF(DR31&gt;0,3,0))))</f>
         <v/>
       </c>
     </row>
@@ -4620,15 +5158,15 @@
       <c r="H32" s="25" t="n"/>
       <c r="I32" s="25" t="n"/>
       <c r="J32" s="28">
-        <f>IF(B32="","",COUNTIF($M32:INDEX($M32:$DA32,MAX(1,N($J$9))),"S")+COUNTIF($M32:INDEX($M32:$DA32,MAX(1,N($J$9))),"MOB")+COUNTIF($M32:INDEX($M32:$DA32,MAX(1,N($J$9))),"DEMOB"))</f>
+        <f>IF(B32="","",DC32+DJ32+DQ32)</f>
         <v/>
       </c>
       <c r="K32" s="28">
-        <f>IF(B32="","",COUNTIF($M32:INDEX($M32:$DA32,MAX(1,N($J$9))),"O"))</f>
+        <f>IF(B32="","",DD32+DK32+DR32)</f>
         <v/>
       </c>
       <c r="L32" s="29">
-        <f>IF(B32="","",DC32+DG32+DK32+DD32+DH32+DL32+DE32+DI32+DM32)</f>
+        <f>IF(B32="","",DF32+DM32+DT32+DG32+DN32+DU32+DH32+DO32+DV32)</f>
         <v/>
       </c>
       <c r="M32" s="30" t="n"/>
@@ -4725,55 +5263,91 @@
       <c r="CZ32" s="30" t="n"/>
       <c r="DA32" s="30" t="n"/>
       <c r="DC32" s="31">
-        <f>IF(OR(B32="",NOT(N($J$9)&gt;0)),0,IF(N(C32)&gt;0,C32,1)*((COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,MIN(31,N($J$9))),"DEMOB"))*N(D32)+(COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,MIN(31,N($J$9))),"O"))*N(E32)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD32" s="31">
-        <f>IF(OR(B32="",A32="Oui",DO32&lt;&gt;1),0,IF(N(C32)&gt;0,C32,1)*(N(F32)+N(H32)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,0+MAX(1,N($DD$9))),"O"))</f>
         <v/>
       </c>
       <c r="DE32" s="31">
-        <f>IF(OR(B32="",NOT(N($J$9)&gt;0)),0,IF(N(C32)&gt;0,C32,1)*(IF((COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,MIN(31,N($J$9))),"VR"))&gt;0,N(G32),0)+IF((COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,MIN(31,N($J$9))),"RC"))&gt;0,N(I32),0)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DF32" s="31">
-        <f>IF(OR(B32="",NOT(N($J$9)&gt;0)),0,IF(N(C32)&gt;0,C32,1)*(COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,MIN(31,N($J$9))),"FOC"))*N(E32))</f>
+        <f>IF(B32="",0,IF(N(C32)&gt;0,C32,1)*(DC32*N(D32)+DD32*N(E32)))</f>
         <v/>
       </c>
       <c r="DG32" s="31">
-        <f>IF(OR(B32="",NOT(N($J$9)&gt;31)),0,IF(N(C32)&gt;0,C32,1)*((COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,MIN(62,N($J$9))),"DEMOB"))*N(D32)+(COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,MIN(62,N($J$9))),"O"))*N(E32)))</f>
+        <f>IF(OR(B32="",A32="Oui",DX32&lt;&gt;1),0,IF(N(C32)&gt;0,C32,1)*(N(F32)+N(H32)))</f>
         <v/>
       </c>
       <c r="DH32" s="31">
-        <f>IF(OR(B32="",A32="Oui",DO32&lt;&gt;2),0,IF(N(C32)&gt;0,C32,1)*(N(F32)+N(H32)))</f>
+        <f>IF(OR(B32="",N($DD$9)=0),0,IF(N(C32)&gt;0,C32,1)*(IF((COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,0+MAX(1,N($DD$9))),"VR"))&gt;0,N(G32),0)+IF((COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,0+MAX(1,N($DD$9))),"RC"))&gt;0,N(I32),0)))</f>
         <v/>
       </c>
       <c r="DI32" s="31">
-        <f>IF(OR(B32="",NOT(N($J$9)&gt;31)),0,IF(N(C32)&gt;0,C32,1)*(IF((COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,MIN(62,N($J$9))),"VR"))&gt;0,N(G32),0)+IF((COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,MIN(62,N($J$9))),"RC"))&gt;0,N(I32),0)))</f>
+        <f>IF(OR(B32="",N($DD$9)=0),0,IF(N(C32)&gt;0,C32,1)*(COUNTIF(INDEX($M32:$DA32,1):INDEX($M32:$DA32,0+MAX(1,N($DD$9))),"FOC"))*N(E32))</f>
         <v/>
       </c>
       <c r="DJ32" s="31">
-        <f>IF(OR(B32="",NOT(N($J$9)&gt;31)),0,IF(N(C32)&gt;0,C32,1)*(COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,MIN(62,N($J$9))),"FOC"))*N(E32))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DK32" s="31">
-        <f>IF(OR(B32="",NOT(N($J$9)&gt;62)),0,IF(N(C32)&gt;0,C32,1)*((COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,MIN(93,N($J$9))),"DEMOB"))*N(D32)+(COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,MIN(93,N($J$9))),"O"))*N(E32)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL32" s="31">
-        <f>IF(OR(B32="",A32="Oui",DO32&lt;&gt;3),0,IF(N(C32)&gt;0,C32,1)*(N(F32)+N(H32)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DM32" s="31">
-        <f>IF(OR(B32="",NOT(N($J$9)&gt;62)),0,IF(N(C32)&gt;0,C32,1)*(IF((COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,MIN(93,N($J$9))),"VR"))&gt;0,N(G32),0)+IF((COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,MIN(93,N($J$9))),"RC"))&gt;0,N(I32),0)))</f>
+        <f>IF(B32="",0,IF(N(C32)&gt;0,C32,1)*(DJ32*N(D32)+DK32*N(E32)))</f>
         <v/>
       </c>
       <c r="DN32" s="31">
-        <f>IF(OR(B32="",NOT(N($J$9)&gt;62)),0,IF(N(C32)&gt;0,C32,1)*(COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,MIN(93,N($J$9))),"FOC"))*N(E32))</f>
+        <f>IF(OR(B32="",A32="Oui",DX32&lt;&gt;2),0,IF(N(C32)&gt;0,C32,1)*(N(F32)+N(H32)))</f>
         <v/>
       </c>
       <c r="DO32" s="31">
-        <f>IF(B32="",0,IFERROR(INT((MATCH("O",$M32:INDEX($M32:$DA32,MAX(1,N($J$9))),0)-1)/31)+1,0))</f>
+        <f>IF(OR(B32="",N($DE$9)=0),0,IF(N(C32)&gt;0,C32,1)*(IF((COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,31+MAX(1,N($DE$9))),"VR"))&gt;0,N(G32),0)+IF((COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,31+MAX(1,N($DE$9))),"RC"))&gt;0,N(I32),0)))</f>
+        <v/>
+      </c>
+      <c r="DP32" s="31">
+        <f>IF(OR(B32="",N($DE$9)=0),0,IF(N(C32)&gt;0,C32,1)*(COUNTIF(INDEX($M32:$DA32,32):INDEX($M32:$DA32,31+MAX(1,N($DE$9))),"FOC"))*N(E32))</f>
+        <v/>
+      </c>
+      <c r="DQ32" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR32" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS32" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT32" s="31">
+        <f>IF(B32="",0,IF(N(C32)&gt;0,C32,1)*(DQ32*N(D32)+DR32*N(E32)))</f>
+        <v/>
+      </c>
+      <c r="DU32" s="31">
+        <f>IF(OR(B32="",A32="Oui",DX32&lt;&gt;3),0,IF(N(C32)&gt;0,C32,1)*(N(F32)+N(H32)))</f>
+        <v/>
+      </c>
+      <c r="DV32" s="31">
+        <f>IF(OR(B32="",N($DF$9)=0),0,IF(N(C32)&gt;0,C32,1)*(IF((COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,62+MAX(1,N($DF$9))),"VR"))&gt;0,N(G32),0)+IF((COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,62+MAX(1,N($DF$9))),"RC"))&gt;0,N(I32),0)))</f>
+        <v/>
+      </c>
+      <c r="DW32" s="31">
+        <f>IF(OR(B32="",N($DF$9)=0),0,IF(N(C32)&gt;0,C32,1)*(COUNTIF(INDEX($M32:$DA32,63):INDEX($M32:$DA32,62+MAX(1,N($DF$9))),"FOC"))*N(E32))</f>
+        <v/>
+      </c>
+      <c r="DX32" s="31">
+        <f>IF(B32="",0,IF(DD32&gt;0,1,IF(DK32&gt;0,2,IF(DR32&gt;0,3,0))))</f>
         <v/>
       </c>
     </row>
@@ -4788,15 +5362,15 @@
       <c r="H33" s="25" t="n"/>
       <c r="I33" s="25" t="n"/>
       <c r="J33" s="28">
-        <f>IF(B33="","",COUNTIF($M33:INDEX($M33:$DA33,MAX(1,N($J$9))),"S")+COUNTIF($M33:INDEX($M33:$DA33,MAX(1,N($J$9))),"MOB")+COUNTIF($M33:INDEX($M33:$DA33,MAX(1,N($J$9))),"DEMOB"))</f>
+        <f>IF(B33="","",DC33+DJ33+DQ33)</f>
         <v/>
       </c>
       <c r="K33" s="28">
-        <f>IF(B33="","",COUNTIF($M33:INDEX($M33:$DA33,MAX(1,N($J$9))),"O"))</f>
+        <f>IF(B33="","",DD33+DK33+DR33)</f>
         <v/>
       </c>
       <c r="L33" s="29">
-        <f>IF(B33="","",DC33+DG33+DK33+DD33+DH33+DL33+DE33+DI33+DM33)</f>
+        <f>IF(B33="","",DF33+DM33+DT33+DG33+DN33+DU33+DH33+DO33+DV33)</f>
         <v/>
       </c>
       <c r="M33" s="30" t="n"/>
@@ -4893,55 +5467,91 @@
       <c r="CZ33" s="30" t="n"/>
       <c r="DA33" s="30" t="n"/>
       <c r="DC33" s="31">
-        <f>IF(OR(B33="",NOT(N($J$9)&gt;0)),0,IF(N(C33)&gt;0,C33,1)*((COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,MIN(31,N($J$9))),"S")+COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,MIN(31,N($J$9))),"MOB")+COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,MIN(31,N($J$9))),"DEMOB"))*N(D33)+(COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,MIN(31,N($J$9))),"O"))*N(E33)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,0+MAX(1,N($DD$9))),"S")+COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DD33" s="31">
-        <f>IF(OR(B33="",A33="Oui",DO33&lt;&gt;1),0,IF(N(C33)&gt;0,C33,1)*(N(F33)+N(H33)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,0+MAX(1,N($DD$9))),"O"))</f>
         <v/>
       </c>
       <c r="DE33" s="31">
-        <f>IF(OR(B33="",NOT(N($J$9)&gt;0)),0,IF(N(C33)&gt;0,C33,1)*(IF((COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,MIN(31,N($J$9))),"VR"))&gt;0,N(G33),0)+IF((COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,MIN(31,N($J$9))),"RC"))&gt;0,N(I33),0)))</f>
+        <f>IF(N($DD$9)=0,0,COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,0+MAX(1,N($DD$9))),"MOB")+COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,0+MAX(1,N($DD$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DF33" s="31">
-        <f>IF(OR(B33="",NOT(N($J$9)&gt;0)),0,IF(N(C33)&gt;0,C33,1)*(COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,MIN(31,N($J$9))),"FOC"))*N(E33))</f>
+        <f>IF(B33="",0,IF(N(C33)&gt;0,C33,1)*(DC33*N(D33)+DD33*N(E33)))</f>
         <v/>
       </c>
       <c r="DG33" s="31">
-        <f>IF(OR(B33="",NOT(N($J$9)&gt;31)),0,IF(N(C33)&gt;0,C33,1)*((COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,MIN(62,N($J$9))),"S")+COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,MIN(62,N($J$9))),"MOB")+COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,MIN(62,N($J$9))),"DEMOB"))*N(D33)+(COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,MIN(62,N($J$9))),"O"))*N(E33)))</f>
+        <f>IF(OR(B33="",A33="Oui",DX33&lt;&gt;1),0,IF(N(C33)&gt;0,C33,1)*(N(F33)+N(H33)))</f>
         <v/>
       </c>
       <c r="DH33" s="31">
-        <f>IF(OR(B33="",A33="Oui",DO33&lt;&gt;2),0,IF(N(C33)&gt;0,C33,1)*(N(F33)+N(H33)))</f>
+        <f>IF(OR(B33="",N($DD$9)=0),0,IF(N(C33)&gt;0,C33,1)*(IF((COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,0+MAX(1,N($DD$9))),"VR"))&gt;0,N(G33),0)+IF((COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,0+MAX(1,N($DD$9))),"RC"))&gt;0,N(I33),0)))</f>
         <v/>
       </c>
       <c r="DI33" s="31">
-        <f>IF(OR(B33="",NOT(N($J$9)&gt;31)),0,IF(N(C33)&gt;0,C33,1)*(IF((COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,MIN(62,N($J$9))),"VR"))&gt;0,N(G33),0)+IF((COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,MIN(62,N($J$9))),"RC"))&gt;0,N(I33),0)))</f>
+        <f>IF(OR(B33="",N($DD$9)=0),0,IF(N(C33)&gt;0,C33,1)*(COUNTIF(INDEX($M33:$DA33,1):INDEX($M33:$DA33,0+MAX(1,N($DD$9))),"FOC"))*N(E33))</f>
         <v/>
       </c>
       <c r="DJ33" s="31">
-        <f>IF(OR(B33="",NOT(N($J$9)&gt;31)),0,IF(N(C33)&gt;0,C33,1)*(COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,MIN(62,N($J$9))),"FOC"))*N(E33))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,31+MAX(1,N($DE$9))),"S")+COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DK33" s="31">
-        <f>IF(OR(B33="",NOT(N($J$9)&gt;62)),0,IF(N(C33)&gt;0,C33,1)*((COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,MIN(93,N($J$9))),"S")+COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,MIN(93,N($J$9))),"MOB")+COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,MIN(93,N($J$9))),"DEMOB"))*N(D33)+(COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,MIN(93,N($J$9))),"O"))*N(E33)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,31+MAX(1,N($DE$9))),"O"))</f>
         <v/>
       </c>
       <c r="DL33" s="31">
-        <f>IF(OR(B33="",A33="Oui",DO33&lt;&gt;3),0,IF(N(C33)&gt;0,C33,1)*(N(F33)+N(H33)))</f>
+        <f>IF(N($DE$9)=0,0,COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,31+MAX(1,N($DE$9))),"MOB")+COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,31+MAX(1,N($DE$9))),"DEMOB"))</f>
         <v/>
       </c>
       <c r="DM33" s="31">
-        <f>IF(OR(B33="",NOT(N($J$9)&gt;62)),0,IF(N(C33)&gt;0,C33,1)*(IF((COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,MIN(93,N($J$9))),"VR"))&gt;0,N(G33),0)+IF((COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,MIN(93,N($J$9))),"RC"))&gt;0,N(I33),0)))</f>
+        <f>IF(B33="",0,IF(N(C33)&gt;0,C33,1)*(DJ33*N(D33)+DK33*N(E33)))</f>
         <v/>
       </c>
       <c r="DN33" s="31">
-        <f>IF(OR(B33="",NOT(N($J$9)&gt;62)),0,IF(N(C33)&gt;0,C33,1)*(COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,MIN(93,N($J$9))),"FOC"))*N(E33))</f>
+        <f>IF(OR(B33="",A33="Oui",DX33&lt;&gt;2),0,IF(N(C33)&gt;0,C33,1)*(N(F33)+N(H33)))</f>
         <v/>
       </c>
       <c r="DO33" s="31">
-        <f>IF(B33="",0,IFERROR(INT((MATCH("O",$M33:INDEX($M33:$DA33,MAX(1,N($J$9))),0)-1)/31)+1,0))</f>
+        <f>IF(OR(B33="",N($DE$9)=0),0,IF(N(C33)&gt;0,C33,1)*(IF((COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,31+MAX(1,N($DE$9))),"VR"))&gt;0,N(G33),0)+IF((COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,31+MAX(1,N($DE$9))),"RC"))&gt;0,N(I33),0)))</f>
+        <v/>
+      </c>
+      <c r="DP33" s="31">
+        <f>IF(OR(B33="",N($DE$9)=0),0,IF(N(C33)&gt;0,C33,1)*(COUNTIF(INDEX($M33:$DA33,32):INDEX($M33:$DA33,31+MAX(1,N($DE$9))),"FOC"))*N(E33))</f>
+        <v/>
+      </c>
+      <c r="DQ33" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,62+MAX(1,N($DF$9))),"S")+COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DR33" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,62+MAX(1,N($DF$9))),"O"))</f>
+        <v/>
+      </c>
+      <c r="DS33" s="31">
+        <f>IF(N($DF$9)=0,0,COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,62+MAX(1,N($DF$9))),"MOB")+COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,62+MAX(1,N($DF$9))),"DEMOB"))</f>
+        <v/>
+      </c>
+      <c r="DT33" s="31">
+        <f>IF(B33="",0,IF(N(C33)&gt;0,C33,1)*(DQ33*N(D33)+DR33*N(E33)))</f>
+        <v/>
+      </c>
+      <c r="DU33" s="31">
+        <f>IF(OR(B33="",A33="Oui",DX33&lt;&gt;3),0,IF(N(C33)&gt;0,C33,1)*(N(F33)+N(H33)))</f>
+        <v/>
+      </c>
+      <c r="DV33" s="31">
+        <f>IF(OR(B33="",N($DF$9)=0),0,IF(N(C33)&gt;0,C33,1)*(IF((COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,62+MAX(1,N($DF$9))),"VR"))&gt;0,N(G33),0)+IF((COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,62+MAX(1,N($DF$9))),"RC"))&gt;0,N(I33),0)))</f>
+        <v/>
+      </c>
+      <c r="DW33" s="31">
+        <f>IF(OR(B33="",N($DF$9)=0),0,IF(N(C33)&gt;0,C33,1)*(COUNTIF(INDEX($M33:$DA33,63):INDEX($M33:$DA33,62+MAX(1,N($DF$9))),"FOC"))*N(E33))</f>
+        <v/>
+      </c>
+      <c r="DX33" s="31">
+        <f>IF(B33="",0,IF(DD33&gt;0,1,IF(DK33&gt;0,2,IF(DR33&gt;0,3,0))))</f>
         <v/>
       </c>
     </row>
@@ -5204,6 +5814,33 @@
       <c r="DO36" s="31" t="n">
         <v>0</v>
       </c>
+      <c r="DP36" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DQ36" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DR36" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DS36" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT36" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU36" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV36" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW36" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX36" s="31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="23" t="n"/>
@@ -5353,6 +5990,33 @@
       <c r="DO37" s="31" t="n">
         <v>0</v>
       </c>
+      <c r="DP37" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DQ37" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DR37" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DS37" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT37" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU37" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV37" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW37" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX37" s="31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="23" t="n"/>
@@ -5502,6 +6166,33 @@
       <c r="DO38" s="31" t="n">
         <v>0</v>
       </c>
+      <c r="DP38" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DQ38" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DR38" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DS38" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT38" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU38" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV38" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW38" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX38" s="31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
@@ -5521,7 +6212,7 @@
       <c r="K41" s="1" t="n"/>
       <c r="L41" s="1" t="n"/>
       <c r="M41" s="20">
-        <f>IF(OR($C$9="",N($J$9)&lt;=0),"","FACTURATION DU BLOC "&amp;1&amp;" (hors transport et autres frais)")</f>
+        <f>IF(OR($C$9="",N($DD$9)=0),"","FACTURATION · "&amp;CHOOSE(MONTH($C$9),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR($C$9)&amp;"   (hors transport et autres frais)")</f>
         <v/>
       </c>
       <c r="N41" s="1" t="n"/>
@@ -5555,7 +6246,7 @@
       <c r="AP41" s="1" t="n"/>
       <c r="AQ41" s="1" t="n"/>
       <c r="AR41" s="20">
-        <f>IF(OR($C$9="",N($J$9)&lt;=31),"","FACTURATION DU BLOC "&amp;2&amp;" (hors transport et autres frais)")</f>
+        <f>IF(OR($C$9="",N($DE$9)=0),"","FACTURATION · "&amp;CHOOSE(MONTH(DATE(YEAR($C$9),MONTH($C$9)+1,1)),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR(DATE(YEAR($C$9),MONTH($C$9)+1,1))&amp;"   (hors transport et autres frais)")</f>
         <v/>
       </c>
       <c r="AS41" s="1" t="n"/>
@@ -5589,7 +6280,7 @@
       <c r="BU41" s="1" t="n"/>
       <c r="BV41" s="1" t="n"/>
       <c r="BW41" s="20">
-        <f>IF(OR($C$9="",N($J$9)&lt;=62),"","FACTURATION DU BLOC "&amp;3&amp;" (hors transport et autres frais)")</f>
+        <f>IF(OR($C$9="",N($DF$9)=0),"","FACTURATION · "&amp;CHOOSE(MONTH(DATE(YEAR($C$9),MONTH($C$9)+2,1)),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR(DATE(YEAR($C$9),MONTH($C$9)+2,1))&amp;"   (hors transport et autres frais)")</f>
         <v/>
       </c>
       <c r="BX41" s="1" t="n"/>
@@ -5643,7 +6334,7 @@
       <c r="J42" s="23" t="n"/>
       <c r="K42" s="23" t="n"/>
       <c r="L42" s="36">
-        <f>SUM(DC17:DC19)+SUM(DG17:DG19)+SUM(DK17:DK19)</f>
+        <f>SUM(DF17:DF19)+SUM(DM17:DM19)+SUM(DT17:DT19)</f>
         <v/>
       </c>
       <c r="M42" s="37" t="inlineStr">
@@ -5669,7 +6360,7 @@
       <c r="AC42" s="23" t="n"/>
       <c r="AD42" s="23" t="n"/>
       <c r="AE42" s="29">
-        <f>IF(N($J$9)&lt;=0,"",SUM(DC17:DC19))</f>
+        <f>IF(N($DD$9)=0,"",SUM(DF17:DF19))</f>
         <v/>
       </c>
       <c r="AF42" s="23" t="n"/>
@@ -5702,7 +6393,7 @@
       <c r="BH42" s="23" t="n"/>
       <c r="BI42" s="23" t="n"/>
       <c r="BJ42" s="29">
-        <f>IF(N($J$9)&lt;=31,"",SUM(DG17:DG19))</f>
+        <f>IF(N($DE$9)=0,"",SUM(DM17:DM19))</f>
         <v/>
       </c>
       <c r="BK42" s="23" t="n"/>
@@ -5735,7 +6426,7 @@
       <c r="CM42" s="23" t="n"/>
       <c r="CN42" s="23" t="n"/>
       <c r="CO42" s="29">
-        <f>IF(N($J$9)&lt;=62,"",SUM(DK17:DK19))</f>
+        <f>IF(N($DF$9)=0,"",SUM(DT17:DT19))</f>
         <v/>
       </c>
       <c r="CP42" s="23" t="n"/>
@@ -5766,7 +6457,7 @@
       <c r="J43" s="23" t="n"/>
       <c r="K43" s="23" t="n"/>
       <c r="L43" s="36">
-        <f>SUM(DD17:DD19)+SUM(DH17:DH19)+SUM(DL17:DL19)</f>
+        <f>SUM(DG17:DG19)+SUM(DN17:DN19)+SUM(DU17:DU19)</f>
         <v/>
       </c>
       <c r="M43" s="37" t="inlineStr">
@@ -5792,7 +6483,7 @@
       <c r="AC43" s="23" t="n"/>
       <c r="AD43" s="23" t="n"/>
       <c r="AE43" s="29">
-        <f>IF(N($J$9)&lt;=0,"",SUM(DD17:DD19))</f>
+        <f>IF(N($DD$9)=0,"",SUM(DG17:DG19))</f>
         <v/>
       </c>
       <c r="AF43" s="23" t="n"/>
@@ -5825,7 +6516,7 @@
       <c r="BH43" s="23" t="n"/>
       <c r="BI43" s="23" t="n"/>
       <c r="BJ43" s="29">
-        <f>IF(N($J$9)&lt;=31,"",SUM(DH17:DH19))</f>
+        <f>IF(N($DE$9)=0,"",SUM(DN17:DN19))</f>
         <v/>
       </c>
       <c r="BK43" s="23" t="n"/>
@@ -5858,7 +6549,7 @@
       <c r="CM43" s="23" t="n"/>
       <c r="CN43" s="23" t="n"/>
       <c r="CO43" s="29">
-        <f>IF(N($J$9)&lt;=62,"",SUM(DL17:DL19))</f>
+        <f>IF(N($DF$9)=0,"",SUM(DU17:DU19))</f>
         <v/>
       </c>
       <c r="CP43" s="23" t="n"/>
@@ -5890,7 +6581,7 @@
       <c r="J44" s="23" t="n"/>
       <c r="K44" s="23" t="n"/>
       <c r="L44" s="36">
-        <f>SUM(DC22:DC33)+SUM(DG22:DG33)+SUM(DK22:DK33)</f>
+        <f>SUM(DF22:DF33)+SUM(DM22:DM33)+SUM(DT22:DT33)</f>
         <v/>
       </c>
       <c r="M44" s="37" t="inlineStr">
@@ -5916,7 +6607,7 @@
       <c r="AC44" s="23" t="n"/>
       <c r="AD44" s="23" t="n"/>
       <c r="AE44" s="29">
-        <f>IF(N($J$9)&lt;=0,"",SUM(DC22:DC33))</f>
+        <f>IF(N($DD$9)=0,"",SUM(DF22:DF33))</f>
         <v/>
       </c>
       <c r="AF44" s="23" t="n"/>
@@ -5949,7 +6640,7 @@
       <c r="BH44" s="23" t="n"/>
       <c r="BI44" s="23" t="n"/>
       <c r="BJ44" s="29">
-        <f>IF(N($J$9)&lt;=31,"",SUM(DG22:DG33))</f>
+        <f>IF(N($DE$9)=0,"",SUM(DM22:DM33))</f>
         <v/>
       </c>
       <c r="BK44" s="23" t="n"/>
@@ -5982,7 +6673,7 @@
       <c r="CM44" s="23" t="n"/>
       <c r="CN44" s="23" t="n"/>
       <c r="CO44" s="29">
-        <f>IF(N($J$9)&lt;=62,"",SUM(DK22:DK33))</f>
+        <f>IF(N($DF$9)=0,"",SUM(DT22:DT33))</f>
         <v/>
       </c>
       <c r="CP44" s="23" t="n"/>
@@ -6014,7 +6705,7 @@
       <c r="J45" s="23" t="n"/>
       <c r="K45" s="23" t="n"/>
       <c r="L45" s="36">
-        <f>SUM(DD22:DD33)+SUM(DH22:DH33)+SUM(DL22:DL33)</f>
+        <f>SUM(DG22:DG33)+SUM(DN22:DN33)+SUM(DU22:DU33)</f>
         <v/>
       </c>
       <c r="M45" s="37" t="inlineStr">
@@ -6040,7 +6731,7 @@
       <c r="AC45" s="23" t="n"/>
       <c r="AD45" s="23" t="n"/>
       <c r="AE45" s="29">
-        <f>IF(N($J$9)&lt;=0,"",SUM(DD22:DD33))</f>
+        <f>IF(N($DD$9)=0,"",SUM(DG22:DG33))</f>
         <v/>
       </c>
       <c r="AF45" s="23" t="n"/>
@@ -6073,7 +6764,7 @@
       <c r="BH45" s="23" t="n"/>
       <c r="BI45" s="23" t="n"/>
       <c r="BJ45" s="29">
-        <f>IF(N($J$9)&lt;=31,"",SUM(DH22:DH33))</f>
+        <f>IF(N($DE$9)=0,"",SUM(DN22:DN33))</f>
         <v/>
       </c>
       <c r="BK45" s="23" t="n"/>
@@ -6106,7 +6797,7 @@
       <c r="CM45" s="23" t="n"/>
       <c r="CN45" s="23" t="n"/>
       <c r="CO45" s="29">
-        <f>IF(N($J$9)&lt;=62,"",SUM(DL22:DL33))</f>
+        <f>IF(N($DF$9)=0,"",SUM(DU22:DU33))</f>
         <v/>
       </c>
       <c r="CP45" s="23" t="n"/>
@@ -6134,7 +6825,7 @@
       <c r="J46" s="23" t="n"/>
       <c r="K46" s="23" t="n"/>
       <c r="L46" s="36">
-        <f>SUM(DE22:DE33)+SUM(DI22:DI33)+SUM(DM22:DM33)</f>
+        <f>SUM(DH22:DH33)+SUM(DO22:DO33)+SUM(DV22:DV33)</f>
         <v/>
       </c>
       <c r="M46" s="37" t="inlineStr">
@@ -6160,7 +6851,7 @@
       <c r="AC46" s="23" t="n"/>
       <c r="AD46" s="23" t="n"/>
       <c r="AE46" s="29">
-        <f>IF(N($J$9)&lt;=0,"",SUM(DE22:DE33))</f>
+        <f>IF(N($DD$9)=0,"",SUM(DH22:DH33))</f>
         <v/>
       </c>
       <c r="AF46" s="23" t="n"/>
@@ -6193,7 +6884,7 @@
       <c r="BH46" s="23" t="n"/>
       <c r="BI46" s="23" t="n"/>
       <c r="BJ46" s="29">
-        <f>IF(N($J$9)&lt;=31,"",SUM(DI22:DI33))</f>
+        <f>IF(N($DE$9)=0,"",SUM(DO22:DO33))</f>
         <v/>
       </c>
       <c r="BK46" s="23" t="n"/>
@@ -6226,7 +6917,7 @@
       <c r="CM46" s="23" t="n"/>
       <c r="CN46" s="23" t="n"/>
       <c r="CO46" s="29">
-        <f>IF(N($J$9)&lt;=62,"",SUM(DM22:DM33))</f>
+        <f>IF(N($DF$9)=0,"",SUM(DV22:DV33))</f>
         <v/>
       </c>
       <c r="CP46" s="23" t="n"/>
@@ -6283,7 +6974,7 @@
         <v/>
       </c>
       <c r="M48" s="41">
-        <f>"TOTAL DU BLOC "&amp;1</f>
+        <f>IF(N($DD$9)=0,"","TOTAL À FACTURER · "&amp;CHOOSE(MONTH($C$9),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR($C$9))</f>
         <v/>
       </c>
       <c r="N48" s="42" t="n"/>
@@ -6304,7 +6995,7 @@
       <c r="AC48" s="42" t="n"/>
       <c r="AD48" s="42" t="n"/>
       <c r="AE48" s="43">
-        <f>IF(N($J$9)&lt;=0,"",SUM(AE42:AE46))</f>
+        <f>IF(N($DD$9)=0,"",SUM(AE42:AE46))</f>
         <v/>
       </c>
       <c r="AF48" s="42" t="n"/>
@@ -6315,7 +7006,7 @@
       <c r="AK48" s="42" t="n"/>
       <c r="AL48" s="42" t="n"/>
       <c r="AR48" s="41">
-        <f>"TOTAL DU BLOC "&amp;2</f>
+        <f>IF(N($DE$9)=0,"","TOTAL À FACTURER · "&amp;CHOOSE(MONTH(DATE(YEAR($C$9),MONTH($C$9)+1,1)),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR(DATE(YEAR($C$9),MONTH($C$9)+1,1)))</f>
         <v/>
       </c>
       <c r="AS48" s="42" t="n"/>
@@ -6336,7 +7027,7 @@
       <c r="BH48" s="42" t="n"/>
       <c r="BI48" s="42" t="n"/>
       <c r="BJ48" s="43">
-        <f>IF(N($J$9)&lt;=31,"",SUM(BJ42:BJ46))</f>
+        <f>IF(N($DE$9)=0,"",SUM(BJ42:BJ46))</f>
         <v/>
       </c>
       <c r="BK48" s="42" t="n"/>
@@ -6347,7 +7038,7 @@
       <c r="BP48" s="42" t="n"/>
       <c r="BQ48" s="42" t="n"/>
       <c r="BW48" s="41">
-        <f>"TOTAL DU BLOC "&amp;3</f>
+        <f>IF(N($DF$9)=0,"","TOTAL À FACTURER · "&amp;CHOOSE(MONTH(DATE(YEAR($C$9),MONTH($C$9)+2,1)),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR(DATE(YEAR($C$9),MONTH($C$9)+2,1)))</f>
         <v/>
       </c>
       <c r="BX48" s="42" t="n"/>
@@ -6368,7 +7059,7 @@
       <c r="CM48" s="42" t="n"/>
       <c r="CN48" s="42" t="n"/>
       <c r="CO48" s="43">
-        <f>IF(N($J$9)&lt;=62,"",SUM(CO42:CO46))</f>
+        <f>IF(N($DF$9)=0,"",SUM(CO42:CO46))</f>
         <v/>
       </c>
       <c r="CP48" s="42" t="n"/>
@@ -6386,7 +7077,7 @@
         </is>
       </c>
       <c r="L49" s="45">
-        <f>SUM(DF22:DF33)+SUM(DJ22:DJ33)+SUM(DN22:DN33)</f>
+        <f>SUM(DI22:DI33)+SUM(DP22:DP33)+SUM(DW22:DW33)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Service ticket : codes DEMOB et VR lisibles dans le calendrier
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/service_ticket_2027/Service_Ticket_Enedril_2027.xlsx
+++ b/service_ticket_2027/Service_Ticket_Enedril_2027.xlsx
@@ -105,7 +105,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="000B1B2E"/>
-      <sz val="8.5"/>
+      <sz val="7.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -367,7 +367,7 @@
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -941,39 +941,39 @@
     <col width="5" customWidth="1" min="10" max="10"/>
     <col width="5" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="3.3" customWidth="1" min="13" max="13"/>
-    <col width="3.3" customWidth="1" min="14" max="14"/>
-    <col width="3.3" customWidth="1" min="15" max="15"/>
-    <col width="3.3" customWidth="1" min="16" max="16"/>
-    <col width="3.3" customWidth="1" min="17" max="17"/>
-    <col width="3.3" customWidth="1" min="18" max="18"/>
-    <col width="3.3" customWidth="1" min="19" max="19"/>
-    <col width="3.3" customWidth="1" min="20" max="20"/>
-    <col width="3.3" customWidth="1" min="21" max="21"/>
-    <col width="3.3" customWidth="1" min="22" max="22"/>
-    <col width="3.3" customWidth="1" min="23" max="23"/>
-    <col width="3.3" customWidth="1" min="24" max="24"/>
-    <col width="3.3" customWidth="1" min="25" max="25"/>
-    <col width="3.3" customWidth="1" min="26" max="26"/>
-    <col width="3.3" customWidth="1" min="27" max="27"/>
-    <col width="3.3" customWidth="1" min="28" max="28"/>
-    <col width="3.3" customWidth="1" min="29" max="29"/>
-    <col width="3.3" customWidth="1" min="30" max="30"/>
-    <col width="3.3" customWidth="1" min="31" max="31"/>
-    <col width="3.3" customWidth="1" min="32" max="32"/>
-    <col width="3.3" customWidth="1" min="33" max="33"/>
-    <col width="3.3" customWidth="1" min="34" max="34"/>
-    <col width="3.3" customWidth="1" min="35" max="35"/>
-    <col width="3.3" customWidth="1" min="36" max="36"/>
-    <col width="3.3" customWidth="1" min="37" max="37"/>
-    <col width="3.3" customWidth="1" min="38" max="38"/>
-    <col width="3.3" customWidth="1" min="39" max="39"/>
-    <col width="3.3" customWidth="1" min="40" max="40"/>
-    <col width="3.3" customWidth="1" min="41" max="41"/>
-    <col width="3.3" customWidth="1" min="42" max="42"/>
-    <col width="3.3" customWidth="1" min="43" max="43"/>
-    <col hidden="1" outlineLevel="1" width="3.3" customWidth="1" min="44" max="74"/>
-    <col hidden="1" outlineLevel="1" width="3.3" customWidth="1" min="75" max="105"/>
+    <col width="4.2" customWidth="1" min="13" max="13"/>
+    <col width="4.2" customWidth="1" min="14" max="14"/>
+    <col width="4.2" customWidth="1" min="15" max="15"/>
+    <col width="4.2" customWidth="1" min="16" max="16"/>
+    <col width="4.2" customWidth="1" min="17" max="17"/>
+    <col width="4.2" customWidth="1" min="18" max="18"/>
+    <col width="4.2" customWidth="1" min="19" max="19"/>
+    <col width="4.2" customWidth="1" min="20" max="20"/>
+    <col width="4.2" customWidth="1" min="21" max="21"/>
+    <col width="4.2" customWidth="1" min="22" max="22"/>
+    <col width="4.2" customWidth="1" min="23" max="23"/>
+    <col width="4.2" customWidth="1" min="24" max="24"/>
+    <col width="4.2" customWidth="1" min="25" max="25"/>
+    <col width="4.2" customWidth="1" min="26" max="26"/>
+    <col width="4.2" customWidth="1" min="27" max="27"/>
+    <col width="4.2" customWidth="1" min="28" max="28"/>
+    <col width="4.2" customWidth="1" min="29" max="29"/>
+    <col width="4.2" customWidth="1" min="30" max="30"/>
+    <col width="4.2" customWidth="1" min="31" max="31"/>
+    <col width="4.2" customWidth="1" min="32" max="32"/>
+    <col width="4.2" customWidth="1" min="33" max="33"/>
+    <col width="4.2" customWidth="1" min="34" max="34"/>
+    <col width="4.2" customWidth="1" min="35" max="35"/>
+    <col width="4.2" customWidth="1" min="36" max="36"/>
+    <col width="4.2" customWidth="1" min="37" max="37"/>
+    <col width="4.2" customWidth="1" min="38" max="38"/>
+    <col width="4.2" customWidth="1" min="39" max="39"/>
+    <col width="4.2" customWidth="1" min="40" max="40"/>
+    <col width="4.2" customWidth="1" min="41" max="41"/>
+    <col width="4.2" customWidth="1" min="42" max="42"/>
+    <col width="4.2" customWidth="1" min="43" max="43"/>
+    <col hidden="1" outlineLevel="1" width="4.2" customWidth="1" min="44" max="74"/>
+    <col hidden="1" outlineLevel="1" width="4.2" customWidth="1" min="75" max="105"/>
     <col width="1.5" customWidth="1" min="106" max="106"/>
     <col hidden="1" width="13" customWidth="1" min="107" max="107"/>
     <col hidden="1" width="13" customWidth="1" min="108" max="108"/>
@@ -7267,7 +7267,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.3" right="0.3" top="0.35" bottom="0.4" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" scale="56"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="52"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;C&amp;8 Enedril · Service ticket · &amp;P / &amp;N</oddFooter>

</xml_diff>

<commit_message>
Service ticket : serrages (nombre par jour, prix par serrage, facturation par mois)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/service_ticket_2027/Service_Ticket_Enedril_2027.xlsx
+++ b/service_ticket_2027/Service_Ticket_Enedril_2027.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Service ticket'!$A:$L</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Service ticket'!$A$1:$DA$53</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Service ticket'!$A$1:$DA$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -295,7 +295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -371,6 +371,9 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -926,7 +929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DX53"/>
+  <dimension ref="A1:EA58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -997,6 +1000,9 @@
     <col hidden="1" width="13" customWidth="1" min="126" max="126"/>
     <col hidden="1" width="13" customWidth="1" min="127" max="127"/>
     <col hidden="1" width="13" customWidth="1" min="128" max="128"/>
+    <col hidden="1" width="13" customWidth="1" min="129" max="129"/>
+    <col hidden="1" width="13" customWidth="1" min="130" max="130"/>
+    <col hidden="1" width="13" customWidth="1" min="131" max="131"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -2595,6 +2601,15 @@
       <c r="DX17" s="31" t="n">
         <v>0</v>
       </c>
+      <c r="DY17" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DZ17" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="EA17" s="31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="23" t="n"/>
@@ -2795,6 +2810,15 @@
       <c r="DX18" s="31" t="n">
         <v>0</v>
       </c>
+      <c r="DY18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DZ18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="EA18" s="31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="23" t="n"/>
@@ -2993,6 +3017,15 @@
         <v>0</v>
       </c>
       <c r="DX19" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY19" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DZ19" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="EA19" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3310,6 +3343,9 @@
         <f>IF(B22="",0,IF(DD22&gt;0,1,IF(DK22&gt;0,2,IF(DR22&gt;0,3,0))))</f>
         <v/>
       </c>
+      <c r="DY22" s="31" t="n"/>
+      <c r="DZ22" s="31" t="n"/>
+      <c r="EA22" s="31" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="32" t="n"/>
@@ -3514,6 +3550,9 @@
         <f>IF(B23="",0,IF(DD23&gt;0,1,IF(DK23&gt;0,2,IF(DR23&gt;0,3,0))))</f>
         <v/>
       </c>
+      <c r="DY23" s="31" t="n"/>
+      <c r="DZ23" s="31" t="n"/>
+      <c r="EA23" s="31" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="32" t="n"/>
@@ -3718,6 +3757,9 @@
         <f>IF(B24="",0,IF(DD24&gt;0,1,IF(DK24&gt;0,2,IF(DR24&gt;0,3,0))))</f>
         <v/>
       </c>
+      <c r="DY24" s="31" t="n"/>
+      <c r="DZ24" s="31" t="n"/>
+      <c r="EA24" s="31" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="32" t="n"/>
@@ -3922,6 +3964,9 @@
         <f>IF(B25="",0,IF(DD25&gt;0,1,IF(DK25&gt;0,2,IF(DR25&gt;0,3,0))))</f>
         <v/>
       </c>
+      <c r="DY25" s="31" t="n"/>
+      <c r="DZ25" s="31" t="n"/>
+      <c r="EA25" s="31" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="32" t="n"/>
@@ -4126,6 +4171,9 @@
         <f>IF(B26="",0,IF(DD26&gt;0,1,IF(DK26&gt;0,2,IF(DR26&gt;0,3,0))))</f>
         <v/>
       </c>
+      <c r="DY26" s="31" t="n"/>
+      <c r="DZ26" s="31" t="n"/>
+      <c r="EA26" s="31" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="32" t="n"/>
@@ -4330,6 +4378,9 @@
         <f>IF(B27="",0,IF(DD27&gt;0,1,IF(DK27&gt;0,2,IF(DR27&gt;0,3,0))))</f>
         <v/>
       </c>
+      <c r="DY27" s="31" t="n"/>
+      <c r="DZ27" s="31" t="n"/>
+      <c r="EA27" s="31" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="32" t="n"/>
@@ -4534,6 +4585,9 @@
         <f>IF(B28="",0,IF(DD28&gt;0,1,IF(DK28&gt;0,2,IF(DR28&gt;0,3,0))))</f>
         <v/>
       </c>
+      <c r="DY28" s="31" t="n"/>
+      <c r="DZ28" s="31" t="n"/>
+      <c r="EA28" s="31" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="32" t="n"/>
@@ -4738,6 +4792,9 @@
         <f>IF(B29="",0,IF(DD29&gt;0,1,IF(DK29&gt;0,2,IF(DR29&gt;0,3,0))))</f>
         <v/>
       </c>
+      <c r="DY29" s="31" t="n"/>
+      <c r="DZ29" s="31" t="n"/>
+      <c r="EA29" s="31" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="32" t="n"/>
@@ -4942,6 +4999,9 @@
         <f>IF(B30="",0,IF(DD30&gt;0,1,IF(DK30&gt;0,2,IF(DR30&gt;0,3,0))))</f>
         <v/>
       </c>
+      <c r="DY30" s="31" t="n"/>
+      <c r="DZ30" s="31" t="n"/>
+      <c r="EA30" s="31" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="32" t="n"/>
@@ -5146,6 +5206,9 @@
         <f>IF(B31="",0,IF(DD31&gt;0,1,IF(DK31&gt;0,2,IF(DR31&gt;0,3,0))))</f>
         <v/>
       </c>
+      <c r="DY31" s="31" t="n"/>
+      <c r="DZ31" s="31" t="n"/>
+      <c r="EA31" s="31" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="32" t="n"/>
@@ -5350,6 +5413,9 @@
         <f>IF(B32="",0,IF(DD32&gt;0,1,IF(DK32&gt;0,2,IF(DR32&gt;0,3,0))))</f>
         <v/>
       </c>
+      <c r="DY32" s="31" t="n"/>
+      <c r="DZ32" s="31" t="n"/>
+      <c r="EA32" s="31" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="32" t="n"/>
@@ -5554,11 +5620,14 @@
         <f>IF(B33="",0,IF(DD33&gt;0,1,IF(DK33&gt;0,2,IF(DR33&gt;0,3,0))))</f>
         <v/>
       </c>
+      <c r="DY33" s="31" t="n"/>
+      <c r="DZ33" s="31" t="n"/>
+      <c r="EA33" s="31" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>TRANSPORT ET AUTRES FRAIS   ·   quantité × prix unitaire (colonne « Opér. € »)</t>
+          <t>SERRAGES   ·   saisir dans le calendrier le nombre de serrages effectués chaque jour   ·   prix par serrage en colonne « Opér. € »</t>
         </is>
       </c>
       <c r="B35" s="1" t="n"/>
@@ -5669,17 +5738,20 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="23" t="n"/>
       <c r="B36" s="24" t="n"/>
-      <c r="C36" s="32" t="n"/>
+      <c r="C36" s="23" t="n"/>
       <c r="D36" s="26" t="n"/>
       <c r="E36" s="25" t="n"/>
       <c r="F36" s="26" t="n"/>
       <c r="G36" s="26" t="n"/>
       <c r="H36" s="26" t="n"/>
       <c r="I36" s="26" t="n"/>
-      <c r="J36" s="28" t="n"/>
+      <c r="J36" s="28">
+        <f>IF(B36="","",SUM(INDEX($M36:$DA36,1):INDEX($M36:$DA36,0+MAX(1,N($DD$9))))+SUM(INDEX($M36:$DA36,32):INDEX($M36:$DA36,31+MAX(1,N($DE$9))))+SUM(INDEX($M36:$DA36,63):INDEX($M36:$DA36,62+MAX(1,N($DF$9)))))</f>
+        <v/>
+      </c>
       <c r="K36" s="28" t="n"/>
       <c r="L36" s="29">
-        <f>IF(B36="","",N(C36)*N(E36))</f>
+        <f>IF(B36="","",DY36+DZ36+EA36)</f>
         <v/>
       </c>
       <c r="M36" s="33" t="n"/>
@@ -5841,21 +5913,36 @@
       <c r="DX36" s="31" t="n">
         <v>0</v>
       </c>
+      <c r="DY36" s="31">
+        <f>IF(OR(B36="",N($DD$9)=0),0,SUM(INDEX($M36:$DA36,1):INDEX($M36:$DA36,0+MAX(1,N($DD$9))))*N(E36))</f>
+        <v/>
+      </c>
+      <c r="DZ36" s="31">
+        <f>IF(OR(B36="",N($DE$9)=0),0,SUM(INDEX($M36:$DA36,32):INDEX($M36:$DA36,31+MAX(1,N($DE$9))))*N(E36))</f>
+        <v/>
+      </c>
+      <c r="EA36" s="31">
+        <f>IF(OR(B36="",N($DF$9)=0),0,SUM(INDEX($M36:$DA36,63):INDEX($M36:$DA36,62+MAX(1,N($DF$9))))*N(E36))</f>
+        <v/>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="23" t="n"/>
       <c r="B37" s="24" t="n"/>
-      <c r="C37" s="32" t="n"/>
+      <c r="C37" s="23" t="n"/>
       <c r="D37" s="26" t="n"/>
       <c r="E37" s="25" t="n"/>
       <c r="F37" s="26" t="n"/>
       <c r="G37" s="26" t="n"/>
       <c r="H37" s="26" t="n"/>
       <c r="I37" s="26" t="n"/>
-      <c r="J37" s="28" t="n"/>
+      <c r="J37" s="28">
+        <f>IF(B37="","",SUM(INDEX($M37:$DA37,1):INDEX($M37:$DA37,0+MAX(1,N($DD$9))))+SUM(INDEX($M37:$DA37,32):INDEX($M37:$DA37,31+MAX(1,N($DE$9))))+SUM(INDEX($M37:$DA37,63):INDEX($M37:$DA37,62+MAX(1,N($DF$9)))))</f>
+        <v/>
+      </c>
       <c r="K37" s="28" t="n"/>
       <c r="L37" s="29">
-        <f>IF(B37="","",N(C37)*N(E37))</f>
+        <f>IF(B37="","",DY37+DZ37+EA37)</f>
         <v/>
       </c>
       <c r="M37" s="33" t="n"/>
@@ -6017,820 +6104,831 @@
       <c r="DX37" s="31" t="n">
         <v>0</v>
       </c>
+      <c r="DY37" s="31">
+        <f>IF(OR(B37="",N($DD$9)=0),0,SUM(INDEX($M37:$DA37,1):INDEX($M37:$DA37,0+MAX(1,N($DD$9))))*N(E37))</f>
+        <v/>
+      </c>
+      <c r="DZ37" s="31">
+        <f>IF(OR(B37="",N($DE$9)=0),0,SUM(INDEX($M37:$DA37,32):INDEX($M37:$DA37,31+MAX(1,N($DE$9))))*N(E37))</f>
+        <v/>
+      </c>
+      <c r="EA37" s="31">
+        <f>IF(OR(B37="",N($DF$9)=0),0,SUM(INDEX($M37:$DA37,63):INDEX($M37:$DA37,62+MAX(1,N($DF$9))))*N(E37))</f>
+        <v/>
+      </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="23" t="n"/>
-      <c r="B38" s="24" t="n"/>
-      <c r="C38" s="32" t="n"/>
-      <c r="D38" s="26" t="n"/>
-      <c r="E38" s="25" t="n"/>
-      <c r="F38" s="26" t="n"/>
-      <c r="G38" s="26" t="n"/>
-      <c r="H38" s="26" t="n"/>
-      <c r="I38" s="26" t="n"/>
-      <c r="J38" s="28" t="n"/>
-      <c r="K38" s="28" t="n"/>
-      <c r="L38" s="29">
-        <f>IF(B38="","",N(C38)*N(E38))</f>
-        <v/>
-      </c>
-      <c r="M38" s="33" t="n"/>
-      <c r="N38" s="33" t="n"/>
-      <c r="O38" s="33" t="n"/>
-      <c r="P38" s="33" t="n"/>
-      <c r="Q38" s="33" t="n"/>
-      <c r="R38" s="33" t="n"/>
-      <c r="S38" s="33" t="n"/>
-      <c r="T38" s="33" t="n"/>
-      <c r="U38" s="33" t="n"/>
-      <c r="V38" s="33" t="n"/>
-      <c r="W38" s="33" t="n"/>
-      <c r="X38" s="33" t="n"/>
-      <c r="Y38" s="33" t="n"/>
-      <c r="Z38" s="33" t="n"/>
-      <c r="AA38" s="33" t="n"/>
-      <c r="AB38" s="33" t="n"/>
-      <c r="AC38" s="33" t="n"/>
-      <c r="AD38" s="33" t="n"/>
-      <c r="AE38" s="33" t="n"/>
-      <c r="AF38" s="33" t="n"/>
-      <c r="AG38" s="33" t="n"/>
-      <c r="AH38" s="33" t="n"/>
-      <c r="AI38" s="33" t="n"/>
-      <c r="AJ38" s="33" t="n"/>
-      <c r="AK38" s="33" t="n"/>
-      <c r="AL38" s="33" t="n"/>
-      <c r="AM38" s="33" t="n"/>
-      <c r="AN38" s="33" t="n"/>
-      <c r="AO38" s="33" t="n"/>
-      <c r="AP38" s="33" t="n"/>
-      <c r="AQ38" s="33" t="n"/>
-      <c r="AR38" s="33" t="n"/>
-      <c r="AS38" s="33" t="n"/>
-      <c r="AT38" s="33" t="n"/>
-      <c r="AU38" s="33" t="n"/>
-      <c r="AV38" s="33" t="n"/>
-      <c r="AW38" s="33" t="n"/>
-      <c r="AX38" s="33" t="n"/>
-      <c r="AY38" s="33" t="n"/>
-      <c r="AZ38" s="33" t="n"/>
-      <c r="BA38" s="33" t="n"/>
-      <c r="BB38" s="33" t="n"/>
-      <c r="BC38" s="33" t="n"/>
-      <c r="BD38" s="33" t="n"/>
-      <c r="BE38" s="33" t="n"/>
-      <c r="BF38" s="33" t="n"/>
-      <c r="BG38" s="33" t="n"/>
-      <c r="BH38" s="33" t="n"/>
-      <c r="BI38" s="33" t="n"/>
-      <c r="BJ38" s="33" t="n"/>
-      <c r="BK38" s="33" t="n"/>
-      <c r="BL38" s="33" t="n"/>
-      <c r="BM38" s="33" t="n"/>
-      <c r="BN38" s="33" t="n"/>
-      <c r="BO38" s="33" t="n"/>
-      <c r="BP38" s="33" t="n"/>
-      <c r="BQ38" s="33" t="n"/>
-      <c r="BR38" s="33" t="n"/>
-      <c r="BS38" s="33" t="n"/>
-      <c r="BT38" s="33" t="n"/>
-      <c r="BU38" s="33" t="n"/>
-      <c r="BV38" s="33" t="n"/>
-      <c r="BW38" s="33" t="n"/>
-      <c r="BX38" s="33" t="n"/>
-      <c r="BY38" s="33" t="n"/>
-      <c r="BZ38" s="33" t="n"/>
-      <c r="CA38" s="33" t="n"/>
-      <c r="CB38" s="33" t="n"/>
-      <c r="CC38" s="33" t="n"/>
-      <c r="CD38" s="33" t="n"/>
-      <c r="CE38" s="33" t="n"/>
-      <c r="CF38" s="33" t="n"/>
-      <c r="CG38" s="33" t="n"/>
-      <c r="CH38" s="33" t="n"/>
-      <c r="CI38" s="33" t="n"/>
-      <c r="CJ38" s="33" t="n"/>
-      <c r="CK38" s="33" t="n"/>
-      <c r="CL38" s="33" t="n"/>
-      <c r="CM38" s="33" t="n"/>
-      <c r="CN38" s="33" t="n"/>
-      <c r="CO38" s="33" t="n"/>
-      <c r="CP38" s="33" t="n"/>
-      <c r="CQ38" s="33" t="n"/>
-      <c r="CR38" s="33" t="n"/>
-      <c r="CS38" s="33" t="n"/>
-      <c r="CT38" s="33" t="n"/>
-      <c r="CU38" s="33" t="n"/>
-      <c r="CV38" s="33" t="n"/>
-      <c r="CW38" s="33" t="n"/>
-      <c r="CX38" s="33" t="n"/>
-      <c r="CY38" s="33" t="n"/>
-      <c r="CZ38" s="33" t="n"/>
-      <c r="DA38" s="33" t="n"/>
-      <c r="DC38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DD38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DE38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DF38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DG38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DH38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DI38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DJ38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DK38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DL38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DM38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DN38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DO38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DP38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DQ38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DR38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DS38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DT38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DU38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DV38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DW38" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="DX38" s="31" t="n">
-        <v>0</v>
-      </c>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
+          <t>TRANSPORT ET AUTRES FRAIS   ·   quantité × prix unitaire (colonne « Opér. € »)</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="n"/>
+      <c r="C39" s="1" t="n"/>
+      <c r="D39" s="1" t="n"/>
+      <c r="E39" s="1" t="n"/>
+      <c r="F39" s="1" t="n"/>
+      <c r="G39" s="1" t="n"/>
+      <c r="H39" s="1" t="n"/>
+      <c r="I39" s="1" t="n"/>
+      <c r="J39" s="1" t="n"/>
+      <c r="K39" s="1" t="n"/>
+      <c r="L39" s="1" t="n"/>
+      <c r="M39" s="1" t="n"/>
+      <c r="N39" s="1" t="n"/>
+      <c r="O39" s="1" t="n"/>
+      <c r="P39" s="1" t="n"/>
+      <c r="Q39" s="1" t="n"/>
+      <c r="R39" s="1" t="n"/>
+      <c r="S39" s="1" t="n"/>
+      <c r="T39" s="1" t="n"/>
+      <c r="U39" s="1" t="n"/>
+      <c r="V39" s="1" t="n"/>
+      <c r="W39" s="1" t="n"/>
+      <c r="X39" s="1" t="n"/>
+      <c r="Y39" s="1" t="n"/>
+      <c r="Z39" s="1" t="n"/>
+      <c r="AA39" s="1" t="n"/>
+      <c r="AB39" s="1" t="n"/>
+      <c r="AC39" s="1" t="n"/>
+      <c r="AD39" s="1" t="n"/>
+      <c r="AE39" s="1" t="n"/>
+      <c r="AF39" s="1" t="n"/>
+      <c r="AG39" s="1" t="n"/>
+      <c r="AH39" s="1" t="n"/>
+      <c r="AI39" s="1" t="n"/>
+      <c r="AJ39" s="1" t="n"/>
+      <c r="AK39" s="1" t="n"/>
+      <c r="AL39" s="1" t="n"/>
+      <c r="AM39" s="1" t="n"/>
+      <c r="AN39" s="1" t="n"/>
+      <c r="AO39" s="1" t="n"/>
+      <c r="AP39" s="1" t="n"/>
+      <c r="AQ39" s="1" t="n"/>
+      <c r="AR39" s="1" t="n"/>
+      <c r="AS39" s="1" t="n"/>
+      <c r="AT39" s="1" t="n"/>
+      <c r="AU39" s="1" t="n"/>
+      <c r="AV39" s="1" t="n"/>
+      <c r="AW39" s="1" t="n"/>
+      <c r="AX39" s="1" t="n"/>
+      <c r="AY39" s="1" t="n"/>
+      <c r="AZ39" s="1" t="n"/>
+      <c r="BA39" s="1" t="n"/>
+      <c r="BB39" s="1" t="n"/>
+      <c r="BC39" s="1" t="n"/>
+      <c r="BD39" s="1" t="n"/>
+      <c r="BE39" s="1" t="n"/>
+      <c r="BF39" s="1" t="n"/>
+      <c r="BG39" s="1" t="n"/>
+      <c r="BH39" s="1" t="n"/>
+      <c r="BI39" s="1" t="n"/>
+      <c r="BJ39" s="1" t="n"/>
+      <c r="BK39" s="1" t="n"/>
+      <c r="BL39" s="1" t="n"/>
+      <c r="BM39" s="1" t="n"/>
+      <c r="BN39" s="1" t="n"/>
+      <c r="BO39" s="1" t="n"/>
+      <c r="BP39" s="1" t="n"/>
+      <c r="BQ39" s="1" t="n"/>
+      <c r="BR39" s="1" t="n"/>
+      <c r="BS39" s="1" t="n"/>
+      <c r="BT39" s="1" t="n"/>
+      <c r="BU39" s="1" t="n"/>
+      <c r="BV39" s="1" t="n"/>
+      <c r="BW39" s="1" t="n"/>
+      <c r="BX39" s="1" t="n"/>
+      <c r="BY39" s="1" t="n"/>
+      <c r="BZ39" s="1" t="n"/>
+      <c r="CA39" s="1" t="n"/>
+      <c r="CB39" s="1" t="n"/>
+      <c r="CC39" s="1" t="n"/>
+      <c r="CD39" s="1" t="n"/>
+      <c r="CE39" s="1" t="n"/>
+      <c r="CF39" s="1" t="n"/>
+      <c r="CG39" s="1" t="n"/>
+      <c r="CH39" s="1" t="n"/>
+      <c r="CI39" s="1" t="n"/>
+      <c r="CJ39" s="1" t="n"/>
+      <c r="CK39" s="1" t="n"/>
+      <c r="CL39" s="1" t="n"/>
+      <c r="CM39" s="1" t="n"/>
+      <c r="CN39" s="1" t="n"/>
+      <c r="CO39" s="1" t="n"/>
+      <c r="CP39" s="1" t="n"/>
+      <c r="CQ39" s="1" t="n"/>
+      <c r="CR39" s="1" t="n"/>
+      <c r="CS39" s="1" t="n"/>
+      <c r="CT39" s="1" t="n"/>
+      <c r="CU39" s="1" t="n"/>
+      <c r="CV39" s="1" t="n"/>
+      <c r="CW39" s="1" t="n"/>
+      <c r="CX39" s="1" t="n"/>
+      <c r="CY39" s="1" t="n"/>
+      <c r="CZ39" s="1" t="n"/>
+      <c r="DA39" s="1" t="n"/>
     </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="20" t="inlineStr">
-        <is>
-          <t>RÉCAPITULATIF</t>
-        </is>
-      </c>
-      <c r="B41" s="1" t="n"/>
-      <c r="C41" s="1" t="n"/>
-      <c r="D41" s="1" t="n"/>
-      <c r="E41" s="1" t="n"/>
-      <c r="F41" s="1" t="n"/>
-      <c r="G41" s="1" t="n"/>
-      <c r="H41" s="1" t="n"/>
-      <c r="I41" s="1" t="n"/>
-      <c r="J41" s="1" t="n"/>
-      <c r="K41" s="1" t="n"/>
-      <c r="L41" s="1" t="n"/>
-      <c r="M41" s="20">
-        <f>IF(OR($C$9="",N($DD$9)=0),"","FACTURATION · "&amp;CHOOSE(MONTH($C$9),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR($C$9)&amp;"   (hors transport et autres frais)")</f>
-        <v/>
-      </c>
-      <c r="N41" s="1" t="n"/>
-      <c r="O41" s="1" t="n"/>
-      <c r="P41" s="1" t="n"/>
-      <c r="Q41" s="1" t="n"/>
-      <c r="R41" s="1" t="n"/>
-      <c r="S41" s="1" t="n"/>
-      <c r="T41" s="1" t="n"/>
-      <c r="U41" s="1" t="n"/>
-      <c r="V41" s="1" t="n"/>
-      <c r="W41" s="1" t="n"/>
-      <c r="X41" s="1" t="n"/>
-      <c r="Y41" s="1" t="n"/>
-      <c r="Z41" s="1" t="n"/>
-      <c r="AA41" s="1" t="n"/>
-      <c r="AB41" s="1" t="n"/>
-      <c r="AC41" s="1" t="n"/>
-      <c r="AD41" s="1" t="n"/>
-      <c r="AE41" s="1" t="n"/>
-      <c r="AF41" s="1" t="n"/>
-      <c r="AG41" s="1" t="n"/>
-      <c r="AH41" s="1" t="n"/>
-      <c r="AI41" s="1" t="n"/>
-      <c r="AJ41" s="1" t="n"/>
-      <c r="AK41" s="1" t="n"/>
-      <c r="AL41" s="1" t="n"/>
-      <c r="AM41" s="1" t="n"/>
-      <c r="AN41" s="1" t="n"/>
-      <c r="AO41" s="1" t="n"/>
-      <c r="AP41" s="1" t="n"/>
-      <c r="AQ41" s="1" t="n"/>
-      <c r="AR41" s="20">
-        <f>IF(OR($C$9="",N($DE$9)=0),"","FACTURATION · "&amp;CHOOSE(MONTH(DATE(YEAR($C$9),MONTH($C$9)+1,1)),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR(DATE(YEAR($C$9),MONTH($C$9)+1,1))&amp;"   (hors transport et autres frais)")</f>
-        <v/>
-      </c>
-      <c r="AS41" s="1" t="n"/>
-      <c r="AT41" s="1" t="n"/>
-      <c r="AU41" s="1" t="n"/>
-      <c r="AV41" s="1" t="n"/>
-      <c r="AW41" s="1" t="n"/>
-      <c r="AX41" s="1" t="n"/>
-      <c r="AY41" s="1" t="n"/>
-      <c r="AZ41" s="1" t="n"/>
-      <c r="BA41" s="1" t="n"/>
-      <c r="BB41" s="1" t="n"/>
-      <c r="BC41" s="1" t="n"/>
-      <c r="BD41" s="1" t="n"/>
-      <c r="BE41" s="1" t="n"/>
-      <c r="BF41" s="1" t="n"/>
-      <c r="BG41" s="1" t="n"/>
-      <c r="BH41" s="1" t="n"/>
-      <c r="BI41" s="1" t="n"/>
-      <c r="BJ41" s="1" t="n"/>
-      <c r="BK41" s="1" t="n"/>
-      <c r="BL41" s="1" t="n"/>
-      <c r="BM41" s="1" t="n"/>
-      <c r="BN41" s="1" t="n"/>
-      <c r="BO41" s="1" t="n"/>
-      <c r="BP41" s="1" t="n"/>
-      <c r="BQ41" s="1" t="n"/>
-      <c r="BR41" s="1" t="n"/>
-      <c r="BS41" s="1" t="n"/>
-      <c r="BT41" s="1" t="n"/>
-      <c r="BU41" s="1" t="n"/>
-      <c r="BV41" s="1" t="n"/>
-      <c r="BW41" s="20">
-        <f>IF(OR($C$9="",N($DF$9)=0),"","FACTURATION · "&amp;CHOOSE(MONTH(DATE(YEAR($C$9),MONTH($C$9)+2,1)),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR(DATE(YEAR($C$9),MONTH($C$9)+2,1))&amp;"   (hors transport et autres frais)")</f>
-        <v/>
-      </c>
-      <c r="BX41" s="1" t="n"/>
-      <c r="BY41" s="1" t="n"/>
-      <c r="BZ41" s="1" t="n"/>
-      <c r="CA41" s="1" t="n"/>
-      <c r="CB41" s="1" t="n"/>
-      <c r="CC41" s="1" t="n"/>
-      <c r="CD41" s="1" t="n"/>
-      <c r="CE41" s="1" t="n"/>
-      <c r="CF41" s="1" t="n"/>
-      <c r="CG41" s="1" t="n"/>
-      <c r="CH41" s="1" t="n"/>
-      <c r="CI41" s="1" t="n"/>
-      <c r="CJ41" s="1" t="n"/>
-      <c r="CK41" s="1" t="n"/>
-      <c r="CL41" s="1" t="n"/>
-      <c r="CM41" s="1" t="n"/>
-      <c r="CN41" s="1" t="n"/>
-      <c r="CO41" s="1" t="n"/>
-      <c r="CP41" s="1" t="n"/>
-      <c r="CQ41" s="1" t="n"/>
-      <c r="CR41" s="1" t="n"/>
-      <c r="CS41" s="1" t="n"/>
-      <c r="CT41" s="1" t="n"/>
-      <c r="CU41" s="1" t="n"/>
-      <c r="CV41" s="1" t="n"/>
-      <c r="CW41" s="1" t="n"/>
-      <c r="CX41" s="1" t="n"/>
-      <c r="CY41" s="1" t="n"/>
-      <c r="CZ41" s="1" t="n"/>
-      <c r="DA41" s="1" t="n"/>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="23" t="n"/>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="32" t="n"/>
+      <c r="D40" s="26" t="n"/>
+      <c r="E40" s="25" t="n"/>
+      <c r="F40" s="26" t="n"/>
+      <c r="G40" s="26" t="n"/>
+      <c r="H40" s="26" t="n"/>
+      <c r="I40" s="26" t="n"/>
+      <c r="J40" s="28" t="n"/>
+      <c r="K40" s="28" t="n"/>
+      <c r="L40" s="29">
+        <f>IF(B40="","",N(C40)*N(E40))</f>
+        <v/>
+      </c>
+      <c r="M40" s="34" t="n"/>
+      <c r="N40" s="34" t="n"/>
+      <c r="O40" s="34" t="n"/>
+      <c r="P40" s="34" t="n"/>
+      <c r="Q40" s="34" t="n"/>
+      <c r="R40" s="34" t="n"/>
+      <c r="S40" s="34" t="n"/>
+      <c r="T40" s="34" t="n"/>
+      <c r="U40" s="34" t="n"/>
+      <c r="V40" s="34" t="n"/>
+      <c r="W40" s="34" t="n"/>
+      <c r="X40" s="34" t="n"/>
+      <c r="Y40" s="34" t="n"/>
+      <c r="Z40" s="34" t="n"/>
+      <c r="AA40" s="34" t="n"/>
+      <c r="AB40" s="34" t="n"/>
+      <c r="AC40" s="34" t="n"/>
+      <c r="AD40" s="34" t="n"/>
+      <c r="AE40" s="34" t="n"/>
+      <c r="AF40" s="34" t="n"/>
+      <c r="AG40" s="34" t="n"/>
+      <c r="AH40" s="34" t="n"/>
+      <c r="AI40" s="34" t="n"/>
+      <c r="AJ40" s="34" t="n"/>
+      <c r="AK40" s="34" t="n"/>
+      <c r="AL40" s="34" t="n"/>
+      <c r="AM40" s="34" t="n"/>
+      <c r="AN40" s="34" t="n"/>
+      <c r="AO40" s="34" t="n"/>
+      <c r="AP40" s="34" t="n"/>
+      <c r="AQ40" s="34" t="n"/>
+      <c r="AR40" s="34" t="n"/>
+      <c r="AS40" s="34" t="n"/>
+      <c r="AT40" s="34" t="n"/>
+      <c r="AU40" s="34" t="n"/>
+      <c r="AV40" s="34" t="n"/>
+      <c r="AW40" s="34" t="n"/>
+      <c r="AX40" s="34" t="n"/>
+      <c r="AY40" s="34" t="n"/>
+      <c r="AZ40" s="34" t="n"/>
+      <c r="BA40" s="34" t="n"/>
+      <c r="BB40" s="34" t="n"/>
+      <c r="BC40" s="34" t="n"/>
+      <c r="BD40" s="34" t="n"/>
+      <c r="BE40" s="34" t="n"/>
+      <c r="BF40" s="34" t="n"/>
+      <c r="BG40" s="34" t="n"/>
+      <c r="BH40" s="34" t="n"/>
+      <c r="BI40" s="34" t="n"/>
+      <c r="BJ40" s="34" t="n"/>
+      <c r="BK40" s="34" t="n"/>
+      <c r="BL40" s="34" t="n"/>
+      <c r="BM40" s="34" t="n"/>
+      <c r="BN40" s="34" t="n"/>
+      <c r="BO40" s="34" t="n"/>
+      <c r="BP40" s="34" t="n"/>
+      <c r="BQ40" s="34" t="n"/>
+      <c r="BR40" s="34" t="n"/>
+      <c r="BS40" s="34" t="n"/>
+      <c r="BT40" s="34" t="n"/>
+      <c r="BU40" s="34" t="n"/>
+      <c r="BV40" s="34" t="n"/>
+      <c r="BW40" s="34" t="n"/>
+      <c r="BX40" s="34" t="n"/>
+      <c r="BY40" s="34" t="n"/>
+      <c r="BZ40" s="34" t="n"/>
+      <c r="CA40" s="34" t="n"/>
+      <c r="CB40" s="34" t="n"/>
+      <c r="CC40" s="34" t="n"/>
+      <c r="CD40" s="34" t="n"/>
+      <c r="CE40" s="34" t="n"/>
+      <c r="CF40" s="34" t="n"/>
+      <c r="CG40" s="34" t="n"/>
+      <c r="CH40" s="34" t="n"/>
+      <c r="CI40" s="34" t="n"/>
+      <c r="CJ40" s="34" t="n"/>
+      <c r="CK40" s="34" t="n"/>
+      <c r="CL40" s="34" t="n"/>
+      <c r="CM40" s="34" t="n"/>
+      <c r="CN40" s="34" t="n"/>
+      <c r="CO40" s="34" t="n"/>
+      <c r="CP40" s="34" t="n"/>
+      <c r="CQ40" s="34" t="n"/>
+      <c r="CR40" s="34" t="n"/>
+      <c r="CS40" s="34" t="n"/>
+      <c r="CT40" s="34" t="n"/>
+      <c r="CU40" s="34" t="n"/>
+      <c r="CV40" s="34" t="n"/>
+      <c r="CW40" s="34" t="n"/>
+      <c r="CX40" s="34" t="n"/>
+      <c r="CY40" s="34" t="n"/>
+      <c r="CZ40" s="34" t="n"/>
+      <c r="DA40" s="34" t="n"/>
+      <c r="DC40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DH40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DI40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DO40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DQ40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DR40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DS40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DZ40" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="EA40" s="31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="23" t="n"/>
+      <c r="B41" s="24" t="n"/>
+      <c r="C41" s="32" t="n"/>
+      <c r="D41" s="26" t="n"/>
+      <c r="E41" s="25" t="n"/>
+      <c r="F41" s="26" t="n"/>
+      <c r="G41" s="26" t="n"/>
+      <c r="H41" s="26" t="n"/>
+      <c r="I41" s="26" t="n"/>
+      <c r="J41" s="28" t="n"/>
+      <c r="K41" s="28" t="n"/>
+      <c r="L41" s="29">
+        <f>IF(B41="","",N(C41)*N(E41))</f>
+        <v/>
+      </c>
+      <c r="M41" s="34" t="n"/>
+      <c r="N41" s="34" t="n"/>
+      <c r="O41" s="34" t="n"/>
+      <c r="P41" s="34" t="n"/>
+      <c r="Q41" s="34" t="n"/>
+      <c r="R41" s="34" t="n"/>
+      <c r="S41" s="34" t="n"/>
+      <c r="T41" s="34" t="n"/>
+      <c r="U41" s="34" t="n"/>
+      <c r="V41" s="34" t="n"/>
+      <c r="W41" s="34" t="n"/>
+      <c r="X41" s="34" t="n"/>
+      <c r="Y41" s="34" t="n"/>
+      <c r="Z41" s="34" t="n"/>
+      <c r="AA41" s="34" t="n"/>
+      <c r="AB41" s="34" t="n"/>
+      <c r="AC41" s="34" t="n"/>
+      <c r="AD41" s="34" t="n"/>
+      <c r="AE41" s="34" t="n"/>
+      <c r="AF41" s="34" t="n"/>
+      <c r="AG41" s="34" t="n"/>
+      <c r="AH41" s="34" t="n"/>
+      <c r="AI41" s="34" t="n"/>
+      <c r="AJ41" s="34" t="n"/>
+      <c r="AK41" s="34" t="n"/>
+      <c r="AL41" s="34" t="n"/>
+      <c r="AM41" s="34" t="n"/>
+      <c r="AN41" s="34" t="n"/>
+      <c r="AO41" s="34" t="n"/>
+      <c r="AP41" s="34" t="n"/>
+      <c r="AQ41" s="34" t="n"/>
+      <c r="AR41" s="34" t="n"/>
+      <c r="AS41" s="34" t="n"/>
+      <c r="AT41" s="34" t="n"/>
+      <c r="AU41" s="34" t="n"/>
+      <c r="AV41" s="34" t="n"/>
+      <c r="AW41" s="34" t="n"/>
+      <c r="AX41" s="34" t="n"/>
+      <c r="AY41" s="34" t="n"/>
+      <c r="AZ41" s="34" t="n"/>
+      <c r="BA41" s="34" t="n"/>
+      <c r="BB41" s="34" t="n"/>
+      <c r="BC41" s="34" t="n"/>
+      <c r="BD41" s="34" t="n"/>
+      <c r="BE41" s="34" t="n"/>
+      <c r="BF41" s="34" t="n"/>
+      <c r="BG41" s="34" t="n"/>
+      <c r="BH41" s="34" t="n"/>
+      <c r="BI41" s="34" t="n"/>
+      <c r="BJ41" s="34" t="n"/>
+      <c r="BK41" s="34" t="n"/>
+      <c r="BL41" s="34" t="n"/>
+      <c r="BM41" s="34" t="n"/>
+      <c r="BN41" s="34" t="n"/>
+      <c r="BO41" s="34" t="n"/>
+      <c r="BP41" s="34" t="n"/>
+      <c r="BQ41" s="34" t="n"/>
+      <c r="BR41" s="34" t="n"/>
+      <c r="BS41" s="34" t="n"/>
+      <c r="BT41" s="34" t="n"/>
+      <c r="BU41" s="34" t="n"/>
+      <c r="BV41" s="34" t="n"/>
+      <c r="BW41" s="34" t="n"/>
+      <c r="BX41" s="34" t="n"/>
+      <c r="BY41" s="34" t="n"/>
+      <c r="BZ41" s="34" t="n"/>
+      <c r="CA41" s="34" t="n"/>
+      <c r="CB41" s="34" t="n"/>
+      <c r="CC41" s="34" t="n"/>
+      <c r="CD41" s="34" t="n"/>
+      <c r="CE41" s="34" t="n"/>
+      <c r="CF41" s="34" t="n"/>
+      <c r="CG41" s="34" t="n"/>
+      <c r="CH41" s="34" t="n"/>
+      <c r="CI41" s="34" t="n"/>
+      <c r="CJ41" s="34" t="n"/>
+      <c r="CK41" s="34" t="n"/>
+      <c r="CL41" s="34" t="n"/>
+      <c r="CM41" s="34" t="n"/>
+      <c r="CN41" s="34" t="n"/>
+      <c r="CO41" s="34" t="n"/>
+      <c r="CP41" s="34" t="n"/>
+      <c r="CQ41" s="34" t="n"/>
+      <c r="CR41" s="34" t="n"/>
+      <c r="CS41" s="34" t="n"/>
+      <c r="CT41" s="34" t="n"/>
+      <c r="CU41" s="34" t="n"/>
+      <c r="CV41" s="34" t="n"/>
+      <c r="CW41" s="34" t="n"/>
+      <c r="CX41" s="34" t="n"/>
+      <c r="CY41" s="34" t="n"/>
+      <c r="CZ41" s="34" t="n"/>
+      <c r="DA41" s="34" t="n"/>
+      <c r="DC41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DH41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DI41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DO41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DQ41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DR41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DS41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DZ41" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="EA41" s="31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="34">
-        <f>"Opérateurs · tarif journalier ("&amp;SUM(K17:K19)&amp;" j opérations, "&amp;SUM(J17:J19)&amp;" j stand-by)"</f>
-        <v/>
-      </c>
-      <c r="B42" s="23" t="n"/>
-      <c r="C42" s="23" t="n"/>
-      <c r="D42" s="23" t="n"/>
-      <c r="E42" s="23" t="n"/>
-      <c r="F42" s="23" t="n"/>
-      <c r="G42" s="35" t="inlineStr">
-        <is>
-          <t>910XFISHINGOP</t>
-        </is>
-      </c>
-      <c r="H42" s="23" t="n"/>
-      <c r="I42" s="23" t="n"/>
-      <c r="J42" s="23" t="n"/>
-      <c r="K42" s="23" t="n"/>
-      <c r="L42" s="36">
-        <f>SUM(DF17:DF19)+SUM(DM17:DM19)+SUM(DT17:DT19)</f>
-        <v/>
-      </c>
-      <c r="M42" s="37" t="inlineStr">
-        <is>
-          <t>Opérateurs · jours</t>
-        </is>
-      </c>
-      <c r="N42" s="23" t="n"/>
-      <c r="O42" s="23" t="n"/>
-      <c r="P42" s="23" t="n"/>
-      <c r="Q42" s="23" t="n"/>
-      <c r="R42" s="23" t="n"/>
-      <c r="S42" s="23" t="n"/>
-      <c r="T42" s="23" t="n"/>
-      <c r="U42" s="23" t="n"/>
-      <c r="V42" s="23" t="n"/>
-      <c r="W42" s="23" t="n"/>
-      <c r="X42" s="23" t="n"/>
-      <c r="Y42" s="23" t="n"/>
-      <c r="Z42" s="23" t="n"/>
-      <c r="AA42" s="23" t="n"/>
-      <c r="AB42" s="23" t="n"/>
-      <c r="AC42" s="23" t="n"/>
-      <c r="AD42" s="23" t="n"/>
-      <c r="AE42" s="29">
-        <f>IF(N($DD$9)=0,"",SUM(DF17:DF19))</f>
-        <v/>
-      </c>
-      <c r="AF42" s="23" t="n"/>
-      <c r="AG42" s="23" t="n"/>
-      <c r="AH42" s="23" t="n"/>
-      <c r="AI42" s="23" t="n"/>
-      <c r="AJ42" s="23" t="n"/>
-      <c r="AK42" s="23" t="n"/>
-      <c r="AL42" s="23" t="n"/>
-      <c r="AR42" s="37" t="inlineStr">
-        <is>
-          <t>Opérateurs · jours</t>
-        </is>
-      </c>
-      <c r="AS42" s="23" t="n"/>
-      <c r="AT42" s="23" t="n"/>
-      <c r="AU42" s="23" t="n"/>
-      <c r="AV42" s="23" t="n"/>
-      <c r="AW42" s="23" t="n"/>
-      <c r="AX42" s="23" t="n"/>
-      <c r="AY42" s="23" t="n"/>
-      <c r="AZ42" s="23" t="n"/>
-      <c r="BA42" s="23" t="n"/>
-      <c r="BB42" s="23" t="n"/>
-      <c r="BC42" s="23" t="n"/>
-      <c r="BD42" s="23" t="n"/>
-      <c r="BE42" s="23" t="n"/>
-      <c r="BF42" s="23" t="n"/>
-      <c r="BG42" s="23" t="n"/>
-      <c r="BH42" s="23" t="n"/>
-      <c r="BI42" s="23" t="n"/>
-      <c r="BJ42" s="29">
-        <f>IF(N($DE$9)=0,"",SUM(DM17:DM19))</f>
-        <v/>
-      </c>
-      <c r="BK42" s="23" t="n"/>
-      <c r="BL42" s="23" t="n"/>
-      <c r="BM42" s="23" t="n"/>
-      <c r="BN42" s="23" t="n"/>
-      <c r="BO42" s="23" t="n"/>
-      <c r="BP42" s="23" t="n"/>
-      <c r="BQ42" s="23" t="n"/>
-      <c r="BW42" s="37" t="inlineStr">
-        <is>
-          <t>Opérateurs · jours</t>
-        </is>
-      </c>
-      <c r="BX42" s="23" t="n"/>
-      <c r="BY42" s="23" t="n"/>
-      <c r="BZ42" s="23" t="n"/>
-      <c r="CA42" s="23" t="n"/>
-      <c r="CB42" s="23" t="n"/>
-      <c r="CC42" s="23" t="n"/>
-      <c r="CD42" s="23" t="n"/>
-      <c r="CE42" s="23" t="n"/>
-      <c r="CF42" s="23" t="n"/>
-      <c r="CG42" s="23" t="n"/>
-      <c r="CH42" s="23" t="n"/>
-      <c r="CI42" s="23" t="n"/>
-      <c r="CJ42" s="23" t="n"/>
-      <c r="CK42" s="23" t="n"/>
-      <c r="CL42" s="23" t="n"/>
-      <c r="CM42" s="23" t="n"/>
-      <c r="CN42" s="23" t="n"/>
-      <c r="CO42" s="29">
-        <f>IF(N($DF$9)=0,"",SUM(DT17:DT19))</f>
-        <v/>
-      </c>
-      <c r="CP42" s="23" t="n"/>
-      <c r="CQ42" s="23" t="n"/>
-      <c r="CR42" s="23" t="n"/>
-      <c r="CS42" s="23" t="n"/>
-      <c r="CT42" s="23" t="n"/>
-      <c r="CU42" s="23" t="n"/>
-      <c r="CV42" s="23" t="n"/>
+      <c r="A42" s="23" t="n"/>
+      <c r="B42" s="24" t="n"/>
+      <c r="C42" s="32" t="n"/>
+      <c r="D42" s="26" t="n"/>
+      <c r="E42" s="25" t="n"/>
+      <c r="F42" s="26" t="n"/>
+      <c r="G42" s="26" t="n"/>
+      <c r="H42" s="26" t="n"/>
+      <c r="I42" s="26" t="n"/>
+      <c r="J42" s="28" t="n"/>
+      <c r="K42" s="28" t="n"/>
+      <c r="L42" s="29">
+        <f>IF(B42="","",N(C42)*N(E42))</f>
+        <v/>
+      </c>
+      <c r="M42" s="34" t="n"/>
+      <c r="N42" s="34" t="n"/>
+      <c r="O42" s="34" t="n"/>
+      <c r="P42" s="34" t="n"/>
+      <c r="Q42" s="34" t="n"/>
+      <c r="R42" s="34" t="n"/>
+      <c r="S42" s="34" t="n"/>
+      <c r="T42" s="34" t="n"/>
+      <c r="U42" s="34" t="n"/>
+      <c r="V42" s="34" t="n"/>
+      <c r="W42" s="34" t="n"/>
+      <c r="X42" s="34" t="n"/>
+      <c r="Y42" s="34" t="n"/>
+      <c r="Z42" s="34" t="n"/>
+      <c r="AA42" s="34" t="n"/>
+      <c r="AB42" s="34" t="n"/>
+      <c r="AC42" s="34" t="n"/>
+      <c r="AD42" s="34" t="n"/>
+      <c r="AE42" s="34" t="n"/>
+      <c r="AF42" s="34" t="n"/>
+      <c r="AG42" s="34" t="n"/>
+      <c r="AH42" s="34" t="n"/>
+      <c r="AI42" s="34" t="n"/>
+      <c r="AJ42" s="34" t="n"/>
+      <c r="AK42" s="34" t="n"/>
+      <c r="AL42" s="34" t="n"/>
+      <c r="AM42" s="34" t="n"/>
+      <c r="AN42" s="34" t="n"/>
+      <c r="AO42" s="34" t="n"/>
+      <c r="AP42" s="34" t="n"/>
+      <c r="AQ42" s="34" t="n"/>
+      <c r="AR42" s="34" t="n"/>
+      <c r="AS42" s="34" t="n"/>
+      <c r="AT42" s="34" t="n"/>
+      <c r="AU42" s="34" t="n"/>
+      <c r="AV42" s="34" t="n"/>
+      <c r="AW42" s="34" t="n"/>
+      <c r="AX42" s="34" t="n"/>
+      <c r="AY42" s="34" t="n"/>
+      <c r="AZ42" s="34" t="n"/>
+      <c r="BA42" s="34" t="n"/>
+      <c r="BB42" s="34" t="n"/>
+      <c r="BC42" s="34" t="n"/>
+      <c r="BD42" s="34" t="n"/>
+      <c r="BE42" s="34" t="n"/>
+      <c r="BF42" s="34" t="n"/>
+      <c r="BG42" s="34" t="n"/>
+      <c r="BH42" s="34" t="n"/>
+      <c r="BI42" s="34" t="n"/>
+      <c r="BJ42" s="34" t="n"/>
+      <c r="BK42" s="34" t="n"/>
+      <c r="BL42" s="34" t="n"/>
+      <c r="BM42" s="34" t="n"/>
+      <c r="BN42" s="34" t="n"/>
+      <c r="BO42" s="34" t="n"/>
+      <c r="BP42" s="34" t="n"/>
+      <c r="BQ42" s="34" t="n"/>
+      <c r="BR42" s="34" t="n"/>
+      <c r="BS42" s="34" t="n"/>
+      <c r="BT42" s="34" t="n"/>
+      <c r="BU42" s="34" t="n"/>
+      <c r="BV42" s="34" t="n"/>
+      <c r="BW42" s="34" t="n"/>
+      <c r="BX42" s="34" t="n"/>
+      <c r="BY42" s="34" t="n"/>
+      <c r="BZ42" s="34" t="n"/>
+      <c r="CA42" s="34" t="n"/>
+      <c r="CB42" s="34" t="n"/>
+      <c r="CC42" s="34" t="n"/>
+      <c r="CD42" s="34" t="n"/>
+      <c r="CE42" s="34" t="n"/>
+      <c r="CF42" s="34" t="n"/>
+      <c r="CG42" s="34" t="n"/>
+      <c r="CH42" s="34" t="n"/>
+      <c r="CI42" s="34" t="n"/>
+      <c r="CJ42" s="34" t="n"/>
+      <c r="CK42" s="34" t="n"/>
+      <c r="CL42" s="34" t="n"/>
+      <c r="CM42" s="34" t="n"/>
+      <c r="CN42" s="34" t="n"/>
+      <c r="CO42" s="34" t="n"/>
+      <c r="CP42" s="34" t="n"/>
+      <c r="CQ42" s="34" t="n"/>
+      <c r="CR42" s="34" t="n"/>
+      <c r="CS42" s="34" t="n"/>
+      <c r="CT42" s="34" t="n"/>
+      <c r="CU42" s="34" t="n"/>
+      <c r="CV42" s="34" t="n"/>
+      <c r="CW42" s="34" t="n"/>
+      <c r="CX42" s="34" t="n"/>
+      <c r="CY42" s="34" t="n"/>
+      <c r="CZ42" s="34" t="n"/>
+      <c r="DA42" s="34" t="n"/>
+      <c r="DC42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DH42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DI42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DO42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DP42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DQ42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DR42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DS42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DX42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DY42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="DZ42" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="EA42" s="31" t="n">
+        <v>0</v>
+      </c>
     </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="34">
-        <f>"Opérateurs · mob / demob ("&amp;SUM(I17:I19)&amp;")"</f>
-        <v/>
-      </c>
-      <c r="B43" s="23" t="n"/>
-      <c r="C43" s="23" t="n"/>
-      <c r="D43" s="23" t="n"/>
-      <c r="E43" s="23" t="n"/>
-      <c r="F43" s="23" t="n"/>
-      <c r="G43" s="35" t="inlineStr">
-        <is>
-          <t>900XMOBDEMOB</t>
-        </is>
-      </c>
-      <c r="H43" s="23" t="n"/>
-      <c r="I43" s="23" t="n"/>
-      <c r="J43" s="23" t="n"/>
-      <c r="K43" s="23" t="n"/>
-      <c r="L43" s="36">
-        <f>SUM(DG17:DG19)+SUM(DN17:DN19)+SUM(DU17:DU19)</f>
-        <v/>
-      </c>
-      <c r="M43" s="37" t="inlineStr">
-        <is>
-          <t>Opérateurs · mob / demob</t>
-        </is>
-      </c>
-      <c r="N43" s="23" t="n"/>
-      <c r="O43" s="23" t="n"/>
-      <c r="P43" s="23" t="n"/>
-      <c r="Q43" s="23" t="n"/>
-      <c r="R43" s="23" t="n"/>
-      <c r="S43" s="23" t="n"/>
-      <c r="T43" s="23" t="n"/>
-      <c r="U43" s="23" t="n"/>
-      <c r="V43" s="23" t="n"/>
-      <c r="W43" s="23" t="n"/>
-      <c r="X43" s="23" t="n"/>
-      <c r="Y43" s="23" t="n"/>
-      <c r="Z43" s="23" t="n"/>
-      <c r="AA43" s="23" t="n"/>
-      <c r="AB43" s="23" t="n"/>
-      <c r="AC43" s="23" t="n"/>
-      <c r="AD43" s="23" t="n"/>
-      <c r="AE43" s="29">
-        <f>IF(N($DD$9)=0,"",SUM(DG17:DG19))</f>
-        <v/>
-      </c>
-      <c r="AF43" s="23" t="n"/>
-      <c r="AG43" s="23" t="n"/>
-      <c r="AH43" s="23" t="n"/>
-      <c r="AI43" s="23" t="n"/>
-      <c r="AJ43" s="23" t="n"/>
-      <c r="AK43" s="23" t="n"/>
-      <c r="AL43" s="23" t="n"/>
-      <c r="AR43" s="37" t="inlineStr">
-        <is>
-          <t>Opérateurs · mob / demob</t>
-        </is>
-      </c>
-      <c r="AS43" s="23" t="n"/>
-      <c r="AT43" s="23" t="n"/>
-      <c r="AU43" s="23" t="n"/>
-      <c r="AV43" s="23" t="n"/>
-      <c r="AW43" s="23" t="n"/>
-      <c r="AX43" s="23" t="n"/>
-      <c r="AY43" s="23" t="n"/>
-      <c r="AZ43" s="23" t="n"/>
-      <c r="BA43" s="23" t="n"/>
-      <c r="BB43" s="23" t="n"/>
-      <c r="BC43" s="23" t="n"/>
-      <c r="BD43" s="23" t="n"/>
-      <c r="BE43" s="23" t="n"/>
-      <c r="BF43" s="23" t="n"/>
-      <c r="BG43" s="23" t="n"/>
-      <c r="BH43" s="23" t="n"/>
-      <c r="BI43" s="23" t="n"/>
-      <c r="BJ43" s="29">
-        <f>IF(N($DE$9)=0,"",SUM(DN17:DN19))</f>
-        <v/>
-      </c>
-      <c r="BK43" s="23" t="n"/>
-      <c r="BL43" s="23" t="n"/>
-      <c r="BM43" s="23" t="n"/>
-      <c r="BN43" s="23" t="n"/>
-      <c r="BO43" s="23" t="n"/>
-      <c r="BP43" s="23" t="n"/>
-      <c r="BQ43" s="23" t="n"/>
-      <c r="BW43" s="37" t="inlineStr">
-        <is>
-          <t>Opérateurs · mob / demob</t>
-        </is>
-      </c>
-      <c r="BX43" s="23" t="n"/>
-      <c r="BY43" s="23" t="n"/>
-      <c r="BZ43" s="23" t="n"/>
-      <c r="CA43" s="23" t="n"/>
-      <c r="CB43" s="23" t="n"/>
-      <c r="CC43" s="23" t="n"/>
-      <c r="CD43" s="23" t="n"/>
-      <c r="CE43" s="23" t="n"/>
-      <c r="CF43" s="23" t="n"/>
-      <c r="CG43" s="23" t="n"/>
-      <c r="CH43" s="23" t="n"/>
-      <c r="CI43" s="23" t="n"/>
-      <c r="CJ43" s="23" t="n"/>
-      <c r="CK43" s="23" t="n"/>
-      <c r="CL43" s="23" t="n"/>
-      <c r="CM43" s="23" t="n"/>
-      <c r="CN43" s="23" t="n"/>
-      <c r="CO43" s="29">
-        <f>IF(N($DF$9)=0,"",SUM(DU17:DU19))</f>
-        <v/>
-      </c>
-      <c r="CP43" s="23" t="n"/>
-      <c r="CQ43" s="23" t="n"/>
-      <c r="CR43" s="23" t="n"/>
-      <c r="CS43" s="23" t="n"/>
-      <c r="CT43" s="23" t="n"/>
-      <c r="CU43" s="23" t="n"/>
-      <c r="CV43" s="23" t="n"/>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="34" t="inlineStr">
-        <is>
-          <t>Location du matériel (stand-by + opérations)</t>
-        </is>
-      </c>
-      <c r="B44" s="23" t="n"/>
-      <c r="C44" s="23" t="n"/>
-      <c r="D44" s="23" t="n"/>
-      <c r="E44" s="23" t="n"/>
-      <c r="F44" s="23" t="n"/>
-      <c r="G44" s="35" t="inlineStr">
-        <is>
-          <t>904XRENTALEQUIPMT</t>
-        </is>
-      </c>
-      <c r="H44" s="23" t="n"/>
-      <c r="I44" s="23" t="n"/>
-      <c r="J44" s="23" t="n"/>
-      <c r="K44" s="23" t="n"/>
-      <c r="L44" s="36">
-        <f>SUM(DF22:DF33)+SUM(DM22:DM33)+SUM(DT22:DT33)</f>
-        <v/>
-      </c>
-      <c r="M44" s="37" t="inlineStr">
-        <is>
-          <t>Location du matériel</t>
-        </is>
-      </c>
-      <c r="N44" s="23" t="n"/>
-      <c r="O44" s="23" t="n"/>
-      <c r="P44" s="23" t="n"/>
-      <c r="Q44" s="23" t="n"/>
-      <c r="R44" s="23" t="n"/>
-      <c r="S44" s="23" t="n"/>
-      <c r="T44" s="23" t="n"/>
-      <c r="U44" s="23" t="n"/>
-      <c r="V44" s="23" t="n"/>
-      <c r="W44" s="23" t="n"/>
-      <c r="X44" s="23" t="n"/>
-      <c r="Y44" s="23" t="n"/>
-      <c r="Z44" s="23" t="n"/>
-      <c r="AA44" s="23" t="n"/>
-      <c r="AB44" s="23" t="n"/>
-      <c r="AC44" s="23" t="n"/>
-      <c r="AD44" s="23" t="n"/>
-      <c r="AE44" s="29">
-        <f>IF(N($DD$9)=0,"",SUM(DF22:DF33))</f>
-        <v/>
-      </c>
-      <c r="AF44" s="23" t="n"/>
-      <c r="AG44" s="23" t="n"/>
-      <c r="AH44" s="23" t="n"/>
-      <c r="AI44" s="23" t="n"/>
-      <c r="AJ44" s="23" t="n"/>
-      <c r="AK44" s="23" t="n"/>
-      <c r="AL44" s="23" t="n"/>
-      <c r="AR44" s="37" t="inlineStr">
-        <is>
-          <t>Location du matériel</t>
-        </is>
-      </c>
-      <c r="AS44" s="23" t="n"/>
-      <c r="AT44" s="23" t="n"/>
-      <c r="AU44" s="23" t="n"/>
-      <c r="AV44" s="23" t="n"/>
-      <c r="AW44" s="23" t="n"/>
-      <c r="AX44" s="23" t="n"/>
-      <c r="AY44" s="23" t="n"/>
-      <c r="AZ44" s="23" t="n"/>
-      <c r="BA44" s="23" t="n"/>
-      <c r="BB44" s="23" t="n"/>
-      <c r="BC44" s="23" t="n"/>
-      <c r="BD44" s="23" t="n"/>
-      <c r="BE44" s="23" t="n"/>
-      <c r="BF44" s="23" t="n"/>
-      <c r="BG44" s="23" t="n"/>
-      <c r="BH44" s="23" t="n"/>
-      <c r="BI44" s="23" t="n"/>
-      <c r="BJ44" s="29">
-        <f>IF(N($DE$9)=0,"",SUM(DM22:DM33))</f>
-        <v/>
-      </c>
-      <c r="BK44" s="23" t="n"/>
-      <c r="BL44" s="23" t="n"/>
-      <c r="BM44" s="23" t="n"/>
-      <c r="BN44" s="23" t="n"/>
-      <c r="BO44" s="23" t="n"/>
-      <c r="BP44" s="23" t="n"/>
-      <c r="BQ44" s="23" t="n"/>
-      <c r="BW44" s="37" t="inlineStr">
-        <is>
-          <t>Location du matériel</t>
-        </is>
-      </c>
-      <c r="BX44" s="23" t="n"/>
-      <c r="BY44" s="23" t="n"/>
-      <c r="BZ44" s="23" t="n"/>
-      <c r="CA44" s="23" t="n"/>
-      <c r="CB44" s="23" t="n"/>
-      <c r="CC44" s="23" t="n"/>
-      <c r="CD44" s="23" t="n"/>
-      <c r="CE44" s="23" t="n"/>
-      <c r="CF44" s="23" t="n"/>
-      <c r="CG44" s="23" t="n"/>
-      <c r="CH44" s="23" t="n"/>
-      <c r="CI44" s="23" t="n"/>
-      <c r="CJ44" s="23" t="n"/>
-      <c r="CK44" s="23" t="n"/>
-      <c r="CL44" s="23" t="n"/>
-      <c r="CM44" s="23" t="n"/>
-      <c r="CN44" s="23" t="n"/>
-      <c r="CO44" s="29">
-        <f>IF(N($DF$9)=0,"",SUM(DT22:DT33))</f>
-        <v/>
-      </c>
-      <c r="CP44" s="23" t="n"/>
-      <c r="CQ44" s="23" t="n"/>
-      <c r="CR44" s="23" t="n"/>
-      <c r="CS44" s="23" t="n"/>
-      <c r="CT44" s="23" t="n"/>
-      <c r="CU44" s="23" t="n"/>
-      <c r="CV44" s="23" t="n"/>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="34" t="inlineStr">
-        <is>
-          <t>Utilisation charge et inspection (UC, une seule fois)</t>
-        </is>
-      </c>
-      <c r="B45" s="23" t="n"/>
-      <c r="C45" s="23" t="n"/>
-      <c r="D45" s="23" t="n"/>
-      <c r="E45" s="23" t="n"/>
-      <c r="F45" s="23" t="n"/>
-      <c r="G45" s="35" t="inlineStr">
-        <is>
-          <t>905XUC</t>
-        </is>
-      </c>
-      <c r="H45" s="23" t="n"/>
-      <c r="I45" s="23" t="n"/>
-      <c r="J45" s="23" t="n"/>
-      <c r="K45" s="23" t="n"/>
-      <c r="L45" s="36">
-        <f>SUM(DG22:DG33)+SUM(DN22:DN33)+SUM(DU22:DU33)</f>
-        <v/>
-      </c>
-      <c r="M45" s="37" t="inlineStr">
-        <is>
-          <t>UC et inspection</t>
-        </is>
-      </c>
-      <c r="N45" s="23" t="n"/>
-      <c r="O45" s="23" t="n"/>
-      <c r="P45" s="23" t="n"/>
-      <c r="Q45" s="23" t="n"/>
-      <c r="R45" s="23" t="n"/>
-      <c r="S45" s="23" t="n"/>
-      <c r="T45" s="23" t="n"/>
-      <c r="U45" s="23" t="n"/>
-      <c r="V45" s="23" t="n"/>
-      <c r="W45" s="23" t="n"/>
-      <c r="X45" s="23" t="n"/>
-      <c r="Y45" s="23" t="n"/>
-      <c r="Z45" s="23" t="n"/>
-      <c r="AA45" s="23" t="n"/>
-      <c r="AB45" s="23" t="n"/>
-      <c r="AC45" s="23" t="n"/>
-      <c r="AD45" s="23" t="n"/>
-      <c r="AE45" s="29">
-        <f>IF(N($DD$9)=0,"",SUM(DG22:DG33))</f>
-        <v/>
-      </c>
-      <c r="AF45" s="23" t="n"/>
-      <c r="AG45" s="23" t="n"/>
-      <c r="AH45" s="23" t="n"/>
-      <c r="AI45" s="23" t="n"/>
-      <c r="AJ45" s="23" t="n"/>
-      <c r="AK45" s="23" t="n"/>
-      <c r="AL45" s="23" t="n"/>
-      <c r="AR45" s="37" t="inlineStr">
-        <is>
-          <t>UC et inspection</t>
-        </is>
-      </c>
-      <c r="AS45" s="23" t="n"/>
-      <c r="AT45" s="23" t="n"/>
-      <c r="AU45" s="23" t="n"/>
-      <c r="AV45" s="23" t="n"/>
-      <c r="AW45" s="23" t="n"/>
-      <c r="AX45" s="23" t="n"/>
-      <c r="AY45" s="23" t="n"/>
-      <c r="AZ45" s="23" t="n"/>
-      <c r="BA45" s="23" t="n"/>
-      <c r="BB45" s="23" t="n"/>
-      <c r="BC45" s="23" t="n"/>
-      <c r="BD45" s="23" t="n"/>
-      <c r="BE45" s="23" t="n"/>
-      <c r="BF45" s="23" t="n"/>
-      <c r="BG45" s="23" t="n"/>
-      <c r="BH45" s="23" t="n"/>
-      <c r="BI45" s="23" t="n"/>
-      <c r="BJ45" s="29">
-        <f>IF(N($DE$9)=0,"",SUM(DN22:DN33))</f>
-        <v/>
-      </c>
-      <c r="BK45" s="23" t="n"/>
-      <c r="BL45" s="23" t="n"/>
-      <c r="BM45" s="23" t="n"/>
-      <c r="BN45" s="23" t="n"/>
-      <c r="BO45" s="23" t="n"/>
-      <c r="BP45" s="23" t="n"/>
-      <c r="BQ45" s="23" t="n"/>
-      <c r="BW45" s="37" t="inlineStr">
-        <is>
-          <t>UC et inspection</t>
-        </is>
-      </c>
-      <c r="BX45" s="23" t="n"/>
-      <c r="BY45" s="23" t="n"/>
-      <c r="BZ45" s="23" t="n"/>
-      <c r="CA45" s="23" t="n"/>
-      <c r="CB45" s="23" t="n"/>
-      <c r="CC45" s="23" t="n"/>
-      <c r="CD45" s="23" t="n"/>
-      <c r="CE45" s="23" t="n"/>
-      <c r="CF45" s="23" t="n"/>
-      <c r="CG45" s="23" t="n"/>
-      <c r="CH45" s="23" t="n"/>
-      <c r="CI45" s="23" t="n"/>
-      <c r="CJ45" s="23" t="n"/>
-      <c r="CK45" s="23" t="n"/>
-      <c r="CL45" s="23" t="n"/>
-      <c r="CM45" s="23" t="n"/>
-      <c r="CN45" s="23" t="n"/>
-      <c r="CO45" s="29">
-        <f>IF(N($DF$9)=0,"",SUM(DU22:DU33))</f>
-        <v/>
-      </c>
-      <c r="CP45" s="23" t="n"/>
-      <c r="CQ45" s="23" t="n"/>
-      <c r="CR45" s="23" t="n"/>
-      <c r="CS45" s="23" t="n"/>
-      <c r="CT45" s="23" t="n"/>
-      <c r="CU45" s="23" t="n"/>
-      <c r="CV45" s="23" t="n"/>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>RÉCAPITULATIF</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="n"/>
+      <c r="C45" s="1" t="n"/>
+      <c r="D45" s="1" t="n"/>
+      <c r="E45" s="1" t="n"/>
+      <c r="F45" s="1" t="n"/>
+      <c r="G45" s="1" t="n"/>
+      <c r="H45" s="1" t="n"/>
+      <c r="I45" s="1" t="n"/>
+      <c r="J45" s="1" t="n"/>
+      <c r="K45" s="1" t="n"/>
+      <c r="L45" s="1" t="n"/>
+      <c r="M45" s="20">
+        <f>IF(OR($C$9="",N($DD$9)=0),"","FACTURATION · "&amp;CHOOSE(MONTH($C$9),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR($C$9)&amp;"   (hors transport et autres frais)")</f>
+        <v/>
+      </c>
+      <c r="N45" s="1" t="n"/>
+      <c r="O45" s="1" t="n"/>
+      <c r="P45" s="1" t="n"/>
+      <c r="Q45" s="1" t="n"/>
+      <c r="R45" s="1" t="n"/>
+      <c r="S45" s="1" t="n"/>
+      <c r="T45" s="1" t="n"/>
+      <c r="U45" s="1" t="n"/>
+      <c r="V45" s="1" t="n"/>
+      <c r="W45" s="1" t="n"/>
+      <c r="X45" s="1" t="n"/>
+      <c r="Y45" s="1" t="n"/>
+      <c r="Z45" s="1" t="n"/>
+      <c r="AA45" s="1" t="n"/>
+      <c r="AB45" s="1" t="n"/>
+      <c r="AC45" s="1" t="n"/>
+      <c r="AD45" s="1" t="n"/>
+      <c r="AE45" s="1" t="n"/>
+      <c r="AF45" s="1" t="n"/>
+      <c r="AG45" s="1" t="n"/>
+      <c r="AH45" s="1" t="n"/>
+      <c r="AI45" s="1" t="n"/>
+      <c r="AJ45" s="1" t="n"/>
+      <c r="AK45" s="1" t="n"/>
+      <c r="AL45" s="1" t="n"/>
+      <c r="AM45" s="1" t="n"/>
+      <c r="AN45" s="1" t="n"/>
+      <c r="AO45" s="1" t="n"/>
+      <c r="AP45" s="1" t="n"/>
+      <c r="AQ45" s="1" t="n"/>
+      <c r="AR45" s="20">
+        <f>IF(OR($C$9="",N($DE$9)=0),"","FACTURATION · "&amp;CHOOSE(MONTH(DATE(YEAR($C$9),MONTH($C$9)+1,1)),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR(DATE(YEAR($C$9),MONTH($C$9)+1,1))&amp;"   (hors transport et autres frais)")</f>
+        <v/>
+      </c>
+      <c r="AS45" s="1" t="n"/>
+      <c r="AT45" s="1" t="n"/>
+      <c r="AU45" s="1" t="n"/>
+      <c r="AV45" s="1" t="n"/>
+      <c r="AW45" s="1" t="n"/>
+      <c r="AX45" s="1" t="n"/>
+      <c r="AY45" s="1" t="n"/>
+      <c r="AZ45" s="1" t="n"/>
+      <c r="BA45" s="1" t="n"/>
+      <c r="BB45" s="1" t="n"/>
+      <c r="BC45" s="1" t="n"/>
+      <c r="BD45" s="1" t="n"/>
+      <c r="BE45" s="1" t="n"/>
+      <c r="BF45" s="1" t="n"/>
+      <c r="BG45" s="1" t="n"/>
+      <c r="BH45" s="1" t="n"/>
+      <c r="BI45" s="1" t="n"/>
+      <c r="BJ45" s="1" t="n"/>
+      <c r="BK45" s="1" t="n"/>
+      <c r="BL45" s="1" t="n"/>
+      <c r="BM45" s="1" t="n"/>
+      <c r="BN45" s="1" t="n"/>
+      <c r="BO45" s="1" t="n"/>
+      <c r="BP45" s="1" t="n"/>
+      <c r="BQ45" s="1" t="n"/>
+      <c r="BR45" s="1" t="n"/>
+      <c r="BS45" s="1" t="n"/>
+      <c r="BT45" s="1" t="n"/>
+      <c r="BU45" s="1" t="n"/>
+      <c r="BV45" s="1" t="n"/>
+      <c r="BW45" s="20">
+        <f>IF(OR($C$9="",N($DF$9)=0),"","FACTURATION · "&amp;CHOOSE(MONTH(DATE(YEAR($C$9),MONTH($C$9)+2,1)),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR(DATE(YEAR($C$9),MONTH($C$9)+2,1))&amp;"   (hors transport et autres frais)")</f>
+        <v/>
+      </c>
+      <c r="BX45" s="1" t="n"/>
+      <c r="BY45" s="1" t="n"/>
+      <c r="BZ45" s="1" t="n"/>
+      <c r="CA45" s="1" t="n"/>
+      <c r="CB45" s="1" t="n"/>
+      <c r="CC45" s="1" t="n"/>
+      <c r="CD45" s="1" t="n"/>
+      <c r="CE45" s="1" t="n"/>
+      <c r="CF45" s="1" t="n"/>
+      <c r="CG45" s="1" t="n"/>
+      <c r="CH45" s="1" t="n"/>
+      <c r="CI45" s="1" t="n"/>
+      <c r="CJ45" s="1" t="n"/>
+      <c r="CK45" s="1" t="n"/>
+      <c r="CL45" s="1" t="n"/>
+      <c r="CM45" s="1" t="n"/>
+      <c r="CN45" s="1" t="n"/>
+      <c r="CO45" s="1" t="n"/>
+      <c r="CP45" s="1" t="n"/>
+      <c r="CQ45" s="1" t="n"/>
+      <c r="CR45" s="1" t="n"/>
+      <c r="CS45" s="1" t="n"/>
+      <c r="CT45" s="1" t="n"/>
+      <c r="CU45" s="1" t="n"/>
+      <c r="CV45" s="1" t="n"/>
+      <c r="CW45" s="1" t="n"/>
+      <c r="CX45" s="1" t="n"/>
+      <c r="CY45" s="1" t="n"/>
+      <c r="CZ45" s="1" t="n"/>
+      <c r="DA45" s="1" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="34" t="inlineStr">
-        <is>
-          <t>Valeur de remplacement et restocking</t>
-        </is>
+      <c r="A46" s="35">
+        <f>"Opérateurs · tarif journalier ("&amp;SUM(K17:K19)&amp;" j opérations, "&amp;SUM(J17:J19)&amp;" j stand-by)"</f>
+        <v/>
       </c>
       <c r="B46" s="23" t="n"/>
       <c r="C46" s="23" t="n"/>
       <c r="D46" s="23" t="n"/>
       <c r="E46" s="23" t="n"/>
       <c r="F46" s="23" t="n"/>
-      <c r="G46" s="35" t="inlineStr"/>
+      <c r="G46" s="36" t="inlineStr">
+        <is>
+          <t>910XFISHINGOP</t>
+        </is>
+      </c>
       <c r="H46" s="23" t="n"/>
       <c r="I46" s="23" t="n"/>
       <c r="J46" s="23" t="n"/>
       <c r="K46" s="23" t="n"/>
-      <c r="L46" s="36">
-        <f>SUM(DH22:DH33)+SUM(DO22:DO33)+SUM(DV22:DV33)</f>
-        <v/>
-      </c>
-      <c r="M46" s="37" t="inlineStr">
-        <is>
-          <t>Valeur de remplacement, restocking</t>
+      <c r="L46" s="37">
+        <f>SUM(DF17:DF19)+SUM(DM17:DM19)+SUM(DT17:DT19)</f>
+        <v/>
+      </c>
+      <c r="M46" s="38" t="inlineStr">
+        <is>
+          <t>Opérateurs · jours</t>
         </is>
       </c>
       <c r="N46" s="23" t="n"/>
@@ -6851,7 +6949,7 @@
       <c r="AC46" s="23" t="n"/>
       <c r="AD46" s="23" t="n"/>
       <c r="AE46" s="29">
-        <f>IF(N($DD$9)=0,"",SUM(DH22:DH33))</f>
+        <f>IF(N($DD$9)=0,"",SUM(DF17:DF19))</f>
         <v/>
       </c>
       <c r="AF46" s="23" t="n"/>
@@ -6861,9 +6959,9 @@
       <c r="AJ46" s="23" t="n"/>
       <c r="AK46" s="23" t="n"/>
       <c r="AL46" s="23" t="n"/>
-      <c r="AR46" s="37" t="inlineStr">
-        <is>
-          <t>Valeur de remplacement, restocking</t>
+      <c r="AR46" s="38" t="inlineStr">
+        <is>
+          <t>Opérateurs · jours</t>
         </is>
       </c>
       <c r="AS46" s="23" t="n"/>
@@ -6884,7 +6982,7 @@
       <c r="BH46" s="23" t="n"/>
       <c r="BI46" s="23" t="n"/>
       <c r="BJ46" s="29">
-        <f>IF(N($DE$9)=0,"",SUM(DO22:DO33))</f>
+        <f>IF(N($DE$9)=0,"",SUM(DM17:DM19))</f>
         <v/>
       </c>
       <c r="BK46" s="23" t="n"/>
@@ -6894,9 +6992,9 @@
       <c r="BO46" s="23" t="n"/>
       <c r="BP46" s="23" t="n"/>
       <c r="BQ46" s="23" t="n"/>
-      <c r="BW46" s="37" t="inlineStr">
-        <is>
-          <t>Valeur de remplacement, restocking</t>
+      <c r="BW46" s="38" t="inlineStr">
+        <is>
+          <t>Opérateurs · jours</t>
         </is>
       </c>
       <c r="BX46" s="23" t="n"/>
@@ -6917,7 +7015,7 @@
       <c r="CM46" s="23" t="n"/>
       <c r="CN46" s="23" t="n"/>
       <c r="CO46" s="29">
-        <f>IF(N($DF$9)=0,"",SUM(DV22:DV33))</f>
+        <f>IF(N($DF$9)=0,"",SUM(DT17:DT19))</f>
         <v/>
       </c>
       <c r="CP46" s="23" t="n"/>
@@ -6929,17 +7027,16 @@
       <c r="CV46" s="23" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="34" t="inlineStr">
-        <is>
-          <t>Transport et autres frais</t>
-        </is>
+      <c r="A47" s="35">
+        <f>"Opérateurs · mob / demob ("&amp;SUM(I17:I19)&amp;")"</f>
+        <v/>
       </c>
       <c r="B47" s="23" t="n"/>
       <c r="C47" s="23" t="n"/>
       <c r="D47" s="23" t="n"/>
       <c r="E47" s="23" t="n"/>
       <c r="F47" s="23" t="n"/>
-      <c r="G47" s="35" t="inlineStr">
+      <c r="G47" s="36" t="inlineStr">
         <is>
           <t>900XMOBDEMOB</t>
         </is>
@@ -6948,280 +7045,900 @@
       <c r="I47" s="23" t="n"/>
       <c r="J47" s="23" t="n"/>
       <c r="K47" s="23" t="n"/>
-      <c r="L47" s="36">
-        <f>SUM(L36:L38)</f>
-        <v/>
-      </c>
+      <c r="L47" s="37">
+        <f>SUM(DG17:DG19)+SUM(DN17:DN19)+SUM(DU17:DU19)</f>
+        <v/>
+      </c>
+      <c r="M47" s="38" t="inlineStr">
+        <is>
+          <t>Opérateurs · mob / demob</t>
+        </is>
+      </c>
+      <c r="N47" s="23" t="n"/>
+      <c r="O47" s="23" t="n"/>
+      <c r="P47" s="23" t="n"/>
+      <c r="Q47" s="23" t="n"/>
+      <c r="R47" s="23" t="n"/>
+      <c r="S47" s="23" t="n"/>
+      <c r="T47" s="23" t="n"/>
+      <c r="U47" s="23" t="n"/>
+      <c r="V47" s="23" t="n"/>
+      <c r="W47" s="23" t="n"/>
+      <c r="X47" s="23" t="n"/>
+      <c r="Y47" s="23" t="n"/>
+      <c r="Z47" s="23" t="n"/>
+      <c r="AA47" s="23" t="n"/>
+      <c r="AB47" s="23" t="n"/>
+      <c r="AC47" s="23" t="n"/>
+      <c r="AD47" s="23" t="n"/>
+      <c r="AE47" s="29">
+        <f>IF(N($DD$9)=0,"",SUM(DG17:DG19))</f>
+        <v/>
+      </c>
+      <c r="AF47" s="23" t="n"/>
+      <c r="AG47" s="23" t="n"/>
+      <c r="AH47" s="23" t="n"/>
+      <c r="AI47" s="23" t="n"/>
+      <c r="AJ47" s="23" t="n"/>
+      <c r="AK47" s="23" t="n"/>
+      <c r="AL47" s="23" t="n"/>
+      <c r="AR47" s="38" t="inlineStr">
+        <is>
+          <t>Opérateurs · mob / demob</t>
+        </is>
+      </c>
+      <c r="AS47" s="23" t="n"/>
+      <c r="AT47" s="23" t="n"/>
+      <c r="AU47" s="23" t="n"/>
+      <c r="AV47" s="23" t="n"/>
+      <c r="AW47" s="23" t="n"/>
+      <c r="AX47" s="23" t="n"/>
+      <c r="AY47" s="23" t="n"/>
+      <c r="AZ47" s="23" t="n"/>
+      <c r="BA47" s="23" t="n"/>
+      <c r="BB47" s="23" t="n"/>
+      <c r="BC47" s="23" t="n"/>
+      <c r="BD47" s="23" t="n"/>
+      <c r="BE47" s="23" t="n"/>
+      <c r="BF47" s="23" t="n"/>
+      <c r="BG47" s="23" t="n"/>
+      <c r="BH47" s="23" t="n"/>
+      <c r="BI47" s="23" t="n"/>
+      <c r="BJ47" s="29">
+        <f>IF(N($DE$9)=0,"",SUM(DN17:DN19))</f>
+        <v/>
+      </c>
+      <c r="BK47" s="23" t="n"/>
+      <c r="BL47" s="23" t="n"/>
+      <c r="BM47" s="23" t="n"/>
+      <c r="BN47" s="23" t="n"/>
+      <c r="BO47" s="23" t="n"/>
+      <c r="BP47" s="23" t="n"/>
+      <c r="BQ47" s="23" t="n"/>
+      <c r="BW47" s="38" t="inlineStr">
+        <is>
+          <t>Opérateurs · mob / demob</t>
+        </is>
+      </c>
+      <c r="BX47" s="23" t="n"/>
+      <c r="BY47" s="23" t="n"/>
+      <c r="BZ47" s="23" t="n"/>
+      <c r="CA47" s="23" t="n"/>
+      <c r="CB47" s="23" t="n"/>
+      <c r="CC47" s="23" t="n"/>
+      <c r="CD47" s="23" t="n"/>
+      <c r="CE47" s="23" t="n"/>
+      <c r="CF47" s="23" t="n"/>
+      <c r="CG47" s="23" t="n"/>
+      <c r="CH47" s="23" t="n"/>
+      <c r="CI47" s="23" t="n"/>
+      <c r="CJ47" s="23" t="n"/>
+      <c r="CK47" s="23" t="n"/>
+      <c r="CL47" s="23" t="n"/>
+      <c r="CM47" s="23" t="n"/>
+      <c r="CN47" s="23" t="n"/>
+      <c r="CO47" s="29">
+        <f>IF(N($DF$9)=0,"",SUM(DU17:DU19))</f>
+        <v/>
+      </c>
+      <c r="CP47" s="23" t="n"/>
+      <c r="CQ47" s="23" t="n"/>
+      <c r="CR47" s="23" t="n"/>
+      <c r="CS47" s="23" t="n"/>
+      <c r="CT47" s="23" t="n"/>
+      <c r="CU47" s="23" t="n"/>
+      <c r="CV47" s="23" t="n"/>
     </row>
-    <row r="48" ht="26" customHeight="1">
-      <c r="A48" s="38" t="inlineStr">
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="35" t="inlineStr">
+        <is>
+          <t>Location du matériel (stand-by + opérations)</t>
+        </is>
+      </c>
+      <c r="B48" s="23" t="n"/>
+      <c r="C48" s="23" t="n"/>
+      <c r="D48" s="23" t="n"/>
+      <c r="E48" s="23" t="n"/>
+      <c r="F48" s="23" t="n"/>
+      <c r="G48" s="36" t="inlineStr">
+        <is>
+          <t>904XRENTALEQUIPMT</t>
+        </is>
+      </c>
+      <c r="H48" s="23" t="n"/>
+      <c r="I48" s="23" t="n"/>
+      <c r="J48" s="23" t="n"/>
+      <c r="K48" s="23" t="n"/>
+      <c r="L48" s="37">
+        <f>SUM(DF22:DF33)+SUM(DM22:DM33)+SUM(DT22:DT33)</f>
+        <v/>
+      </c>
+      <c r="M48" s="38" t="inlineStr">
+        <is>
+          <t>Location du matériel</t>
+        </is>
+      </c>
+      <c r="N48" s="23" t="n"/>
+      <c r="O48" s="23" t="n"/>
+      <c r="P48" s="23" t="n"/>
+      <c r="Q48" s="23" t="n"/>
+      <c r="R48" s="23" t="n"/>
+      <c r="S48" s="23" t="n"/>
+      <c r="T48" s="23" t="n"/>
+      <c r="U48" s="23" t="n"/>
+      <c r="V48" s="23" t="n"/>
+      <c r="W48" s="23" t="n"/>
+      <c r="X48" s="23" t="n"/>
+      <c r="Y48" s="23" t="n"/>
+      <c r="Z48" s="23" t="n"/>
+      <c r="AA48" s="23" t="n"/>
+      <c r="AB48" s="23" t="n"/>
+      <c r="AC48" s="23" t="n"/>
+      <c r="AD48" s="23" t="n"/>
+      <c r="AE48" s="29">
+        <f>IF(N($DD$9)=0,"",SUM(DF22:DF33))</f>
+        <v/>
+      </c>
+      <c r="AF48" s="23" t="n"/>
+      <c r="AG48" s="23" t="n"/>
+      <c r="AH48" s="23" t="n"/>
+      <c r="AI48" s="23" t="n"/>
+      <c r="AJ48" s="23" t="n"/>
+      <c r="AK48" s="23" t="n"/>
+      <c r="AL48" s="23" t="n"/>
+      <c r="AR48" s="38" t="inlineStr">
+        <is>
+          <t>Location du matériel</t>
+        </is>
+      </c>
+      <c r="AS48" s="23" t="n"/>
+      <c r="AT48" s="23" t="n"/>
+      <c r="AU48" s="23" t="n"/>
+      <c r="AV48" s="23" t="n"/>
+      <c r="AW48" s="23" t="n"/>
+      <c r="AX48" s="23" t="n"/>
+      <c r="AY48" s="23" t="n"/>
+      <c r="AZ48" s="23" t="n"/>
+      <c r="BA48" s="23" t="n"/>
+      <c r="BB48" s="23" t="n"/>
+      <c r="BC48" s="23" t="n"/>
+      <c r="BD48" s="23" t="n"/>
+      <c r="BE48" s="23" t="n"/>
+      <c r="BF48" s="23" t="n"/>
+      <c r="BG48" s="23" t="n"/>
+      <c r="BH48" s="23" t="n"/>
+      <c r="BI48" s="23" t="n"/>
+      <c r="BJ48" s="29">
+        <f>IF(N($DE$9)=0,"",SUM(DM22:DM33))</f>
+        <v/>
+      </c>
+      <c r="BK48" s="23" t="n"/>
+      <c r="BL48" s="23" t="n"/>
+      <c r="BM48" s="23" t="n"/>
+      <c r="BN48" s="23" t="n"/>
+      <c r="BO48" s="23" t="n"/>
+      <c r="BP48" s="23" t="n"/>
+      <c r="BQ48" s="23" t="n"/>
+      <c r="BW48" s="38" t="inlineStr">
+        <is>
+          <t>Location du matériel</t>
+        </is>
+      </c>
+      <c r="BX48" s="23" t="n"/>
+      <c r="BY48" s="23" t="n"/>
+      <c r="BZ48" s="23" t="n"/>
+      <c r="CA48" s="23" t="n"/>
+      <c r="CB48" s="23" t="n"/>
+      <c r="CC48" s="23" t="n"/>
+      <c r="CD48" s="23" t="n"/>
+      <c r="CE48" s="23" t="n"/>
+      <c r="CF48" s="23" t="n"/>
+      <c r="CG48" s="23" t="n"/>
+      <c r="CH48" s="23" t="n"/>
+      <c r="CI48" s="23" t="n"/>
+      <c r="CJ48" s="23" t="n"/>
+      <c r="CK48" s="23" t="n"/>
+      <c r="CL48" s="23" t="n"/>
+      <c r="CM48" s="23" t="n"/>
+      <c r="CN48" s="23" t="n"/>
+      <c r="CO48" s="29">
+        <f>IF(N($DF$9)=0,"",SUM(DT22:DT33))</f>
+        <v/>
+      </c>
+      <c r="CP48" s="23" t="n"/>
+      <c r="CQ48" s="23" t="n"/>
+      <c r="CR48" s="23" t="n"/>
+      <c r="CS48" s="23" t="n"/>
+      <c r="CT48" s="23" t="n"/>
+      <c r="CU48" s="23" t="n"/>
+      <c r="CV48" s="23" t="n"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="35" t="inlineStr">
+        <is>
+          <t>Utilisation charge et inspection (UC, une seule fois)</t>
+        </is>
+      </c>
+      <c r="B49" s="23" t="n"/>
+      <c r="C49" s="23" t="n"/>
+      <c r="D49" s="23" t="n"/>
+      <c r="E49" s="23" t="n"/>
+      <c r="F49" s="23" t="n"/>
+      <c r="G49" s="36" t="inlineStr">
+        <is>
+          <t>905XUC</t>
+        </is>
+      </c>
+      <c r="H49" s="23" t="n"/>
+      <c r="I49" s="23" t="n"/>
+      <c r="J49" s="23" t="n"/>
+      <c r="K49" s="23" t="n"/>
+      <c r="L49" s="37">
+        <f>SUM(DG22:DG33)+SUM(DN22:DN33)+SUM(DU22:DU33)</f>
+        <v/>
+      </c>
+      <c r="M49" s="38" t="inlineStr">
+        <is>
+          <t>UC et inspection</t>
+        </is>
+      </c>
+      <c r="N49" s="23" t="n"/>
+      <c r="O49" s="23" t="n"/>
+      <c r="P49" s="23" t="n"/>
+      <c r="Q49" s="23" t="n"/>
+      <c r="R49" s="23" t="n"/>
+      <c r="S49" s="23" t="n"/>
+      <c r="T49" s="23" t="n"/>
+      <c r="U49" s="23" t="n"/>
+      <c r="V49" s="23" t="n"/>
+      <c r="W49" s="23" t="n"/>
+      <c r="X49" s="23" t="n"/>
+      <c r="Y49" s="23" t="n"/>
+      <c r="Z49" s="23" t="n"/>
+      <c r="AA49" s="23" t="n"/>
+      <c r="AB49" s="23" t="n"/>
+      <c r="AC49" s="23" t="n"/>
+      <c r="AD49" s="23" t="n"/>
+      <c r="AE49" s="29">
+        <f>IF(N($DD$9)=0,"",SUM(DG22:DG33))</f>
+        <v/>
+      </c>
+      <c r="AF49" s="23" t="n"/>
+      <c r="AG49" s="23" t="n"/>
+      <c r="AH49" s="23" t="n"/>
+      <c r="AI49" s="23" t="n"/>
+      <c r="AJ49" s="23" t="n"/>
+      <c r="AK49" s="23" t="n"/>
+      <c r="AL49" s="23" t="n"/>
+      <c r="AR49" s="38" t="inlineStr">
+        <is>
+          <t>UC et inspection</t>
+        </is>
+      </c>
+      <c r="AS49" s="23" t="n"/>
+      <c r="AT49" s="23" t="n"/>
+      <c r="AU49" s="23" t="n"/>
+      <c r="AV49" s="23" t="n"/>
+      <c r="AW49" s="23" t="n"/>
+      <c r="AX49" s="23" t="n"/>
+      <c r="AY49" s="23" t="n"/>
+      <c r="AZ49" s="23" t="n"/>
+      <c r="BA49" s="23" t="n"/>
+      <c r="BB49" s="23" t="n"/>
+      <c r="BC49" s="23" t="n"/>
+      <c r="BD49" s="23" t="n"/>
+      <c r="BE49" s="23" t="n"/>
+      <c r="BF49" s="23" t="n"/>
+      <c r="BG49" s="23" t="n"/>
+      <c r="BH49" s="23" t="n"/>
+      <c r="BI49" s="23" t="n"/>
+      <c r="BJ49" s="29">
+        <f>IF(N($DE$9)=0,"",SUM(DN22:DN33))</f>
+        <v/>
+      </c>
+      <c r="BK49" s="23" t="n"/>
+      <c r="BL49" s="23" t="n"/>
+      <c r="BM49" s="23" t="n"/>
+      <c r="BN49" s="23" t="n"/>
+      <c r="BO49" s="23" t="n"/>
+      <c r="BP49" s="23" t="n"/>
+      <c r="BQ49" s="23" t="n"/>
+      <c r="BW49" s="38" t="inlineStr">
+        <is>
+          <t>UC et inspection</t>
+        </is>
+      </c>
+      <c r="BX49" s="23" t="n"/>
+      <c r="BY49" s="23" t="n"/>
+      <c r="BZ49" s="23" t="n"/>
+      <c r="CA49" s="23" t="n"/>
+      <c r="CB49" s="23" t="n"/>
+      <c r="CC49" s="23" t="n"/>
+      <c r="CD49" s="23" t="n"/>
+      <c r="CE49" s="23" t="n"/>
+      <c r="CF49" s="23" t="n"/>
+      <c r="CG49" s="23" t="n"/>
+      <c r="CH49" s="23" t="n"/>
+      <c r="CI49" s="23" t="n"/>
+      <c r="CJ49" s="23" t="n"/>
+      <c r="CK49" s="23" t="n"/>
+      <c r="CL49" s="23" t="n"/>
+      <c r="CM49" s="23" t="n"/>
+      <c r="CN49" s="23" t="n"/>
+      <c r="CO49" s="29">
+        <f>IF(N($DF$9)=0,"",SUM(DU22:DU33))</f>
+        <v/>
+      </c>
+      <c r="CP49" s="23" t="n"/>
+      <c r="CQ49" s="23" t="n"/>
+      <c r="CR49" s="23" t="n"/>
+      <c r="CS49" s="23" t="n"/>
+      <c r="CT49" s="23" t="n"/>
+      <c r="CU49" s="23" t="n"/>
+      <c r="CV49" s="23" t="n"/>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="35" t="inlineStr">
+        <is>
+          <t>Valeur de remplacement et restocking</t>
+        </is>
+      </c>
+      <c r="B50" s="23" t="n"/>
+      <c r="C50" s="23" t="n"/>
+      <c r="D50" s="23" t="n"/>
+      <c r="E50" s="23" t="n"/>
+      <c r="F50" s="23" t="n"/>
+      <c r="G50" s="36" t="inlineStr"/>
+      <c r="H50" s="23" t="n"/>
+      <c r="I50" s="23" t="n"/>
+      <c r="J50" s="23" t="n"/>
+      <c r="K50" s="23" t="n"/>
+      <c r="L50" s="37">
+        <f>SUM(DH22:DH33)+SUM(DO22:DO33)+SUM(DV22:DV33)</f>
+        <v/>
+      </c>
+      <c r="M50" s="38" t="inlineStr">
+        <is>
+          <t>Valeur de remplacement, restocking</t>
+        </is>
+      </c>
+      <c r="N50" s="23" t="n"/>
+      <c r="O50" s="23" t="n"/>
+      <c r="P50" s="23" t="n"/>
+      <c r="Q50" s="23" t="n"/>
+      <c r="R50" s="23" t="n"/>
+      <c r="S50" s="23" t="n"/>
+      <c r="T50" s="23" t="n"/>
+      <c r="U50" s="23" t="n"/>
+      <c r="V50" s="23" t="n"/>
+      <c r="W50" s="23" t="n"/>
+      <c r="X50" s="23" t="n"/>
+      <c r="Y50" s="23" t="n"/>
+      <c r="Z50" s="23" t="n"/>
+      <c r="AA50" s="23" t="n"/>
+      <c r="AB50" s="23" t="n"/>
+      <c r="AC50" s="23" t="n"/>
+      <c r="AD50" s="23" t="n"/>
+      <c r="AE50" s="29">
+        <f>IF(N($DD$9)=0,"",SUM(DH22:DH33))</f>
+        <v/>
+      </c>
+      <c r="AF50" s="23" t="n"/>
+      <c r="AG50" s="23" t="n"/>
+      <c r="AH50" s="23" t="n"/>
+      <c r="AI50" s="23" t="n"/>
+      <c r="AJ50" s="23" t="n"/>
+      <c r="AK50" s="23" t="n"/>
+      <c r="AL50" s="23" t="n"/>
+      <c r="AR50" s="38" t="inlineStr">
+        <is>
+          <t>Valeur de remplacement, restocking</t>
+        </is>
+      </c>
+      <c r="AS50" s="23" t="n"/>
+      <c r="AT50" s="23" t="n"/>
+      <c r="AU50" s="23" t="n"/>
+      <c r="AV50" s="23" t="n"/>
+      <c r="AW50" s="23" t="n"/>
+      <c r="AX50" s="23" t="n"/>
+      <c r="AY50" s="23" t="n"/>
+      <c r="AZ50" s="23" t="n"/>
+      <c r="BA50" s="23" t="n"/>
+      <c r="BB50" s="23" t="n"/>
+      <c r="BC50" s="23" t="n"/>
+      <c r="BD50" s="23" t="n"/>
+      <c r="BE50" s="23" t="n"/>
+      <c r="BF50" s="23" t="n"/>
+      <c r="BG50" s="23" t="n"/>
+      <c r="BH50" s="23" t="n"/>
+      <c r="BI50" s="23" t="n"/>
+      <c r="BJ50" s="29">
+        <f>IF(N($DE$9)=0,"",SUM(DO22:DO33))</f>
+        <v/>
+      </c>
+      <c r="BK50" s="23" t="n"/>
+      <c r="BL50" s="23" t="n"/>
+      <c r="BM50" s="23" t="n"/>
+      <c r="BN50" s="23" t="n"/>
+      <c r="BO50" s="23" t="n"/>
+      <c r="BP50" s="23" t="n"/>
+      <c r="BQ50" s="23" t="n"/>
+      <c r="BW50" s="38" t="inlineStr">
+        <is>
+          <t>Valeur de remplacement, restocking</t>
+        </is>
+      </c>
+      <c r="BX50" s="23" t="n"/>
+      <c r="BY50" s="23" t="n"/>
+      <c r="BZ50" s="23" t="n"/>
+      <c r="CA50" s="23" t="n"/>
+      <c r="CB50" s="23" t="n"/>
+      <c r="CC50" s="23" t="n"/>
+      <c r="CD50" s="23" t="n"/>
+      <c r="CE50" s="23" t="n"/>
+      <c r="CF50" s="23" t="n"/>
+      <c r="CG50" s="23" t="n"/>
+      <c r="CH50" s="23" t="n"/>
+      <c r="CI50" s="23" t="n"/>
+      <c r="CJ50" s="23" t="n"/>
+      <c r="CK50" s="23" t="n"/>
+      <c r="CL50" s="23" t="n"/>
+      <c r="CM50" s="23" t="n"/>
+      <c r="CN50" s="23" t="n"/>
+      <c r="CO50" s="29">
+        <f>IF(N($DF$9)=0,"",SUM(DV22:DV33))</f>
+        <v/>
+      </c>
+      <c r="CP50" s="23" t="n"/>
+      <c r="CQ50" s="23" t="n"/>
+      <c r="CR50" s="23" t="n"/>
+      <c r="CS50" s="23" t="n"/>
+      <c r="CT50" s="23" t="n"/>
+      <c r="CU50" s="23" t="n"/>
+      <c r="CV50" s="23" t="n"/>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="35" t="inlineStr">
+        <is>
+          <t>Serrages</t>
+        </is>
+      </c>
+      <c r="B51" s="23" t="n"/>
+      <c r="C51" s="23" t="n"/>
+      <c r="D51" s="23" t="n"/>
+      <c r="E51" s="23" t="n"/>
+      <c r="F51" s="23" t="n"/>
+      <c r="G51" s="36" t="inlineStr"/>
+      <c r="H51" s="23" t="n"/>
+      <c r="I51" s="23" t="n"/>
+      <c r="J51" s="23" t="n"/>
+      <c r="K51" s="23" t="n"/>
+      <c r="L51" s="37">
+        <f>SUM(L36:L37)</f>
+        <v/>
+      </c>
+      <c r="M51" s="38" t="inlineStr">
+        <is>
+          <t>Serrages</t>
+        </is>
+      </c>
+      <c r="N51" s="23" t="n"/>
+      <c r="O51" s="23" t="n"/>
+      <c r="P51" s="23" t="n"/>
+      <c r="Q51" s="23" t="n"/>
+      <c r="R51" s="23" t="n"/>
+      <c r="S51" s="23" t="n"/>
+      <c r="T51" s="23" t="n"/>
+      <c r="U51" s="23" t="n"/>
+      <c r="V51" s="23" t="n"/>
+      <c r="W51" s="23" t="n"/>
+      <c r="X51" s="23" t="n"/>
+      <c r="Y51" s="23" t="n"/>
+      <c r="Z51" s="23" t="n"/>
+      <c r="AA51" s="23" t="n"/>
+      <c r="AB51" s="23" t="n"/>
+      <c r="AC51" s="23" t="n"/>
+      <c r="AD51" s="23" t="n"/>
+      <c r="AE51" s="29">
+        <f>IF(N($DD$9)=0,"",SUM(DY36:DY37))</f>
+        <v/>
+      </c>
+      <c r="AF51" s="23" t="n"/>
+      <c r="AG51" s="23" t="n"/>
+      <c r="AH51" s="23" t="n"/>
+      <c r="AI51" s="23" t="n"/>
+      <c r="AJ51" s="23" t="n"/>
+      <c r="AK51" s="23" t="n"/>
+      <c r="AL51" s="23" t="n"/>
+      <c r="AR51" s="38" t="inlineStr">
+        <is>
+          <t>Serrages</t>
+        </is>
+      </c>
+      <c r="AS51" s="23" t="n"/>
+      <c r="AT51" s="23" t="n"/>
+      <c r="AU51" s="23" t="n"/>
+      <c r="AV51" s="23" t="n"/>
+      <c r="AW51" s="23" t="n"/>
+      <c r="AX51" s="23" t="n"/>
+      <c r="AY51" s="23" t="n"/>
+      <c r="AZ51" s="23" t="n"/>
+      <c r="BA51" s="23" t="n"/>
+      <c r="BB51" s="23" t="n"/>
+      <c r="BC51" s="23" t="n"/>
+      <c r="BD51" s="23" t="n"/>
+      <c r="BE51" s="23" t="n"/>
+      <c r="BF51" s="23" t="n"/>
+      <c r="BG51" s="23" t="n"/>
+      <c r="BH51" s="23" t="n"/>
+      <c r="BI51" s="23" t="n"/>
+      <c r="BJ51" s="29">
+        <f>IF(N($DE$9)=0,"",SUM(DZ36:DZ37))</f>
+        <v/>
+      </c>
+      <c r="BK51" s="23" t="n"/>
+      <c r="BL51" s="23" t="n"/>
+      <c r="BM51" s="23" t="n"/>
+      <c r="BN51" s="23" t="n"/>
+      <c r="BO51" s="23" t="n"/>
+      <c r="BP51" s="23" t="n"/>
+      <c r="BQ51" s="23" t="n"/>
+      <c r="BW51" s="38" t="inlineStr">
+        <is>
+          <t>Serrages</t>
+        </is>
+      </c>
+      <c r="BX51" s="23" t="n"/>
+      <c r="BY51" s="23" t="n"/>
+      <c r="BZ51" s="23" t="n"/>
+      <c r="CA51" s="23" t="n"/>
+      <c r="CB51" s="23" t="n"/>
+      <c r="CC51" s="23" t="n"/>
+      <c r="CD51" s="23" t="n"/>
+      <c r="CE51" s="23" t="n"/>
+      <c r="CF51" s="23" t="n"/>
+      <c r="CG51" s="23" t="n"/>
+      <c r="CH51" s="23" t="n"/>
+      <c r="CI51" s="23" t="n"/>
+      <c r="CJ51" s="23" t="n"/>
+      <c r="CK51" s="23" t="n"/>
+      <c r="CL51" s="23" t="n"/>
+      <c r="CM51" s="23" t="n"/>
+      <c r="CN51" s="23" t="n"/>
+      <c r="CO51" s="29">
+        <f>IF(N($DF$9)=0,"",SUM(EA36:EA37))</f>
+        <v/>
+      </c>
+      <c r="CP51" s="23" t="n"/>
+      <c r="CQ51" s="23" t="n"/>
+      <c r="CR51" s="23" t="n"/>
+      <c r="CS51" s="23" t="n"/>
+      <c r="CT51" s="23" t="n"/>
+      <c r="CU51" s="23" t="n"/>
+      <c r="CV51" s="23" t="n"/>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="35" t="inlineStr">
+        <is>
+          <t>Transport et autres frais</t>
+        </is>
+      </c>
+      <c r="B52" s="23" t="n"/>
+      <c r="C52" s="23" t="n"/>
+      <c r="D52" s="23" t="n"/>
+      <c r="E52" s="23" t="n"/>
+      <c r="F52" s="23" t="n"/>
+      <c r="G52" s="36" t="inlineStr">
+        <is>
+          <t>900XMOBDEMOB</t>
+        </is>
+      </c>
+      <c r="H52" s="23" t="n"/>
+      <c r="I52" s="23" t="n"/>
+      <c r="J52" s="23" t="n"/>
+      <c r="K52" s="23" t="n"/>
+      <c r="L52" s="37">
+        <f>SUM(L40:L42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="26" customHeight="1">
+      <c r="A53" s="39" t="inlineStr">
         <is>
           <t>TOTAL HT À FACTURER</t>
         </is>
       </c>
-      <c r="B48" s="39" t="n"/>
-      <c r="C48" s="39" t="n"/>
-      <c r="D48" s="39" t="n"/>
-      <c r="E48" s="39" t="n"/>
-      <c r="F48" s="39" t="n"/>
-      <c r="G48" s="39" t="n"/>
-      <c r="H48" s="39" t="n"/>
-      <c r="I48" s="39" t="n"/>
-      <c r="J48" s="39" t="n"/>
-      <c r="K48" s="39" t="n"/>
-      <c r="L48" s="40">
-        <f>SUM(L42:L47)</f>
-        <v/>
-      </c>
-      <c r="M48" s="41">
+      <c r="B53" s="40" t="n"/>
+      <c r="C53" s="40" t="n"/>
+      <c r="D53" s="40" t="n"/>
+      <c r="E53" s="40" t="n"/>
+      <c r="F53" s="40" t="n"/>
+      <c r="G53" s="40" t="n"/>
+      <c r="H53" s="40" t="n"/>
+      <c r="I53" s="40" t="n"/>
+      <c r="J53" s="40" t="n"/>
+      <c r="K53" s="40" t="n"/>
+      <c r="L53" s="41">
+        <f>SUM(L46:L52)</f>
+        <v/>
+      </c>
+      <c r="M53" s="42">
         <f>IF(N($DD$9)=0,"","TOTAL À FACTURER · "&amp;CHOOSE(MONTH($C$9),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR($C$9))</f>
         <v/>
       </c>
-      <c r="N48" s="42" t="n"/>
-      <c r="O48" s="42" t="n"/>
-      <c r="P48" s="42" t="n"/>
-      <c r="Q48" s="42" t="n"/>
-      <c r="R48" s="42" t="n"/>
-      <c r="S48" s="42" t="n"/>
-      <c r="T48" s="42" t="n"/>
-      <c r="U48" s="42" t="n"/>
-      <c r="V48" s="42" t="n"/>
-      <c r="W48" s="42" t="n"/>
-      <c r="X48" s="42" t="n"/>
-      <c r="Y48" s="42" t="n"/>
-      <c r="Z48" s="42" t="n"/>
-      <c r="AA48" s="42" t="n"/>
-      <c r="AB48" s="42" t="n"/>
-      <c r="AC48" s="42" t="n"/>
-      <c r="AD48" s="42" t="n"/>
-      <c r="AE48" s="43">
-        <f>IF(N($DD$9)=0,"",SUM(AE42:AE46))</f>
-        <v/>
-      </c>
-      <c r="AF48" s="42" t="n"/>
-      <c r="AG48" s="42" t="n"/>
-      <c r="AH48" s="42" t="n"/>
-      <c r="AI48" s="42" t="n"/>
-      <c r="AJ48" s="42" t="n"/>
-      <c r="AK48" s="42" t="n"/>
-      <c r="AL48" s="42" t="n"/>
-      <c r="AR48" s="41">
+      <c r="N53" s="43" t="n"/>
+      <c r="O53" s="43" t="n"/>
+      <c r="P53" s="43" t="n"/>
+      <c r="Q53" s="43" t="n"/>
+      <c r="R53" s="43" t="n"/>
+      <c r="S53" s="43" t="n"/>
+      <c r="T53" s="43" t="n"/>
+      <c r="U53" s="43" t="n"/>
+      <c r="V53" s="43" t="n"/>
+      <c r="W53" s="43" t="n"/>
+      <c r="X53" s="43" t="n"/>
+      <c r="Y53" s="43" t="n"/>
+      <c r="Z53" s="43" t="n"/>
+      <c r="AA53" s="43" t="n"/>
+      <c r="AB53" s="43" t="n"/>
+      <c r="AC53" s="43" t="n"/>
+      <c r="AD53" s="43" t="n"/>
+      <c r="AE53" s="44">
+        <f>IF(N($DD$9)=0,"",SUM(AE46:AE51))</f>
+        <v/>
+      </c>
+      <c r="AF53" s="43" t="n"/>
+      <c r="AG53" s="43" t="n"/>
+      <c r="AH53" s="43" t="n"/>
+      <c r="AI53" s="43" t="n"/>
+      <c r="AJ53" s="43" t="n"/>
+      <c r="AK53" s="43" t="n"/>
+      <c r="AL53" s="43" t="n"/>
+      <c r="AR53" s="42">
         <f>IF(N($DE$9)=0,"","TOTAL À FACTURER · "&amp;CHOOSE(MONTH(DATE(YEAR($C$9),MONTH($C$9)+1,1)),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR(DATE(YEAR($C$9),MONTH($C$9)+1,1)))</f>
         <v/>
       </c>
-      <c r="AS48" s="42" t="n"/>
-      <c r="AT48" s="42" t="n"/>
-      <c r="AU48" s="42" t="n"/>
-      <c r="AV48" s="42" t="n"/>
-      <c r="AW48" s="42" t="n"/>
-      <c r="AX48" s="42" t="n"/>
-      <c r="AY48" s="42" t="n"/>
-      <c r="AZ48" s="42" t="n"/>
-      <c r="BA48" s="42" t="n"/>
-      <c r="BB48" s="42" t="n"/>
-      <c r="BC48" s="42" t="n"/>
-      <c r="BD48" s="42" t="n"/>
-      <c r="BE48" s="42" t="n"/>
-      <c r="BF48" s="42" t="n"/>
-      <c r="BG48" s="42" t="n"/>
-      <c r="BH48" s="42" t="n"/>
-      <c r="BI48" s="42" t="n"/>
-      <c r="BJ48" s="43">
-        <f>IF(N($DE$9)=0,"",SUM(BJ42:BJ46))</f>
-        <v/>
-      </c>
-      <c r="BK48" s="42" t="n"/>
-      <c r="BL48" s="42" t="n"/>
-      <c r="BM48" s="42" t="n"/>
-      <c r="BN48" s="42" t="n"/>
-      <c r="BO48" s="42" t="n"/>
-      <c r="BP48" s="42" t="n"/>
-      <c r="BQ48" s="42" t="n"/>
-      <c r="BW48" s="41">
+      <c r="AS53" s="43" t="n"/>
+      <c r="AT53" s="43" t="n"/>
+      <c r="AU53" s="43" t="n"/>
+      <c r="AV53" s="43" t="n"/>
+      <c r="AW53" s="43" t="n"/>
+      <c r="AX53" s="43" t="n"/>
+      <c r="AY53" s="43" t="n"/>
+      <c r="AZ53" s="43" t="n"/>
+      <c r="BA53" s="43" t="n"/>
+      <c r="BB53" s="43" t="n"/>
+      <c r="BC53" s="43" t="n"/>
+      <c r="BD53" s="43" t="n"/>
+      <c r="BE53" s="43" t="n"/>
+      <c r="BF53" s="43" t="n"/>
+      <c r="BG53" s="43" t="n"/>
+      <c r="BH53" s="43" t="n"/>
+      <c r="BI53" s="43" t="n"/>
+      <c r="BJ53" s="44">
+        <f>IF(N($DE$9)=0,"",SUM(BJ46:BJ51))</f>
+        <v/>
+      </c>
+      <c r="BK53" s="43" t="n"/>
+      <c r="BL53" s="43" t="n"/>
+      <c r="BM53" s="43" t="n"/>
+      <c r="BN53" s="43" t="n"/>
+      <c r="BO53" s="43" t="n"/>
+      <c r="BP53" s="43" t="n"/>
+      <c r="BQ53" s="43" t="n"/>
+      <c r="BW53" s="42">
         <f>IF(N($DF$9)=0,"","TOTAL À FACTURER · "&amp;CHOOSE(MONTH(DATE(YEAR($C$9),MONTH($C$9)+2,1)),"JANVIER","FÉVRIER","MARS","AVRIL","MAI","JUIN","JUILLET","AOÛT","SEPTEMBRE","OCTOBRE","NOVEMBRE","DÉCEMBRE")&amp;" "&amp;YEAR(DATE(YEAR($C$9),MONTH($C$9)+2,1)))</f>
         <v/>
       </c>
-      <c r="BX48" s="42" t="n"/>
-      <c r="BY48" s="42" t="n"/>
-      <c r="BZ48" s="42" t="n"/>
-      <c r="CA48" s="42" t="n"/>
-      <c r="CB48" s="42" t="n"/>
-      <c r="CC48" s="42" t="n"/>
-      <c r="CD48" s="42" t="n"/>
-      <c r="CE48" s="42" t="n"/>
-      <c r="CF48" s="42" t="n"/>
-      <c r="CG48" s="42" t="n"/>
-      <c r="CH48" s="42" t="n"/>
-      <c r="CI48" s="42" t="n"/>
-      <c r="CJ48" s="42" t="n"/>
-      <c r="CK48" s="42" t="n"/>
-      <c r="CL48" s="42" t="n"/>
-      <c r="CM48" s="42" t="n"/>
-      <c r="CN48" s="42" t="n"/>
-      <c r="CO48" s="43">
-        <f>IF(N($DF$9)=0,"",SUM(CO42:CO46))</f>
-        <v/>
-      </c>
-      <c r="CP48" s="42" t="n"/>
-      <c r="CQ48" s="42" t="n"/>
-      <c r="CR48" s="42" t="n"/>
-      <c r="CS48" s="42" t="n"/>
-      <c r="CT48" s="42" t="n"/>
-      <c r="CU48" s="42" t="n"/>
-      <c r="CV48" s="42" t="n"/>
+      <c r="BX53" s="43" t="n"/>
+      <c r="BY53" s="43" t="n"/>
+      <c r="BZ53" s="43" t="n"/>
+      <c r="CA53" s="43" t="n"/>
+      <c r="CB53" s="43" t="n"/>
+      <c r="CC53" s="43" t="n"/>
+      <c r="CD53" s="43" t="n"/>
+      <c r="CE53" s="43" t="n"/>
+      <c r="CF53" s="43" t="n"/>
+      <c r="CG53" s="43" t="n"/>
+      <c r="CH53" s="43" t="n"/>
+      <c r="CI53" s="43" t="n"/>
+      <c r="CJ53" s="43" t="n"/>
+      <c r="CK53" s="43" t="n"/>
+      <c r="CL53" s="43" t="n"/>
+      <c r="CM53" s="43" t="n"/>
+      <c r="CN53" s="43" t="n"/>
+      <c r="CO53" s="44">
+        <f>IF(N($DF$9)=0,"",SUM(CO46:CO51))</f>
+        <v/>
+      </c>
+      <c r="CP53" s="43" t="n"/>
+      <c r="CQ53" s="43" t="n"/>
+      <c r="CR53" s="43" t="n"/>
+      <c r="CS53" s="43" t="n"/>
+      <c r="CT53" s="43" t="n"/>
+      <c r="CU53" s="43" t="n"/>
+      <c r="CV53" s="43" t="n"/>
     </row>
-    <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="44" t="inlineStr">
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="45" t="inlineStr">
         <is>
           <t>Gratuit (FOC), pour information</t>
         </is>
       </c>
-      <c r="L49" s="45">
+      <c r="L54" s="46">
         <f>SUM(DI22:DI33)+SUM(DP22:DP33)+SUM(DW22:DW33)</f>
         <v/>
       </c>
     </row>
-    <row r="51" ht="17" customHeight="1">
-      <c r="A51" s="46" t="inlineStr">
+    <row r="56" ht="17" customHeight="1">
+      <c r="A56" s="47" t="inlineStr">
         <is>
           <t>POUR ENEDRIL · Nom, date, signature</t>
         </is>
       </c>
-      <c r="B51" s="47" t="n"/>
-      <c r="C51" s="47" t="n"/>
-      <c r="D51" s="47" t="n"/>
-      <c r="E51" s="48" t="n"/>
-      <c r="F51" s="46" t="inlineStr">
+      <c r="B56" s="48" t="n"/>
+      <c r="C56" s="48" t="n"/>
+      <c r="D56" s="48" t="n"/>
+      <c r="E56" s="49" t="n"/>
+      <c r="F56" s="47" t="inlineStr">
         <is>
           <t>POUR LE CLIENT · Nom, date, signature, cachet</t>
         </is>
       </c>
-      <c r="G51" s="47" t="n"/>
-      <c r="H51" s="47" t="n"/>
-      <c r="I51" s="47" t="n"/>
-      <c r="J51" s="47" t="n"/>
-      <c r="K51" s="47" t="n"/>
-      <c r="L51" s="48" t="n"/>
+      <c r="G56" s="48" t="n"/>
+      <c r="H56" s="48" t="n"/>
+      <c r="I56" s="48" t="n"/>
+      <c r="J56" s="48" t="n"/>
+      <c r="K56" s="48" t="n"/>
+      <c r="L56" s="49" t="n"/>
     </row>
-    <row r="52" ht="17" customHeight="1">
-      <c r="A52" s="49" t="n"/>
-      <c r="B52" s="50" t="n"/>
-      <c r="C52" s="50" t="n"/>
-      <c r="D52" s="50" t="n"/>
-      <c r="E52" s="51" t="n"/>
-      <c r="F52" s="49" t="n"/>
-      <c r="G52" s="50" t="n"/>
-      <c r="H52" s="50" t="n"/>
-      <c r="I52" s="50" t="n"/>
-      <c r="J52" s="50" t="n"/>
-      <c r="K52" s="50" t="n"/>
-      <c r="L52" s="51" t="n"/>
+    <row r="57" ht="17" customHeight="1">
+      <c r="A57" s="50" t="n"/>
+      <c r="B57" s="51" t="n"/>
+      <c r="C57" s="51" t="n"/>
+      <c r="D57" s="51" t="n"/>
+      <c r="E57" s="52" t="n"/>
+      <c r="F57" s="50" t="n"/>
+      <c r="G57" s="51" t="n"/>
+      <c r="H57" s="51" t="n"/>
+      <c r="I57" s="51" t="n"/>
+      <c r="J57" s="51" t="n"/>
+      <c r="K57" s="51" t="n"/>
+      <c r="L57" s="52" t="n"/>
     </row>
-    <row r="53" ht="17" customHeight="1">
-      <c r="A53" s="52" t="n"/>
-      <c r="B53" s="23" t="n"/>
-      <c r="C53" s="23" t="n"/>
-      <c r="D53" s="23" t="n"/>
-      <c r="E53" s="53" t="n"/>
-      <c r="F53" s="52" t="n"/>
-      <c r="G53" s="23" t="n"/>
-      <c r="H53" s="23" t="n"/>
-      <c r="I53" s="23" t="n"/>
-      <c r="J53" s="23" t="n"/>
-      <c r="K53" s="23" t="n"/>
-      <c r="L53" s="53" t="n"/>
+    <row r="58" ht="17" customHeight="1">
+      <c r="A58" s="53" t="n"/>
+      <c r="B58" s="23" t="n"/>
+      <c r="C58" s="23" t="n"/>
+      <c r="D58" s="23" t="n"/>
+      <c r="E58" s="54" t="n"/>
+      <c r="F58" s="53" t="n"/>
+      <c r="G58" s="23" t="n"/>
+      <c r="H58" s="23" t="n"/>
+      <c r="I58" s="23" t="n"/>
+      <c r="J58" s="23" t="n"/>
+      <c r="K58" s="23" t="n"/>
+      <c r="L58" s="54" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="87">
-    <mergeCell ref="BJ45:BQ45"/>
+  <mergeCells count="95">
     <mergeCell ref="AR48:BI48"/>
     <mergeCell ref="CO46:CV46"/>
-    <mergeCell ref="BJ42:BQ42"/>
     <mergeCell ref="BW12:DA12"/>
+    <mergeCell ref="A50:F50"/>
     <mergeCell ref="CO48:CV48"/>
-    <mergeCell ref="BJ44:BQ44"/>
+    <mergeCell ref="G48:K48"/>
     <mergeCell ref="A47:F47"/>
+    <mergeCell ref="A54:K54"/>
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="D13:D14"/>
     <mergeCell ref="C6:F6"/>
-    <mergeCell ref="M45:AD45"/>
-    <mergeCell ref="M42:AD42"/>
     <mergeCell ref="F13:F14"/>
-    <mergeCell ref="BW43:CN43"/>
+    <mergeCell ref="CO49:CV49"/>
     <mergeCell ref="H13:H14"/>
-    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="AR51:BI51"/>
+    <mergeCell ref="M47:AD47"/>
     <mergeCell ref="G9:I9"/>
-    <mergeCell ref="BW42:CN42"/>
+    <mergeCell ref="AR50:BI50"/>
     <mergeCell ref="BJ48:BQ48"/>
-    <mergeCell ref="BW44:CN44"/>
-    <mergeCell ref="AR43:BI43"/>
-    <mergeCell ref="M44:AD44"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A53:K53"/>
+    <mergeCell ref="G50:K50"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="BW46:CN46"/>
-    <mergeCell ref="BJ43:BQ43"/>
-    <mergeCell ref="A48:K48"/>
+    <mergeCell ref="CO53:CV53"/>
+    <mergeCell ref="G52:K52"/>
+    <mergeCell ref="M51:AD51"/>
     <mergeCell ref="G6:I6"/>
     <mergeCell ref="E13:E14"/>
     <mergeCell ref="BW48:CN48"/>
     <mergeCell ref="G13:G14"/>
-    <mergeCell ref="G42:K42"/>
-    <mergeCell ref="BW45:CN45"/>
-    <mergeCell ref="A42:F42"/>
-    <mergeCell ref="AE43:AL43"/>
+    <mergeCell ref="BW47:CN47"/>
+    <mergeCell ref="BJ50:BQ50"/>
+    <mergeCell ref="AR53:BI53"/>
     <mergeCell ref="BJ46:BQ46"/>
     <mergeCell ref="C5:F5"/>
-    <mergeCell ref="AE42:AL42"/>
-    <mergeCell ref="AE44:AL44"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="M53:AD53"/>
     <mergeCell ref="A8:B8"/>
+    <mergeCell ref="M50:AD50"/>
     <mergeCell ref="J5:L5"/>
+    <mergeCell ref="BW51:CN51"/>
+    <mergeCell ref="G51:K51"/>
+    <mergeCell ref="BJ47:BQ47"/>
     <mergeCell ref="G8:I8"/>
-    <mergeCell ref="AE45:AL45"/>
+    <mergeCell ref="M49:AD49"/>
+    <mergeCell ref="CO50:CV50"/>
     <mergeCell ref="M48:AD48"/>
     <mergeCell ref="J6:L6"/>
     <mergeCell ref="A46:F46"/>
-    <mergeCell ref="G43:K43"/>
     <mergeCell ref="C8:F8"/>
-    <mergeCell ref="CO43:CV43"/>
-    <mergeCell ref="A49:K49"/>
-    <mergeCell ref="CO42:CV42"/>
     <mergeCell ref="AE46:AL46"/>
     <mergeCell ref="AR12:BV12"/>
+    <mergeCell ref="BJ51:BQ51"/>
+    <mergeCell ref="AE47:AL47"/>
     <mergeCell ref="G5:I5"/>
-    <mergeCell ref="CO44:CV44"/>
-    <mergeCell ref="AR45:BI45"/>
+    <mergeCell ref="BJ49:BQ49"/>
+    <mergeCell ref="CO51:CV51"/>
     <mergeCell ref="A13:A14"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="AE48:AL48"/>
     <mergeCell ref="J8:L8"/>
-    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="AR47:BI47"/>
     <mergeCell ref="M1:AQ1"/>
-    <mergeCell ref="AR44:BI44"/>
-    <mergeCell ref="AR42:BI42"/>
-    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="BW50:CN50"/>
     <mergeCell ref="G47:K47"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="F51:L53"/>
+    <mergeCell ref="BJ53:BQ53"/>
+    <mergeCell ref="AE49:AL49"/>
     <mergeCell ref="J9:L9"/>
     <mergeCell ref="G46:K46"/>
+    <mergeCell ref="BW49:CN49"/>
     <mergeCell ref="M12:AQ12"/>
     <mergeCell ref="J13:J14"/>
     <mergeCell ref="L13:L14"/>
+    <mergeCell ref="AE51:AL51"/>
+    <mergeCell ref="AE50:AL50"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A51:E53"/>
+    <mergeCell ref="AR49:BI49"/>
     <mergeCell ref="M46:AD46"/>
-    <mergeCell ref="A43:F43"/>
+    <mergeCell ref="BW53:CN53"/>
+    <mergeCell ref="G49:K49"/>
+    <mergeCell ref="A52:F52"/>
     <mergeCell ref="A10:L10"/>
     <mergeCell ref="I13:I14"/>
     <mergeCell ref="K13:K14"/>
-    <mergeCell ref="CO45:CV45"/>
+    <mergeCell ref="A56:E58"/>
+    <mergeCell ref="AE53:AL53"/>
     <mergeCell ref="C13:C14"/>
     <mergeCell ref="C9:F9"/>
-    <mergeCell ref="M43:AD43"/>
     <mergeCell ref="M2:AQ2"/>
     <mergeCell ref="A11:L11"/>
+    <mergeCell ref="CO47:CV47"/>
     <mergeCell ref="AR46:BI46"/>
+    <mergeCell ref="F56:L58"/>
   </mergeCells>
-  <conditionalFormatting sqref="M17:DA19 M22:DA33">
+  <conditionalFormatting sqref="M17:DA19 M22:DA33 M36:DA37">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>M$13=""</formula>
     </cfRule>
@@ -7299,17 +8016,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="54" t="inlineStr">
+      <c r="A1" s="55" t="inlineStr">
         <is>
           <t>Ingénieur Enedril</t>
         </is>
       </c>
-      <c r="C1" s="54" t="inlineStr">
+      <c r="C1" s="55" t="inlineStr">
         <is>
           <t>Codes du calendrier</t>
         </is>
       </c>
-      <c r="E1" s="54" t="inlineStr">
+      <c r="E1" s="55" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>

</xml_diff>